<commit_message>
refactor(Inspection Data): Turned varoius inspection related data from object properties to data properties. Issue #23
</commit_message>
<xml_diff>
--- a/M150-Onto_Metamodel_Rework.xlsx
+++ b/M150-Onto_Metamodel_Rework.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jluis\GitHub\ICOM\m150-onto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0162A0FE-2B63-46C4-975B-19CEF852F31E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43ED0766-5420-4B98-8CBB-195F4422D426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="930" windowWidth="33120" windowHeight="19860" firstSheet="1" activeTab="1" xr2:uid="{FEE85CB8-E22B-44F8-B2C8-C132767C24A8}"/>
+    <workbookView xWindow="90" yWindow="420" windowWidth="30135" windowHeight="19860" firstSheet="1" activeTab="1" xr2:uid="{FEE85CB8-E22B-44F8-B2C8-C132767C24A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Template Scoring Matrix" sheetId="8" r:id="rId1"/>
@@ -285,7 +285,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3948" uniqueCount="2160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3950" uniqueCount="2162">
   <si>
     <t>Kennung</t>
   </si>
@@ -6767,13 +6767,19 @@
   </si>
   <si>
     <t>New Class Classifier. New individual based on XML.</t>
+  </si>
+  <si>
+    <t>Reference Table Data has been removed from M150-Onto.</t>
+  </si>
+  <si>
+    <t>Format Data has been removed from M150-Onto.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6900,6 +6906,15 @@
     <font>
       <sz val="18"/>
       <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="18"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -7341,7 +7356,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="163">
+  <cellXfs count="164">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -7574,6 +7589,52 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="29" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="31" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="29" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="31" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="10" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="26" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="27" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="7" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="12" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="26" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="27" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="6" borderId="30" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -7598,23 +7659,17 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="31" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="30" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="31" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="30" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="9" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="31" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="10" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="26" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="27" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="31" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -7622,13 +7677,10 @@
     <xf numFmtId="49" fontId="6" fillId="5" borderId="7" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="12" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="29" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="3" borderId="21" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -7649,19 +7701,13 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="7" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -7671,6 +7717,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="29" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="29" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -7684,6 +7733,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="5" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="30" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="30" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="31" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="29" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -7727,9 +7785,6 @@
     <xf numFmtId="49" fontId="7" fillId="3" borderId="14" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="25" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -7739,47 +7794,8 @@
     <xf numFmtId="49" fontId="6" fillId="5" borderId="22" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="9" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="10" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="29" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="31" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="29" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="31" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="10" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="26" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="27" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -8518,13 +8534,13 @@
       <c r="C4" s="20" t="s">
         <v>1017</v>
       </c>
-      <c r="E4" s="129" t="s">
+      <c r="E4" s="146" t="s">
         <v>695</v>
       </c>
-      <c r="F4" s="130" t="s">
+      <c r="F4" s="147" t="s">
         <v>799</v>
       </c>
-      <c r="G4" s="130" t="s">
+      <c r="G4" s="147" t="s">
         <v>611</v>
       </c>
     </row>
@@ -8538,9 +8554,9 @@
       <c r="C5" s="20" t="s">
         <v>838</v>
       </c>
-      <c r="E5" s="129"/>
-      <c r="F5" s="130"/>
-      <c r="G5" s="130"/>
+      <c r="E5" s="146"/>
+      <c r="F5" s="147"/>
+      <c r="G5" s="147"/>
     </row>
     <row r="6" spans="1:20" ht="30" x14ac:dyDescent="0.4">
       <c r="A6" s="18" t="s">
@@ -8552,11 +8568,11 @@
       <c r="C6" s="20" t="s">
         <v>1018</v>
       </c>
-      <c r="E6" s="129"/>
-      <c r="F6" s="131" t="s">
+      <c r="E6" s="146"/>
+      <c r="F6" s="148" t="s">
         <v>800</v>
       </c>
-      <c r="G6" s="130" t="s">
+      <c r="G6" s="147" t="s">
         <v>611</v>
       </c>
     </row>
@@ -8570,9 +8586,9 @@
       <c r="C7" s="20" t="s">
         <v>839</v>
       </c>
-      <c r="E7" s="129"/>
-      <c r="F7" s="131"/>
-      <c r="G7" s="130"/>
+      <c r="E7" s="146"/>
+      <c r="F7" s="148"/>
+      <c r="G7" s="147"/>
       <c r="N7" t="s">
         <v>2123</v>
       </c>
@@ -8587,16 +8603,16 @@
       <c r="C9" s="20" t="s">
         <v>801</v>
       </c>
-      <c r="D9" s="143" t="s">
+      <c r="D9" s="163" t="s">
         <v>976</v>
       </c>
-      <c r="E9" s="100" t="s">
+      <c r="E9" s="143" t="s">
         <v>694</v>
       </c>
-      <c r="F9" s="123" t="s">
+      <c r="F9" s="136" t="s">
         <v>699</v>
       </c>
-      <c r="G9" s="120" t="s">
+      <c r="G9" s="134" t="s">
         <v>611</v>
       </c>
       <c r="H9" s="89" t="s">
@@ -8613,10 +8629,10 @@
       <c r="C10" s="20" t="s">
         <v>801</v>
       </c>
-      <c r="D10" s="143"/>
-      <c r="E10" s="96"/>
-      <c r="F10" s="123"/>
-      <c r="G10" s="120"/>
+      <c r="D10" s="163"/>
+      <c r="E10" s="116"/>
+      <c r="F10" s="136"/>
+      <c r="G10" s="134"/>
       <c r="N10" t="s">
         <v>2124</v>
       </c>
@@ -8634,11 +8650,11 @@
       <c r="C11" s="20" t="s">
         <v>802</v>
       </c>
-      <c r="E11" s="96"/>
-      <c r="F11" s="123" t="s">
+      <c r="E11" s="116"/>
+      <c r="F11" s="136" t="s">
         <v>698</v>
       </c>
-      <c r="G11" s="120" t="s">
+      <c r="G11" s="134" t="s">
         <v>611</v>
       </c>
       <c r="H11" s="89" t="s">
@@ -8658,9 +8674,9 @@
       <c r="C12" s="20" t="s">
         <v>802</v>
       </c>
-      <c r="E12" s="96"/>
-      <c r="F12" s="123"/>
-      <c r="G12" s="120"/>
+      <c r="E12" s="116"/>
+      <c r="F12" s="136"/>
+      <c r="G12" s="134"/>
       <c r="P12" t="s">
         <v>2119</v>
       </c>
@@ -8678,14 +8694,14 @@
       <c r="C13" s="20" t="s">
         <v>788</v>
       </c>
-      <c r="D13" s="143" t="s">
+      <c r="D13" s="163" t="s">
         <v>977</v>
       </c>
-      <c r="E13" s="96"/>
-      <c r="F13" s="123" t="s">
+      <c r="E13" s="116"/>
+      <c r="F13" s="136" t="s">
         <v>700</v>
       </c>
-      <c r="G13" s="120" t="s">
+      <c r="G13" s="134" t="s">
         <v>611</v>
       </c>
       <c r="H13" s="89" t="s">
@@ -8708,10 +8724,10 @@
       <c r="C14" s="20" t="s">
         <v>788</v>
       </c>
-      <c r="D14" s="143"/>
-      <c r="E14" s="96"/>
-      <c r="F14" s="123"/>
-      <c r="G14" s="120"/>
+      <c r="D14" s="163"/>
+      <c r="E14" s="116"/>
+      <c r="F14" s="136"/>
+      <c r="G14" s="134"/>
       <c r="P14" t="s">
         <v>2122</v>
       </c>
@@ -8729,11 +8745,11 @@
       <c r="C15" s="20" t="s">
         <v>803</v>
       </c>
-      <c r="E15" s="96"/>
-      <c r="F15" s="123" t="s">
+      <c r="E15" s="116"/>
+      <c r="F15" s="136" t="s">
         <v>701</v>
       </c>
-      <c r="G15" s="120" t="s">
+      <c r="G15" s="134" t="s">
         <v>611</v>
       </c>
       <c r="H15" s="89" t="s">
@@ -8753,9 +8769,9 @@
       <c r="C16" s="20" t="s">
         <v>803</v>
       </c>
-      <c r="E16" s="96"/>
-      <c r="F16" s="123"/>
-      <c r="G16" s="120"/>
+      <c r="E16" s="116"/>
+      <c r="F16" s="136"/>
+      <c r="G16" s="134"/>
       <c r="P16" t="s">
         <v>2109</v>
       </c>
@@ -8773,14 +8789,14 @@
       <c r="C17" s="20" t="s">
         <v>794</v>
       </c>
-      <c r="D17" s="143" t="s">
+      <c r="D17" s="163" t="s">
         <v>978</v>
       </c>
-      <c r="E17" s="96"/>
-      <c r="F17" s="122" t="s">
+      <c r="E17" s="116"/>
+      <c r="F17" s="135" t="s">
         <v>795</v>
       </c>
-      <c r="G17" s="120" t="s">
+      <c r="G17" s="134" t="s">
         <v>611</v>
       </c>
       <c r="H17" s="89" t="s">
@@ -8803,10 +8819,10 @@
       <c r="C18" s="20" t="s">
         <v>794</v>
       </c>
-      <c r="D18" s="143"/>
-      <c r="E18" s="96"/>
-      <c r="F18" s="122"/>
-      <c r="G18" s="120"/>
+      <c r="D18" s="163"/>
+      <c r="E18" s="116"/>
+      <c r="F18" s="135"/>
+      <c r="G18" s="134"/>
       <c r="P18" t="s">
         <v>2111</v>
       </c>
@@ -8824,14 +8840,14 @@
       <c r="C19" s="20" t="s">
         <v>796</v>
       </c>
-      <c r="D19" s="143" t="s">
+      <c r="D19" s="163" t="s">
         <v>979</v>
       </c>
-      <c r="E19" s="96"/>
-      <c r="F19" s="122" t="s">
+      <c r="E19" s="116"/>
+      <c r="F19" s="135" t="s">
         <v>797</v>
       </c>
-      <c r="G19" s="120" t="s">
+      <c r="G19" s="134" t="s">
         <v>611</v>
       </c>
       <c r="H19" s="89" t="s">
@@ -8854,10 +8870,10 @@
       <c r="C20" s="20" t="s">
         <v>796</v>
       </c>
-      <c r="D20" s="143"/>
-      <c r="E20" s="96"/>
-      <c r="F20" s="122"/>
-      <c r="G20" s="120"/>
+      <c r="D20" s="163"/>
+      <c r="E20" s="116"/>
+      <c r="F20" s="135"/>
+      <c r="G20" s="134"/>
       <c r="O20" t="s">
         <v>2125</v>
       </c>
@@ -8872,14 +8888,14 @@
       <c r="C21" s="20" t="s">
         <v>804</v>
       </c>
-      <c r="D21" s="143" t="s">
+      <c r="D21" s="163" t="s">
         <v>980</v>
       </c>
-      <c r="E21" s="96"/>
-      <c r="F21" s="123" t="s">
+      <c r="E21" s="116"/>
+      <c r="F21" s="136" t="s">
         <v>702</v>
       </c>
-      <c r="G21" s="120" t="s">
+      <c r="G21" s="134" t="s">
         <v>611</v>
       </c>
       <c r="H21" s="89" t="s">
@@ -8905,10 +8921,10 @@
       <c r="C22" s="20" t="s">
         <v>804</v>
       </c>
-      <c r="D22" s="143"/>
-      <c r="E22" s="96"/>
-      <c r="F22" s="123"/>
-      <c r="G22" s="120"/>
+      <c r="D22" s="163"/>
+      <c r="E22" s="116"/>
+      <c r="F22" s="136"/>
+      <c r="G22" s="134"/>
       <c r="P22" t="s">
         <v>2149</v>
       </c>
@@ -8929,14 +8945,14 @@
       <c r="C23" s="20" t="s">
         <v>805</v>
       </c>
-      <c r="D23" s="143" t="s">
+      <c r="D23" s="163" t="s">
         <v>981</v>
       </c>
-      <c r="E23" s="96"/>
-      <c r="F23" s="123" t="s">
+      <c r="E23" s="116"/>
+      <c r="F23" s="136" t="s">
         <v>703</v>
       </c>
-      <c r="G23" s="120" t="s">
+      <c r="G23" s="134" t="s">
         <v>611</v>
       </c>
       <c r="H23" s="89" t="s">
@@ -8956,10 +8972,10 @@
       <c r="C24" s="20" t="s">
         <v>805</v>
       </c>
-      <c r="D24" s="143"/>
-      <c r="E24" s="96"/>
-      <c r="F24" s="123"/>
-      <c r="G24" s="120"/>
+      <c r="D24" s="163"/>
+      <c r="E24" s="116"/>
+      <c r="F24" s="136"/>
+      <c r="G24" s="134"/>
       <c r="P24" t="s">
         <v>2134</v>
       </c>
@@ -8977,14 +8993,14 @@
       <c r="C25" s="20" t="s">
         <v>807</v>
       </c>
-      <c r="D25" s="143" t="s">
+      <c r="D25" s="163" t="s">
         <v>982</v>
       </c>
-      <c r="E25" s="96"/>
-      <c r="F25" s="123" t="s">
+      <c r="E25" s="116"/>
+      <c r="F25" s="136" t="s">
         <v>704</v>
       </c>
-      <c r="G25" s="120" t="s">
+      <c r="G25" s="134" t="s">
         <v>611</v>
       </c>
       <c r="P25" t="s">
@@ -9004,10 +9020,10 @@
       <c r="C26" s="20" t="s">
         <v>807</v>
       </c>
-      <c r="D26" s="143"/>
-      <c r="E26" s="96"/>
-      <c r="F26" s="123"/>
-      <c r="G26" s="120"/>
+      <c r="D26" s="163"/>
+      <c r="E26" s="116"/>
+      <c r="F26" s="136"/>
+      <c r="G26" s="134"/>
       <c r="O26" t="s">
         <v>2136</v>
       </c>
@@ -9022,14 +9038,14 @@
       <c r="C27" s="20" t="s">
         <v>808</v>
       </c>
-      <c r="D27" s="143" t="s">
+      <c r="D27" s="163" t="s">
         <v>983</v>
       </c>
-      <c r="E27" s="96"/>
-      <c r="F27" s="123" t="s">
+      <c r="E27" s="116"/>
+      <c r="F27" s="136" t="s">
         <v>2080</v>
       </c>
-      <c r="G27" s="120" t="s">
+      <c r="G27" s="134" t="s">
         <v>611</v>
       </c>
       <c r="P27" t="s">
@@ -9049,10 +9065,10 @@
       <c r="C28" s="20" t="s">
         <v>808</v>
       </c>
-      <c r="D28" s="143"/>
-      <c r="E28" s="96"/>
-      <c r="F28" s="123"/>
-      <c r="G28" s="120"/>
+      <c r="D28" s="163"/>
+      <c r="E28" s="117"/>
+      <c r="F28" s="136"/>
+      <c r="G28" s="134"/>
       <c r="P28" t="s">
         <v>643</v>
       </c>
@@ -9070,13 +9086,13 @@
       <c r="C29" s="20" t="s">
         <v>809</v>
       </c>
-      <c r="E29" s="101" t="s">
+      <c r="E29" s="144" t="s">
         <v>695</v>
       </c>
-      <c r="F29" s="125" t="s">
+      <c r="F29" s="139" t="s">
         <v>705</v>
       </c>
-      <c r="G29" s="136" t="s">
+      <c r="G29" s="153" t="s">
         <v>873</v>
       </c>
       <c r="P29" t="s">
@@ -9093,9 +9109,9 @@
       <c r="C30" s="20" t="s">
         <v>809</v>
       </c>
-      <c r="E30" s="102"/>
-      <c r="F30" s="126"/>
-      <c r="G30" s="137"/>
+      <c r="E30" s="145"/>
+      <c r="F30" s="140"/>
+      <c r="G30" s="154"/>
       <c r="P30" t="s">
         <v>653</v>
       </c>
@@ -9110,16 +9126,16 @@
       <c r="C31" s="20" t="s">
         <v>810</v>
       </c>
-      <c r="D31" s="143" t="s">
+      <c r="D31" s="163" t="s">
         <v>984</v>
       </c>
-      <c r="E31" s="100" t="s">
+      <c r="E31" s="143" t="s">
         <v>694</v>
       </c>
-      <c r="F31" s="127" t="s">
+      <c r="F31" s="141" t="s">
         <v>706</v>
       </c>
-      <c r="G31" s="134" t="s">
+      <c r="G31" s="151" t="s">
         <v>611</v>
       </c>
       <c r="P31" t="s">
@@ -9136,10 +9152,10 @@
       <c r="C32" s="20" t="s">
         <v>810</v>
       </c>
-      <c r="D32" s="143"/>
-      <c r="E32" s="99"/>
-      <c r="F32" s="128"/>
-      <c r="G32" s="135"/>
+      <c r="D32" s="163"/>
+      <c r="E32" s="117"/>
+      <c r="F32" s="142"/>
+      <c r="G32" s="152"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A34" s="18" t="s">
@@ -9154,13 +9170,13 @@
       <c r="D34" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E34" s="101" t="s">
+      <c r="E34" s="144" t="s">
         <v>695</v>
       </c>
-      <c r="F34" s="132" t="s">
+      <c r="F34" s="149" t="s">
         <v>709</v>
       </c>
-      <c r="G34" s="133" t="s">
+      <c r="G34" s="150" t="s">
         <v>614</v>
       </c>
     </row>
@@ -9174,9 +9190,9 @@
       <c r="C35" s="20" t="s">
         <v>806</v>
       </c>
-      <c r="E35" s="102"/>
-      <c r="F35" s="132"/>
-      <c r="G35" s="133"/>
+      <c r="E35" s="145"/>
+      <c r="F35" s="149"/>
+      <c r="G35" s="150"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A37" s="18" t="s">
@@ -9188,16 +9204,16 @@
       <c r="C37" s="20" t="s">
         <v>831</v>
       </c>
-      <c r="D37" s="143" t="s">
+      <c r="D37" s="163" t="s">
         <v>993</v>
       </c>
-      <c r="E37" s="124" t="s">
+      <c r="E37" s="137" t="s">
         <v>694</v>
       </c>
-      <c r="F37" s="123" t="s">
+      <c r="F37" s="136" t="s">
         <v>711</v>
       </c>
-      <c r="G37" s="120" t="s">
+      <c r="G37" s="134" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9211,10 +9227,10 @@
       <c r="C38" s="20" t="s">
         <v>831</v>
       </c>
-      <c r="D38" s="143"/>
-      <c r="E38" s="110"/>
-      <c r="F38" s="123"/>
-      <c r="G38" s="120"/>
+      <c r="D38" s="163"/>
+      <c r="E38" s="138"/>
+      <c r="F38" s="136"/>
+      <c r="G38" s="134"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A39" s="18" t="s">
@@ -9226,14 +9242,14 @@
       <c r="C39" s="20" t="s">
         <v>566</v>
       </c>
-      <c r="D39" s="143" t="s">
+      <c r="D39" s="163" t="s">
         <v>994</v>
       </c>
-      <c r="E39" s="110"/>
-      <c r="F39" s="123" t="s">
+      <c r="E39" s="138"/>
+      <c r="F39" s="136" t="s">
         <v>712</v>
       </c>
-      <c r="G39" s="120" t="s">
+      <c r="G39" s="134" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9247,10 +9263,10 @@
       <c r="C40" s="20" t="s">
         <v>566</v>
       </c>
-      <c r="D40" s="143"/>
-      <c r="E40" s="110"/>
-      <c r="F40" s="123"/>
-      <c r="G40" s="120"/>
+      <c r="D40" s="163"/>
+      <c r="E40" s="138"/>
+      <c r="F40" s="136"/>
+      <c r="G40" s="134"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A41" s="18" t="s">
@@ -9262,14 +9278,14 @@
       <c r="C41" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="D41" s="143" t="s">
+      <c r="D41" s="163" t="s">
         <v>995</v>
       </c>
-      <c r="E41" s="110"/>
-      <c r="F41" s="123" t="s">
+      <c r="E41" s="138"/>
+      <c r="F41" s="136" t="s">
         <v>717</v>
       </c>
-      <c r="G41" s="120" t="s">
+      <c r="G41" s="134" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9283,10 +9299,10 @@
       <c r="C42" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="D42" s="143"/>
-      <c r="E42" s="110"/>
-      <c r="F42" s="123"/>
-      <c r="G42" s="120"/>
+      <c r="D42" s="163"/>
+      <c r="E42" s="138"/>
+      <c r="F42" s="136"/>
+      <c r="G42" s="134"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A43" s="18" t="s">
@@ -9298,14 +9314,14 @@
       <c r="C43" s="20" t="s">
         <v>833</v>
       </c>
-      <c r="D43" s="143" t="s">
+      <c r="D43" s="163" t="s">
         <v>996</v>
       </c>
-      <c r="E43" s="110"/>
-      <c r="F43" s="123" t="s">
+      <c r="E43" s="138"/>
+      <c r="F43" s="136" t="s">
         <v>713</v>
       </c>
-      <c r="G43" s="120" t="s">
+      <c r="G43" s="134" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9319,10 +9335,10 @@
       <c r="C44" s="20" t="s">
         <v>833</v>
       </c>
-      <c r="D44" s="143"/>
-      <c r="E44" s="110"/>
-      <c r="F44" s="123"/>
-      <c r="G44" s="120"/>
+      <c r="D44" s="163"/>
+      <c r="E44" s="138"/>
+      <c r="F44" s="136"/>
+      <c r="G44" s="134"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A45" s="18" t="s">
@@ -9334,14 +9350,14 @@
       <c r="C45" s="20" t="s">
         <v>834</v>
       </c>
-      <c r="D45" s="143" t="s">
+      <c r="D45" s="163" t="s">
         <v>997</v>
       </c>
-      <c r="E45" s="110"/>
-      <c r="F45" s="123" t="s">
+      <c r="E45" s="138"/>
+      <c r="F45" s="136" t="s">
         <v>714</v>
       </c>
-      <c r="G45" s="120" t="s">
+      <c r="G45" s="134" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9355,10 +9371,10 @@
       <c r="C46" s="20" t="s">
         <v>834</v>
       </c>
-      <c r="D46" s="143"/>
-      <c r="E46" s="110"/>
-      <c r="F46" s="123"/>
-      <c r="G46" s="120"/>
+      <c r="D46" s="163"/>
+      <c r="E46" s="138"/>
+      <c r="F46" s="136"/>
+      <c r="G46" s="134"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A47" s="18" t="s">
@@ -9370,14 +9386,14 @@
       <c r="C47" s="20" t="s">
         <v>835</v>
       </c>
-      <c r="D47" s="143" t="s">
+      <c r="D47" s="163" t="s">
         <v>998</v>
       </c>
-      <c r="E47" s="110"/>
-      <c r="F47" s="123" t="s">
+      <c r="E47" s="138"/>
+      <c r="F47" s="136" t="s">
         <v>864</v>
       </c>
-      <c r="G47" s="120" t="s">
+      <c r="G47" s="134" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9391,10 +9407,10 @@
       <c r="C48" s="20" t="s">
         <v>835</v>
       </c>
-      <c r="D48" s="143"/>
-      <c r="E48" s="110"/>
-      <c r="F48" s="123"/>
-      <c r="G48" s="120"/>
+      <c r="D48" s="163"/>
+      <c r="E48" s="138"/>
+      <c r="F48" s="136"/>
+      <c r="G48" s="134"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A49" s="18" t="s">
@@ -9406,14 +9422,14 @@
       <c r="C49" s="20" t="s">
         <v>836</v>
       </c>
-      <c r="D49" s="143" t="s">
+      <c r="D49" s="163" t="s">
         <v>999</v>
       </c>
-      <c r="E49" s="110"/>
-      <c r="F49" s="123" t="s">
+      <c r="E49" s="138"/>
+      <c r="F49" s="136" t="s">
         <v>715</v>
       </c>
-      <c r="G49" s="120" t="s">
+      <c r="G49" s="134" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9427,10 +9443,10 @@
       <c r="C50" s="20" t="s">
         <v>836</v>
       </c>
-      <c r="D50" s="143"/>
-      <c r="E50" s="110"/>
-      <c r="F50" s="123"/>
-      <c r="G50" s="120"/>
+      <c r="D50" s="163"/>
+      <c r="E50" s="138"/>
+      <c r="F50" s="136"/>
+      <c r="G50" s="134"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A51" s="18" t="s">
@@ -9442,14 +9458,14 @@
       <c r="C51" s="20" t="s">
         <v>860</v>
       </c>
-      <c r="D51" s="143" t="s">
+      <c r="D51" s="163" t="s">
         <v>1000</v>
       </c>
-      <c r="E51" s="110"/>
-      <c r="F51" s="122" t="s">
+      <c r="E51" s="138"/>
+      <c r="F51" s="135" t="s">
         <v>798</v>
       </c>
-      <c r="G51" s="120" t="s">
+      <c r="G51" s="134" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9463,10 +9479,10 @@
       <c r="C52" s="20" t="s">
         <v>860</v>
       </c>
-      <c r="D52" s="143"/>
-      <c r="E52" s="110"/>
-      <c r="F52" s="122"/>
-      <c r="G52" s="120"/>
+      <c r="D52" s="163"/>
+      <c r="E52" s="138"/>
+      <c r="F52" s="135"/>
+      <c r="G52" s="134"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A53" s="18" t="s">
@@ -9478,14 +9494,14 @@
       <c r="C53" s="20" t="s">
         <v>837</v>
       </c>
-      <c r="D53" s="143" t="s">
+      <c r="D53" s="163" t="s">
         <v>1001</v>
       </c>
-      <c r="E53" s="110"/>
-      <c r="F53" s="123" t="s">
+      <c r="E53" s="138"/>
+      <c r="F53" s="136" t="s">
         <v>716</v>
       </c>
-      <c r="G53" s="120" t="s">
+      <c r="G53" s="134" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9499,16 +9515,16 @@
       <c r="C54" s="20" t="s">
         <v>837</v>
       </c>
-      <c r="D54" s="143"/>
-      <c r="E54" s="110"/>
-      <c r="F54" s="123"/>
-      <c r="G54" s="120"/>
+      <c r="D54" s="163"/>
+      <c r="E54" s="138"/>
+      <c r="F54" s="136"/>
+      <c r="G54" s="134"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="E56" s="117" t="s">
+      <c r="E56" s="104" t="s">
         <v>790</v>
       </c>
-      <c r="F56" s="117"/>
+      <c r="F56" s="104"/>
       <c r="G56" s="28" t="s">
         <v>613</v>
       </c>
@@ -9544,7 +9560,7 @@
       <c r="D58" s="32" t="s">
         <v>616</v>
       </c>
-      <c r="E58" s="103" t="s">
+      <c r="E58" s="108" t="s">
         <v>694</v>
       </c>
       <c r="F58" s="61" t="s">
@@ -9565,7 +9581,7 @@
       <c r="D59" s="32" t="s">
         <v>616</v>
       </c>
-      <c r="E59" s="104"/>
+      <c r="E59" s="109"/>
       <c r="F59" s="63" t="s">
         <v>2098</v>
       </c>
@@ -9584,7 +9600,7 @@
       <c r="D60" s="32" t="s">
         <v>616</v>
       </c>
-      <c r="E60" s="104"/>
+      <c r="E60" s="109"/>
       <c r="F60" s="65" t="s">
         <v>2099</v>
       </c>
@@ -9603,7 +9619,7 @@
       <c r="D61" s="32" t="s">
         <v>2052</v>
       </c>
-      <c r="E61" s="105"/>
+      <c r="E61" s="118"/>
       <c r="F61" s="27" t="s">
         <v>923</v>
       </c>
@@ -9736,7 +9752,7 @@
       <c r="C67" s="20" t="s">
         <v>567</v>
       </c>
-      <c r="E67" s="103" t="s">
+      <c r="E67" s="108" t="s">
         <v>694</v>
       </c>
       <c r="F67" s="34" t="s">
@@ -9757,7 +9773,7 @@
       <c r="D68" s="32" t="s">
         <v>2054</v>
       </c>
-      <c r="E68" s="104"/>
+      <c r="E68" s="109"/>
       <c r="F68" s="27" t="s">
         <v>929</v>
       </c>
@@ -9778,7 +9794,7 @@
       <c r="D69" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E69" s="92" t="s">
+      <c r="E69" s="110" t="s">
         <v>695</v>
       </c>
       <c r="F69" s="73" t="s">
@@ -9801,7 +9817,7 @@
       <c r="D70" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E70" s="93"/>
+      <c r="E70" s="111"/>
       <c r="F70" s="73" t="s">
         <v>931</v>
       </c>
@@ -9822,7 +9838,7 @@
       <c r="D71" s="32" t="s">
         <v>2055</v>
       </c>
-      <c r="E71" s="103" t="s">
+      <c r="E71" s="108" t="s">
         <v>694</v>
       </c>
       <c r="F71" s="27" t="s">
@@ -9845,7 +9861,7 @@
       <c r="D72" s="32" t="s">
         <v>984</v>
       </c>
-      <c r="E72" s="104"/>
+      <c r="E72" s="109"/>
       <c r="F72" s="27" t="s">
         <v>933</v>
       </c>
@@ -9866,7 +9882,7 @@
       <c r="D73" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E73" s="92" t="s">
+      <c r="E73" s="110" t="s">
         <v>695</v>
       </c>
       <c r="F73" s="73" t="s">
@@ -9889,7 +9905,7 @@
       <c r="D74" s="32" t="s">
         <v>605</v>
       </c>
-      <c r="E74" s="93"/>
+      <c r="E74" s="111"/>
       <c r="F74" s="73" t="s">
         <v>708</v>
       </c>
@@ -9976,7 +9992,7 @@
       <c r="C78" s="20" t="s">
         <v>859</v>
       </c>
-      <c r="E78" s="92" t="s">
+      <c r="E78" s="110" t="s">
         <v>695</v>
       </c>
       <c r="F78" s="73" t="s">
@@ -9999,7 +10015,7 @@
       <c r="D79" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E79" s="97"/>
+      <c r="E79" s="115"/>
       <c r="F79" s="73" t="s">
         <v>936</v>
       </c>
@@ -10040,11 +10056,11 @@
       <c r="C81" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E81" s="118" t="s">
+      <c r="E81" s="105" t="s">
         <v>620</v>
       </c>
-      <c r="F81" s="118"/>
-      <c r="G81" s="117" t="s">
+      <c r="F81" s="105"/>
+      <c r="G81" s="104" t="s">
         <v>611</v>
       </c>
     </row>
@@ -10058,9 +10074,9 @@
       <c r="C82" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E82" s="108"/>
-      <c r="F82" s="109"/>
-      <c r="G82" s="121"/>
+      <c r="E82" s="106"/>
+      <c r="F82" s="107"/>
+      <c r="G82" s="125"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E83" s="54"/>
@@ -10068,10 +10084,10 @@
       <c r="G83" s="23"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E84" s="117" t="s">
+      <c r="E84" s="104" t="s">
         <v>868</v>
       </c>
-      <c r="F84" s="117"/>
+      <c r="F84" s="104"/>
       <c r="G84" s="28" t="s">
         <v>613</v>
       </c>
@@ -10107,7 +10123,7 @@
       <c r="D86" s="32" t="s">
         <v>985</v>
       </c>
-      <c r="E86" s="95" t="s">
+      <c r="E86" s="113" t="s">
         <v>694</v>
       </c>
       <c r="F86" s="27" t="s">
@@ -10130,7 +10146,7 @@
       <c r="D87" s="32" t="s">
         <v>986</v>
       </c>
-      <c r="E87" s="98"/>
+      <c r="E87" s="116"/>
       <c r="F87" s="27" t="s">
         <v>939</v>
       </c>
@@ -10151,7 +10167,7 @@
       <c r="D88" s="32" t="s">
         <v>987</v>
       </c>
-      <c r="E88" s="98"/>
+      <c r="E88" s="116"/>
       <c r="F88" s="27" t="s">
         <v>940</v>
       </c>
@@ -10172,7 +10188,7 @@
       <c r="D89" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E89" s="92" t="s">
+      <c r="E89" s="110" t="s">
         <v>695</v>
       </c>
       <c r="F89" s="73" t="s">
@@ -10195,7 +10211,7 @@
       <c r="D90" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E90" s="93"/>
+      <c r="E90" s="111"/>
       <c r="F90" s="73" t="s">
         <v>942</v>
       </c>
@@ -10216,7 +10232,7 @@
       <c r="D91" s="32" t="s">
         <v>987</v>
       </c>
-      <c r="E91" s="95" t="s">
+      <c r="E91" s="113" t="s">
         <v>694</v>
       </c>
       <c r="F91" s="27" t="s">
@@ -10239,7 +10255,7 @@
       <c r="D92" s="32" t="s">
         <v>984</v>
       </c>
-      <c r="E92" s="98"/>
+      <c r="E92" s="116"/>
       <c r="F92" s="27" t="s">
         <v>944</v>
       </c>
@@ -10260,7 +10276,7 @@
       <c r="D93" s="32" t="s">
         <v>988</v>
       </c>
-      <c r="E93" s="98"/>
+      <c r="E93" s="116"/>
       <c r="F93" s="27" t="s">
         <v>2067</v>
       </c>
@@ -10281,7 +10297,7 @@
       <c r="D94" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E94" s="92" t="s">
+      <c r="E94" s="110" t="s">
         <v>695</v>
       </c>
       <c r="F94" s="73" t="s">
@@ -10304,7 +10320,7 @@
       <c r="D95" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E95" s="93"/>
+      <c r="E95" s="111"/>
       <c r="F95" s="73" t="s">
         <v>946</v>
       </c>
@@ -10322,7 +10338,7 @@
       <c r="C96" s="20" t="s">
         <v>819</v>
       </c>
-      <c r="E96" s="93"/>
+      <c r="E96" s="111"/>
       <c r="F96" s="73" t="s">
         <v>947</v>
       </c>
@@ -10385,7 +10401,7 @@
       <c r="D99" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E99" s="92" t="s">
+      <c r="E99" s="110" t="s">
         <v>695</v>
       </c>
       <c r="F99" s="73" t="s">
@@ -10408,7 +10424,7 @@
       <c r="D100" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E100" s="93"/>
+      <c r="E100" s="111"/>
       <c r="F100" s="73" t="s">
         <v>951</v>
       </c>
@@ -10572,11 +10588,11 @@
       <c r="C108" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E108" s="118" t="s">
+      <c r="E108" s="105" t="s">
         <v>620</v>
       </c>
-      <c r="F108" s="118"/>
-      <c r="G108" s="117" t="s">
+      <c r="F108" s="105"/>
+      <c r="G108" s="104" t="s">
         <v>611</v>
       </c>
     </row>
@@ -10590,15 +10606,15 @@
       <c r="C109" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E109" s="108"/>
-      <c r="F109" s="109"/>
-      <c r="G109" s="121"/>
+      <c r="E109" s="106"/>
+      <c r="F109" s="107"/>
+      <c r="G109" s="125"/>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E111" s="117" t="s">
+      <c r="E111" s="104" t="s">
         <v>868</v>
       </c>
-      <c r="F111" s="117"/>
+      <c r="F111" s="104"/>
       <c r="G111" s="28" t="s">
         <v>613</v>
       </c>
@@ -10675,7 +10691,7 @@
       <c r="C115" s="20" t="s">
         <v>914</v>
       </c>
-      <c r="E115" s="92" t="s">
+      <c r="E115" s="110" t="s">
         <v>695</v>
       </c>
       <c r="F115" s="78" t="s">
@@ -10698,7 +10714,7 @@
       <c r="D116" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E116" s="93"/>
+      <c r="E116" s="111"/>
       <c r="F116" s="78" t="s">
         <v>919</v>
       </c>
@@ -10719,7 +10735,7 @@
       <c r="D117" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E117" s="93"/>
+      <c r="E117" s="111"/>
       <c r="F117" s="78" t="s">
         <v>920</v>
       </c>
@@ -10740,7 +10756,7 @@
       <c r="D118" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E118" s="94"/>
+      <c r="E118" s="112"/>
       <c r="F118" s="78" t="s">
         <v>921</v>
       </c>
@@ -10779,11 +10795,11 @@
       <c r="C120" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E120" s="118" t="s">
+      <c r="E120" s="105" t="s">
         <v>620</v>
       </c>
-      <c r="F120" s="118"/>
-      <c r="G120" s="117" t="s">
+      <c r="F120" s="105"/>
+      <c r="G120" s="104" t="s">
         <v>611</v>
       </c>
     </row>
@@ -10797,9 +10813,9 @@
       <c r="C121" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E121" s="118"/>
-      <c r="F121" s="118"/>
-      <c r="G121" s="117"/>
+      <c r="E121" s="105"/>
+      <c r="F121" s="105"/>
+      <c r="G121" s="104"/>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.4">
       <c r="E122" s="55"/>
@@ -10825,7 +10841,7 @@
         <v>1031</v>
       </c>
       <c r="G124" s="60"/>
-      <c r="H124" s="90" t="s">
+      <c r="H124" s="103" t="s">
         <v>2100</v>
       </c>
     </row>
@@ -10840,7 +10856,7 @@
         <v>1021</v>
       </c>
       <c r="D125" s="45"/>
-      <c r="E125" s="144" t="s">
+      <c r="E125" s="160" t="s">
         <v>694</v>
       </c>
       <c r="F125" s="24" t="s">
@@ -10861,12 +10877,15 @@
         <v>1022</v>
       </c>
       <c r="D126" s="45"/>
-      <c r="E126" s="145"/>
+      <c r="E126" s="161"/>
       <c r="F126" s="51" t="s">
         <v>1028</v>
       </c>
       <c r="G126" s="25" t="s">
         <v>611</v>
+      </c>
+      <c r="H126" s="89" t="s">
+        <v>2160</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.4">
@@ -10880,7 +10899,7 @@
         <v>1023</v>
       </c>
       <c r="D127" s="45"/>
-      <c r="E127" s="145"/>
+      <c r="E127" s="161"/>
       <c r="F127" s="24" t="s">
         <v>1029</v>
       </c>
@@ -10899,7 +10918,7 @@
         <v>1024</v>
       </c>
       <c r="D128" s="45"/>
-      <c r="E128" s="146"/>
+      <c r="E128" s="162"/>
       <c r="F128" s="24" t="s">
         <v>1030</v>
       </c>
@@ -10918,10 +10937,10 @@
         <v>601</v>
       </c>
       <c r="D129" s="45"/>
-      <c r="E129" s="141" t="s">
+      <c r="E129" s="158" t="s">
         <v>620</v>
       </c>
-      <c r="F129" s="142"/>
+      <c r="F129" s="159"/>
       <c r="G129" s="26" t="s">
         <v>611</v>
       </c>
@@ -10962,7 +10981,7 @@
         <v>2069</v>
       </c>
       <c r="G132" s="60"/>
-      <c r="H132" s="90" t="s">
+      <c r="H132" s="103" t="s">
         <v>2100</v>
       </c>
     </row>
@@ -10977,7 +10996,7 @@
         <v>1025</v>
       </c>
       <c r="D133" s="45"/>
-      <c r="E133" s="95" t="s">
+      <c r="E133" s="113" t="s">
         <v>694</v>
       </c>
       <c r="F133" s="24" t="s">
@@ -10985,6 +11004,9 @@
       </c>
       <c r="G133" s="25" t="s">
         <v>611</v>
+      </c>
+      <c r="H133" s="89" t="s">
+        <v>2161</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.4">
@@ -10998,7 +11020,7 @@
         <v>1026</v>
       </c>
       <c r="D134" s="45"/>
-      <c r="E134" s="96"/>
+      <c r="E134" s="114"/>
       <c r="F134" s="24" t="s">
         <v>2068</v>
       </c>
@@ -11017,10 +11039,10 @@
       <c r="H136" s="91"/>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="E138" s="140" t="s">
+      <c r="E138" s="157" t="s">
         <v>907</v>
       </c>
-      <c r="F138" s="140"/>
+      <c r="F138" s="157"/>
       <c r="G138" s="28" t="s">
         <v>613</v>
       </c>
@@ -11078,7 +11100,7 @@
       <c r="D141" s="32" t="s">
         <v>2058</v>
       </c>
-      <c r="E141" s="95" t="s">
+      <c r="E141" s="113" t="s">
         <v>694</v>
       </c>
       <c r="F141" s="27" t="s">
@@ -11101,7 +11123,7 @@
       <c r="D142" s="32" t="s">
         <v>2059</v>
       </c>
-      <c r="E142" s="96"/>
+      <c r="E142" s="114"/>
       <c r="F142" s="27" t="s">
         <v>719</v>
       </c>
@@ -11119,11 +11141,11 @@
       <c r="C143" s="20" t="s">
         <v>589</v>
       </c>
-      <c r="E143" s="118" t="s">
+      <c r="E143" s="105" t="s">
         <v>620</v>
       </c>
-      <c r="F143" s="118"/>
-      <c r="G143" s="117" t="s">
+      <c r="F143" s="105"/>
+      <c r="G143" s="104" t="s">
         <v>611</v>
       </c>
     </row>
@@ -11137,9 +11159,9 @@
       <c r="C144" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E144" s="118"/>
-      <c r="F144" s="118"/>
-      <c r="G144" s="117"/>
+      <c r="E144" s="105"/>
+      <c r="F144" s="105"/>
+      <c r="G144" s="104"/>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A145" s="18" t="s">
@@ -11151,15 +11173,15 @@
       <c r="C145" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E145" s="118"/>
-      <c r="F145" s="118"/>
-      <c r="G145" s="117"/>
+      <c r="E145" s="105"/>
+      <c r="F145" s="105"/>
+      <c r="G145" s="104"/>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="E147" s="140" t="s">
+      <c r="E147" s="157" t="s">
         <v>908</v>
       </c>
-      <c r="F147" s="140"/>
+      <c r="F147" s="157"/>
       <c r="G147" s="28" t="s">
         <v>613</v>
       </c>
@@ -11235,7 +11257,7 @@
       <c r="C151" s="20" t="s">
         <v>590</v>
       </c>
-      <c r="E151" s="92" t="s">
+      <c r="E151" s="110" t="s">
         <v>695</v>
       </c>
       <c r="F151" s="78" t="s">
@@ -11255,7 +11277,7 @@
       <c r="C152" s="20" t="s">
         <v>591</v>
       </c>
-      <c r="E152" s="93"/>
+      <c r="E152" s="111"/>
       <c r="F152" s="78" t="s">
         <v>722</v>
       </c>
@@ -11273,7 +11295,7 @@
       <c r="C153" s="20" t="s">
         <v>596</v>
       </c>
-      <c r="E153" s="93"/>
+      <c r="E153" s="111"/>
       <c r="F153" s="78" t="s">
         <v>723</v>
       </c>
@@ -11291,7 +11313,7 @@
       <c r="C154" s="20" t="s">
         <v>597</v>
       </c>
-      <c r="E154" s="93"/>
+      <c r="E154" s="111"/>
       <c r="F154" s="78" t="s">
         <v>724</v>
       </c>
@@ -11309,7 +11331,7 @@
       <c r="C155" s="20" t="s">
         <v>592</v>
       </c>
-      <c r="E155" s="97"/>
+      <c r="E155" s="115"/>
       <c r="F155" s="78" t="s">
         <v>725</v>
       </c>
@@ -11330,7 +11352,7 @@
       <c r="D156" s="32" t="s">
         <v>2060</v>
       </c>
-      <c r="E156" s="95" t="s">
+      <c r="E156" s="113" t="s">
         <v>694</v>
       </c>
       <c r="F156" s="24" t="s">
@@ -11353,7 +11375,7 @@
       <c r="D157" s="32" t="s">
         <v>2061</v>
       </c>
-      <c r="E157" s="98"/>
+      <c r="E157" s="116"/>
       <c r="F157" s="24" t="s">
         <v>727</v>
       </c>
@@ -11374,7 +11396,7 @@
       <c r="D158" s="32" t="s">
         <v>2062</v>
       </c>
-      <c r="E158" s="98"/>
+      <c r="E158" s="116"/>
       <c r="F158" s="24" t="s">
         <v>728</v>
       </c>
@@ -11395,7 +11417,7 @@
       <c r="D159" s="32" t="s">
         <v>2063</v>
       </c>
-      <c r="E159" s="98"/>
+      <c r="E159" s="116"/>
       <c r="F159" s="24" t="s">
         <v>729</v>
       </c>
@@ -11416,7 +11438,7 @@
       <c r="D160" s="33" t="s">
         <v>2101</v>
       </c>
-      <c r="E160" s="99"/>
+      <c r="E160" s="117"/>
       <c r="F160" s="24" t="s">
         <v>730</v>
       </c>
@@ -11437,10 +11459,10 @@
       <c r="C161" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E161" s="118" t="s">
+      <c r="E161" s="105" t="s">
         <v>620</v>
       </c>
-      <c r="F161" s="118"/>
+      <c r="F161" s="105"/>
       <c r="G161" s="26" t="s">
         <v>611</v>
       </c>
@@ -11465,10 +11487,10 @@
       <c r="G164"/>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="E165" s="106" t="s">
+      <c r="E165" s="122" t="s">
         <v>2089</v>
       </c>
-      <c r="F165" s="106"/>
+      <c r="F165" s="122"/>
       <c r="G165" s="28" t="s">
         <v>613</v>
       </c>
@@ -11506,7 +11528,7 @@
       <c r="E167" s="77" t="s">
         <v>694</v>
       </c>
-      <c r="F167" s="107" t="s">
+      <c r="F167" s="123" t="s">
         <v>732</v>
       </c>
       <c r="G167" s="24" t="s">
@@ -11528,7 +11550,7 @@
       </c>
       <c r="D168" s="45"/>
       <c r="E168" s="77"/>
-      <c r="F168" s="107"/>
+      <c r="F168" s="123"/>
       <c r="G168" s="24" t="s">
         <v>611</v>
       </c>
@@ -11543,10 +11565,10 @@
       <c r="C169" s="18" t="s">
         <v>627</v>
       </c>
-      <c r="E169" s="92" t="s">
+      <c r="E169" s="110" t="s">
         <v>695</v>
       </c>
-      <c r="F169" s="147" t="s">
+      <c r="F169" s="124" t="s">
         <v>733</v>
       </c>
       <c r="G169" s="78" t="s">
@@ -11565,8 +11587,8 @@
         <v>627</v>
       </c>
       <c r="D170" s="45"/>
-      <c r="E170" s="94"/>
-      <c r="F170" s="147"/>
+      <c r="E170" s="112"/>
+      <c r="F170" s="124"/>
       <c r="G170" s="78" t="s">
         <v>611</v>
       </c>
@@ -11581,10 +11603,10 @@
       <c r="C171" s="18" t="s">
         <v>628</v>
       </c>
-      <c r="E171" s="92" t="s">
+      <c r="E171" s="110" t="s">
         <v>695</v>
       </c>
-      <c r="F171" s="132" t="s">
+      <c r="F171" s="149" t="s">
         <v>791</v>
       </c>
       <c r="G171" s="72" t="s">
@@ -11602,8 +11624,8 @@
         <v>628</v>
       </c>
       <c r="D172" s="45"/>
-      <c r="E172" s="94"/>
-      <c r="F172" s="132"/>
+      <c r="E172" s="112"/>
+      <c r="F172" s="149"/>
       <c r="G172" s="72" t="s">
         <v>873</v>
       </c>
@@ -11618,11 +11640,11 @@
       <c r="C173" s="18" t="s">
         <v>874</v>
       </c>
-      <c r="D173" s="143" t="s">
+      <c r="D173" s="163" t="s">
         <v>1003</v>
       </c>
       <c r="E173" s="77"/>
-      <c r="F173" s="107" t="s">
+      <c r="F173" s="123" t="s">
         <v>883</v>
       </c>
       <c r="G173" s="24" t="s">
@@ -11639,9 +11661,9 @@
       <c r="C174" t="s">
         <v>874</v>
       </c>
-      <c r="D174" s="143"/>
+      <c r="D174" s="163"/>
       <c r="E174" s="77"/>
-      <c r="F174" s="107"/>
+      <c r="F174" s="123"/>
       <c r="G174" s="24" t="s">
         <v>611</v>
       </c>
@@ -11656,11 +11678,11 @@
       <c r="C175" s="18" t="s">
         <v>629</v>
       </c>
-      <c r="D175" s="143" t="s">
+      <c r="D175" s="163" t="s">
         <v>1004</v>
       </c>
       <c r="E175" s="77"/>
-      <c r="F175" s="107" t="s">
+      <c r="F175" s="123" t="s">
         <v>734</v>
       </c>
       <c r="G175" s="24" t="s">
@@ -11677,9 +11699,9 @@
       <c r="C176" t="s">
         <v>629</v>
       </c>
-      <c r="D176" s="143"/>
+      <c r="D176" s="163"/>
       <c r="E176" s="77"/>
-      <c r="F176" s="107"/>
+      <c r="F176" s="123"/>
       <c r="G176" s="24" t="s">
         <v>611</v>
       </c>
@@ -11695,7 +11717,7 @@
         <v>630</v>
       </c>
       <c r="E177" s="77"/>
-      <c r="F177" s="107" t="s">
+      <c r="F177" s="123" t="s">
         <v>735</v>
       </c>
       <c r="G177" s="24" t="s">
@@ -11717,7 +11739,7 @@
       </c>
       <c r="D178" s="45"/>
       <c r="E178" s="77"/>
-      <c r="F178" s="107"/>
+      <c r="F178" s="123"/>
       <c r="G178" s="24" t="s">
         <v>611</v>
       </c>
@@ -11732,11 +11754,11 @@
       <c r="C179" s="18" t="s">
         <v>631</v>
       </c>
-      <c r="D179" s="143" t="s">
+      <c r="D179" s="163" t="s">
         <v>1005</v>
       </c>
       <c r="E179" s="77"/>
-      <c r="F179" s="107" t="s">
+      <c r="F179" s="123" t="s">
         <v>736</v>
       </c>
       <c r="G179" s="24" t="s">
@@ -11753,9 +11775,9 @@
       <c r="C180" t="s">
         <v>631</v>
       </c>
-      <c r="D180" s="143"/>
+      <c r="D180" s="163"/>
       <c r="E180" s="77"/>
-      <c r="F180" s="107"/>
+      <c r="F180" s="123"/>
       <c r="G180" s="24" t="s">
         <v>611</v>
       </c>
@@ -11770,10 +11792,10 @@
       <c r="C181" s="18" t="s">
         <v>632</v>
       </c>
-      <c r="E181" s="92" t="s">
+      <c r="E181" s="110" t="s">
         <v>695</v>
       </c>
-      <c r="F181" s="147" t="s">
+      <c r="F181" s="124" t="s">
         <v>737</v>
       </c>
       <c r="G181" s="78" t="s">
@@ -11791,8 +11813,8 @@
         <v>632</v>
       </c>
       <c r="D182" s="45"/>
-      <c r="E182" s="94"/>
-      <c r="F182" s="147"/>
+      <c r="E182" s="112"/>
+      <c r="F182" s="124"/>
       <c r="G182" s="78" t="s">
         <v>611</v>
       </c>
@@ -11807,13 +11829,13 @@
       <c r="C184" s="18" t="s">
         <v>635</v>
       </c>
-      <c r="D184" s="143" t="s">
+      <c r="D184" s="163" t="s">
         <v>1008</v>
       </c>
       <c r="E184" s="79" t="s">
         <v>694</v>
       </c>
-      <c r="F184" s="107" t="s">
+      <c r="F184" s="123" t="s">
         <v>890</v>
       </c>
       <c r="G184" s="24" t="s">
@@ -11830,9 +11852,9 @@
       <c r="C185" t="s">
         <v>635</v>
       </c>
-      <c r="D185" s="143"/>
+      <c r="D185" s="163"/>
       <c r="E185" s="77"/>
-      <c r="F185" s="107"/>
+      <c r="F185" s="123"/>
       <c r="G185" s="24" t="s">
         <v>611</v>
       </c>
@@ -11847,13 +11869,13 @@
       <c r="C186" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="E186" s="92" t="s">
+      <c r="E186" s="110" t="s">
         <v>695</v>
       </c>
-      <c r="F186" s="148" t="s">
+      <c r="F186" s="119" t="s">
         <v>2094</v>
       </c>
-      <c r="G186" s="149" t="s">
+      <c r="G186" s="92" t="s">
         <v>2095</v>
       </c>
     </row>
@@ -11868,9 +11890,9 @@
         <v>636</v>
       </c>
       <c r="D187" s="45"/>
-      <c r="E187" s="93"/>
-      <c r="F187" s="150"/>
-      <c r="G187" s="149" t="s">
+      <c r="E187" s="111"/>
+      <c r="F187" s="120"/>
+      <c r="G187" s="92" t="s">
         <v>2095</v>
       </c>
     </row>
@@ -11884,9 +11906,9 @@
       <c r="C188" s="18" t="s">
         <v>637</v>
       </c>
-      <c r="E188" s="93"/>
-      <c r="F188" s="150"/>
-      <c r="G188" s="149" t="s">
+      <c r="E188" s="111"/>
+      <c r="F188" s="120"/>
+      <c r="G188" s="92" t="s">
         <v>2095</v>
       </c>
     </row>
@@ -11901,9 +11923,9 @@
         <v>637</v>
       </c>
       <c r="D189" s="45"/>
-      <c r="E189" s="94"/>
-      <c r="F189" s="151"/>
-      <c r="G189" s="149" t="s">
+      <c r="E189" s="112"/>
+      <c r="F189" s="121"/>
+      <c r="G189" s="92" t="s">
         <v>2095</v>
       </c>
     </row>
@@ -11917,11 +11939,11 @@
       <c r="C190" s="18" t="s">
         <v>638</v>
       </c>
-      <c r="D190" s="143" t="s">
+      <c r="D190" s="163" t="s">
         <v>1009</v>
       </c>
       <c r="E190" s="77"/>
-      <c r="F190" s="107" t="s">
+      <c r="F190" s="123" t="s">
         <v>738</v>
       </c>
       <c r="G190" s="24" t="s">
@@ -11938,9 +11960,9 @@
       <c r="C191" t="s">
         <v>638</v>
       </c>
-      <c r="D191" s="143"/>
+      <c r="D191" s="163"/>
       <c r="E191" s="77"/>
-      <c r="F191" s="107"/>
+      <c r="F191" s="123"/>
       <c r="G191" s="24" t="s">
         <v>611</v>
       </c>
@@ -11955,11 +11977,11 @@
       <c r="C192" s="18" t="s">
         <v>639</v>
       </c>
-      <c r="D192" s="143" t="s">
+      <c r="D192" s="163" t="s">
         <v>1010</v>
       </c>
       <c r="E192" s="77"/>
-      <c r="F192" s="107" t="s">
+      <c r="F192" s="123" t="s">
         <v>739</v>
       </c>
       <c r="G192" s="24" t="s">
@@ -11976,9 +11998,9 @@
       <c r="C193" t="s">
         <v>639</v>
       </c>
-      <c r="D193" s="143"/>
+      <c r="D193" s="163"/>
       <c r="E193" s="77"/>
-      <c r="F193" s="107"/>
+      <c r="F193" s="123"/>
       <c r="G193" s="24" t="s">
         <v>611</v>
       </c>
@@ -11993,13 +12015,13 @@
       <c r="C194" s="18" t="s">
         <v>640</v>
       </c>
-      <c r="D194" s="143" t="s">
+      <c r="D194" s="163" t="s">
         <v>606</v>
       </c>
-      <c r="E194" s="92" t="s">
+      <c r="E194" s="110" t="s">
         <v>695</v>
       </c>
-      <c r="F194" s="147" t="s">
+      <c r="F194" s="124" t="s">
         <v>740</v>
       </c>
       <c r="G194" s="78" t="s">
@@ -12016,9 +12038,9 @@
       <c r="C195" t="s">
         <v>640</v>
       </c>
-      <c r="D195" s="143"/>
-      <c r="E195" s="94"/>
-      <c r="F195" s="147"/>
+      <c r="D195" s="163"/>
+      <c r="E195" s="112"/>
+      <c r="F195" s="124"/>
       <c r="G195" s="78" t="s">
         <v>873</v>
       </c>
@@ -12033,11 +12055,11 @@
       <c r="C196" s="18" t="s">
         <v>877</v>
       </c>
-      <c r="D196" s="143" t="s">
+      <c r="D196" s="163" t="s">
         <v>1011</v>
       </c>
       <c r="E196" s="77"/>
-      <c r="F196" s="107" t="s">
+      <c r="F196" s="123" t="s">
         <v>741</v>
       </c>
       <c r="G196" s="24" t="s">
@@ -12054,9 +12076,9 @@
       <c r="C197" t="s">
         <v>877</v>
       </c>
-      <c r="D197" s="143"/>
+      <c r="D197" s="163"/>
       <c r="E197" s="77"/>
-      <c r="F197" s="107"/>
+      <c r="F197" s="123"/>
       <c r="G197" s="24" t="s">
         <v>611</v>
       </c>
@@ -12071,10 +12093,10 @@
       <c r="C198" s="18" t="s">
         <v>641</v>
       </c>
-      <c r="E198" s="92" t="s">
+      <c r="E198" s="110" t="s">
         <v>695</v>
       </c>
-      <c r="F198" s="147" t="s">
+      <c r="F198" s="124" t="s">
         <v>742</v>
       </c>
       <c r="G198" s="78" t="s">
@@ -12092,8 +12114,8 @@
         <v>641</v>
       </c>
       <c r="D199" s="45"/>
-      <c r="E199" s="94"/>
-      <c r="F199" s="147"/>
+      <c r="E199" s="112"/>
+      <c r="F199" s="124"/>
       <c r="G199" s="78" t="s">
         <v>873</v>
       </c>
@@ -12109,7 +12131,7 @@
         <v>642</v>
       </c>
       <c r="E200" s="77"/>
-      <c r="F200" s="107" t="s">
+      <c r="F200" s="123" t="s">
         <v>743</v>
       </c>
       <c r="G200" s="24" t="s">
@@ -12131,7 +12153,7 @@
       </c>
       <c r="D201" s="45"/>
       <c r="E201" s="77"/>
-      <c r="F201" s="107"/>
+      <c r="F201" s="123"/>
       <c r="G201" s="24" t="s">
         <v>611</v>
       </c>
@@ -12147,7 +12169,7 @@
         <v>643</v>
       </c>
       <c r="E202" s="77"/>
-      <c r="F202" s="107" t="s">
+      <c r="F202" s="123" t="s">
         <v>744</v>
       </c>
       <c r="G202" s="24" t="s">
@@ -12169,7 +12191,7 @@
       </c>
       <c r="D203" s="45"/>
       <c r="E203" s="77"/>
-      <c r="F203" s="107"/>
+      <c r="F203" s="123"/>
       <c r="G203" s="24" t="s">
         <v>611</v>
       </c>
@@ -12185,7 +12207,7 @@
         <v>644</v>
       </c>
       <c r="E204" s="77"/>
-      <c r="F204" s="107" t="s">
+      <c r="F204" s="123" t="s">
         <v>745</v>
       </c>
       <c r="G204" s="24" t="s">
@@ -12204,7 +12226,7 @@
       </c>
       <c r="D205" s="45"/>
       <c r="E205" s="77"/>
-      <c r="F205" s="107"/>
+      <c r="F205" s="123"/>
       <c r="G205" s="24" t="s">
         <v>611</v>
       </c>
@@ -12219,11 +12241,11 @@
       <c r="C206" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="D206" s="143" t="s">
+      <c r="D206" s="163" t="s">
         <v>1012</v>
       </c>
       <c r="E206" s="77"/>
-      <c r="F206" s="107" t="s">
+      <c r="F206" s="123" t="s">
         <v>746</v>
       </c>
       <c r="G206" s="24" t="s">
@@ -12240,9 +12262,9 @@
       <c r="C207" t="s">
         <v>645</v>
       </c>
-      <c r="D207" s="143"/>
+      <c r="D207" s="163"/>
       <c r="E207" s="77"/>
-      <c r="F207" s="107"/>
+      <c r="F207" s="123"/>
       <c r="G207" s="24" t="s">
         <v>611</v>
       </c>
@@ -12258,7 +12280,7 @@
         <v>646</v>
       </c>
       <c r="E208" s="77"/>
-      <c r="F208" s="107" t="s">
+      <c r="F208" s="123" t="s">
         <v>891</v>
       </c>
       <c r="G208" s="24" t="s">
@@ -12280,7 +12302,7 @@
       </c>
       <c r="D209" s="45"/>
       <c r="E209" s="77"/>
-      <c r="F209" s="107"/>
+      <c r="F209" s="123"/>
       <c r="G209" s="24" t="s">
         <v>611</v>
       </c>
@@ -12299,7 +12321,7 @@
         <v>647</v>
       </c>
       <c r="E210" s="77"/>
-      <c r="F210" s="107" t="s">
+      <c r="F210" s="123" t="s">
         <v>892</v>
       </c>
       <c r="G210" s="24" t="s">
@@ -12321,7 +12343,7 @@
       </c>
       <c r="D211" s="45"/>
       <c r="E211" s="77"/>
-      <c r="F211" s="107"/>
+      <c r="F211" s="123"/>
       <c r="G211" s="24" t="s">
         <v>611</v>
       </c>
@@ -12336,11 +12358,11 @@
       <c r="C212" s="18" t="s">
         <v>648</v>
       </c>
-      <c r="D212" s="143" t="s">
+      <c r="D212" s="163" t="s">
         <v>1013</v>
       </c>
       <c r="E212" s="77"/>
-      <c r="F212" s="107" t="s">
+      <c r="F212" s="123" t="s">
         <v>747</v>
       </c>
       <c r="G212" s="24" t="s">
@@ -12357,9 +12379,9 @@
       <c r="C213" t="s">
         <v>648</v>
       </c>
-      <c r="D213" s="143"/>
+      <c r="D213" s="163"/>
       <c r="E213" s="77"/>
-      <c r="F213" s="107"/>
+      <c r="F213" s="123"/>
       <c r="G213" s="24" t="s">
         <v>611</v>
       </c>
@@ -12383,13 +12405,13 @@
       <c r="C215" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="D215" s="143" t="s">
+      <c r="D215" s="163" t="s">
         <v>1015</v>
       </c>
       <c r="E215" s="77" t="s">
         <v>695</v>
       </c>
-      <c r="F215" s="119" t="s">
+      <c r="F215" s="132" t="s">
         <v>748</v>
       </c>
       <c r="G215" s="24" t="s">
@@ -12406,9 +12428,9 @@
       <c r="C216" t="s">
         <v>649</v>
       </c>
-      <c r="D216" s="143"/>
+      <c r="D216" s="163"/>
       <c r="E216" s="77"/>
-      <c r="F216" s="119"/>
+      <c r="F216" s="132"/>
       <c r="G216" s="24" t="s">
         <v>611</v>
       </c>
@@ -12423,9 +12445,9 @@
       <c r="C217" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="D217" s="143"/>
+      <c r="D217" s="163"/>
       <c r="E217" s="77"/>
-      <c r="F217" s="119"/>
+      <c r="F217" s="132"/>
       <c r="G217" s="24" t="s">
         <v>611</v>
       </c>
@@ -12440,9 +12462,9 @@
       <c r="C218" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="D218" s="143"/>
+      <c r="D218" s="163"/>
       <c r="E218" s="77"/>
-      <c r="F218" s="119"/>
+      <c r="F218" s="132"/>
       <c r="G218" s="24" t="s">
         <v>611</v>
       </c>
@@ -12457,13 +12479,13 @@
       <c r="C219" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="E219" s="92" t="s">
+      <c r="E219" s="110" t="s">
         <v>695</v>
       </c>
-      <c r="F219" s="152" t="s">
+      <c r="F219" s="133" t="s">
         <v>749</v>
       </c>
-      <c r="G219" s="149" t="s">
+      <c r="G219" s="92" t="s">
         <v>2095</v>
       </c>
     </row>
@@ -12478,9 +12500,9 @@
         <v>650</v>
       </c>
       <c r="D220" s="45"/>
-      <c r="E220" s="93"/>
-      <c r="F220" s="152"/>
-      <c r="G220" s="149" t="s">
+      <c r="E220" s="111"/>
+      <c r="F220" s="133"/>
+      <c r="G220" s="92" t="s">
         <v>2095</v>
       </c>
     </row>
@@ -12494,9 +12516,9 @@
       <c r="C221" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="E221" s="93"/>
-      <c r="F221" s="152"/>
-      <c r="G221" s="149" t="s">
+      <c r="E221" s="111"/>
+      <c r="F221" s="133"/>
+      <c r="G221" s="92" t="s">
         <v>2095</v>
       </c>
     </row>
@@ -12510,9 +12532,9 @@
       <c r="C222" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="E222" s="94"/>
-      <c r="F222" s="152"/>
-      <c r="G222" s="149" t="s">
+      <c r="E222" s="112"/>
+      <c r="F222" s="133"/>
+      <c r="G222" s="92" t="s">
         <v>2095</v>
       </c>
     </row>
@@ -12527,7 +12549,7 @@
         <v>651</v>
       </c>
       <c r="E223" s="77"/>
-      <c r="F223" s="119" t="s">
+      <c r="F223" s="132" t="s">
         <v>750</v>
       </c>
       <c r="G223" s="24" t="s">
@@ -12549,7 +12571,7 @@
       </c>
       <c r="D224" s="45"/>
       <c r="E224" s="77"/>
-      <c r="F224" s="119"/>
+      <c r="F224" s="132"/>
       <c r="G224" s="24" t="s">
         <v>611</v>
       </c>
@@ -12568,7 +12590,7 @@
         <v>651</v>
       </c>
       <c r="E225" s="77"/>
-      <c r="F225" s="119"/>
+      <c r="F225" s="132"/>
       <c r="G225" s="24" t="s">
         <v>611</v>
       </c>
@@ -12584,7 +12606,7 @@
         <v>651</v>
       </c>
       <c r="E226" s="77"/>
-      <c r="F226" s="119"/>
+      <c r="F226" s="132"/>
       <c r="G226" s="24" t="s">
         <v>611</v>
       </c>
@@ -12599,10 +12621,10 @@
       <c r="C227" s="18" t="s">
         <v>652</v>
       </c>
-      <c r="E227" s="92" t="s">
+      <c r="E227" s="110" t="s">
         <v>695</v>
       </c>
-      <c r="F227" s="147" t="s">
+      <c r="F227" s="124" t="s">
         <v>751</v>
       </c>
       <c r="G227" s="78" t="s">
@@ -12620,8 +12642,8 @@
         <v>652</v>
       </c>
       <c r="D228" s="45"/>
-      <c r="E228" s="94"/>
-      <c r="F228" s="147"/>
+      <c r="E228" s="112"/>
+      <c r="F228" s="124"/>
       <c r="G228" s="78" t="s">
         <v>2095</v>
       </c>
@@ -12637,7 +12659,7 @@
         <v>653</v>
       </c>
       <c r="E229" s="77"/>
-      <c r="F229" s="107" t="s">
+      <c r="F229" s="123" t="s">
         <v>752</v>
       </c>
       <c r="G229" s="24" t="s">
@@ -12659,7 +12681,7 @@
       </c>
       <c r="D230" s="45"/>
       <c r="E230" s="77"/>
-      <c r="F230" s="107"/>
+      <c r="F230" s="123"/>
       <c r="G230" s="24" t="s">
         <v>611</v>
       </c>
@@ -12677,10 +12699,10 @@
       <c r="D231" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E231" s="92" t="s">
+      <c r="E231" s="110" t="s">
         <v>695</v>
       </c>
-      <c r="F231" s="147" t="s">
+      <c r="F231" s="124" t="s">
         <v>753</v>
       </c>
       <c r="G231" s="78" t="s">
@@ -12701,8 +12723,8 @@
         <v>654</v>
       </c>
       <c r="D232" s="45"/>
-      <c r="E232" s="94"/>
-      <c r="F232" s="147"/>
+      <c r="E232" s="112"/>
+      <c r="F232" s="124"/>
       <c r="G232" s="78" t="s">
         <v>873</v>
       </c>
@@ -12720,8 +12742,8 @@
       <c r="D233" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E233" s="153"/>
-      <c r="F233" s="147" t="s">
+      <c r="E233" s="93"/>
+      <c r="F233" s="124" t="s">
         <v>754</v>
       </c>
       <c r="G233" s="78" t="s">
@@ -12739,8 +12761,8 @@
         <v>655</v>
       </c>
       <c r="D234" s="45"/>
-      <c r="E234" s="153"/>
-      <c r="F234" s="147"/>
+      <c r="E234" s="93"/>
+      <c r="F234" s="124"/>
       <c r="G234" s="78" t="s">
         <v>873</v>
       </c>
@@ -12758,8 +12780,8 @@
       <c r="D235" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E235" s="153"/>
-      <c r="F235" s="147" t="s">
+      <c r="E235" s="93"/>
+      <c r="F235" s="124" t="s">
         <v>755</v>
       </c>
       <c r="G235" s="78" t="s">
@@ -12777,8 +12799,8 @@
         <v>656</v>
       </c>
       <c r="D236" s="45"/>
-      <c r="E236" s="153"/>
-      <c r="F236" s="147"/>
+      <c r="E236" s="93"/>
+      <c r="F236" s="124"/>
       <c r="G236" s="78" t="s">
         <v>873</v>
       </c>
@@ -12796,8 +12818,8 @@
       <c r="D237" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E237" s="153"/>
-      <c r="F237" s="147" t="s">
+      <c r="E237" s="93"/>
+      <c r="F237" s="124" t="s">
         <v>756</v>
       </c>
       <c r="G237" s="78" t="s">
@@ -12815,8 +12837,8 @@
         <v>657</v>
       </c>
       <c r="D238" s="45"/>
-      <c r="E238" s="153"/>
-      <c r="F238" s="147"/>
+      <c r="E238" s="93"/>
+      <c r="F238" s="124"/>
       <c r="G238" s="78" t="s">
         <v>873</v>
       </c>
@@ -12834,8 +12856,8 @@
       <c r="D239" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E239" s="153"/>
-      <c r="F239" s="147" t="s">
+      <c r="E239" s="93"/>
+      <c r="F239" s="124" t="s">
         <v>757</v>
       </c>
       <c r="G239" s="78" t="s">
@@ -12853,8 +12875,8 @@
         <v>658</v>
       </c>
       <c r="D240" s="45"/>
-      <c r="E240" s="153"/>
-      <c r="F240" s="147"/>
+      <c r="E240" s="93"/>
+      <c r="F240" s="124"/>
       <c r="G240" s="78" t="s">
         <v>873</v>
       </c>
@@ -12872,8 +12894,8 @@
       <c r="D241" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E241" s="153"/>
-      <c r="F241" s="147" t="s">
+      <c r="E241" s="93"/>
+      <c r="F241" s="124" t="s">
         <v>758</v>
       </c>
       <c r="G241" s="78" t="s">
@@ -12891,8 +12913,8 @@
         <v>659</v>
       </c>
       <c r="D242" s="45"/>
-      <c r="E242" s="153"/>
-      <c r="F242" s="147"/>
+      <c r="E242" s="93"/>
+      <c r="F242" s="124"/>
       <c r="G242" s="78" t="s">
         <v>873</v>
       </c>
@@ -12910,8 +12932,8 @@
       <c r="D243" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E243" s="153"/>
-      <c r="F243" s="147" t="s">
+      <c r="E243" s="93"/>
+      <c r="F243" s="124" t="s">
         <v>759</v>
       </c>
       <c r="G243" s="78" t="s">
@@ -12929,8 +12951,8 @@
         <v>660</v>
       </c>
       <c r="D244" s="45"/>
-      <c r="E244" s="153"/>
-      <c r="F244" s="147"/>
+      <c r="E244" s="93"/>
+      <c r="F244" s="124"/>
       <c r="G244" s="78" t="s">
         <v>873</v>
       </c>
@@ -12948,8 +12970,8 @@
       <c r="D245" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E245" s="153"/>
-      <c r="F245" s="147" t="s">
+      <c r="E245" s="93"/>
+      <c r="F245" s="124" t="s">
         <v>760</v>
       </c>
       <c r="G245" s="78" t="s">
@@ -12967,8 +12989,8 @@
         <v>661</v>
       </c>
       <c r="D246" s="45"/>
-      <c r="E246" s="153"/>
-      <c r="F246" s="147"/>
+      <c r="E246" s="93"/>
+      <c r="F246" s="124"/>
       <c r="G246" s="78" t="s">
         <v>873</v>
       </c>
@@ -12986,8 +13008,8 @@
       <c r="D247" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E247" s="153"/>
-      <c r="F247" s="147" t="s">
+      <c r="E247" s="93"/>
+      <c r="F247" s="124" t="s">
         <v>761</v>
       </c>
       <c r="G247" s="78" t="s">
@@ -13005,8 +13027,8 @@
         <v>662</v>
       </c>
       <c r="D248" s="45"/>
-      <c r="E248" s="153"/>
-      <c r="F248" s="147"/>
+      <c r="E248" s="93"/>
+      <c r="F248" s="124"/>
       <c r="G248" s="78" t="s">
         <v>873</v>
       </c>
@@ -13024,8 +13046,8 @@
       <c r="D249" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E249" s="153"/>
-      <c r="F249" s="147" t="s">
+      <c r="E249" s="93"/>
+      <c r="F249" s="124" t="s">
         <v>2072</v>
       </c>
       <c r="G249" s="78" t="s">
@@ -13043,8 +13065,8 @@
         <v>663</v>
       </c>
       <c r="D250" s="45"/>
-      <c r="E250" s="153"/>
-      <c r="F250" s="147"/>
+      <c r="E250" s="93"/>
+      <c r="F250" s="124"/>
       <c r="G250" s="78" t="s">
         <v>873</v>
       </c>
@@ -13062,8 +13084,8 @@
       <c r="D251" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E251" s="153"/>
-      <c r="F251" s="147" t="s">
+      <c r="E251" s="93"/>
+      <c r="F251" s="124" t="s">
         <v>762</v>
       </c>
       <c r="G251" s="78" t="s">
@@ -13081,8 +13103,8 @@
         <v>664</v>
       </c>
       <c r="D252" s="45"/>
-      <c r="E252" s="153"/>
-      <c r="F252" s="147"/>
+      <c r="E252" s="93"/>
+      <c r="F252" s="124"/>
       <c r="G252" s="78" t="s">
         <v>873</v>
       </c>
@@ -13097,8 +13119,8 @@
       <c r="C253" s="18" t="s">
         <v>665</v>
       </c>
-      <c r="E253" s="153"/>
-      <c r="F253" s="147" t="s">
+      <c r="E253" s="93"/>
+      <c r="F253" s="124" t="s">
         <v>763</v>
       </c>
       <c r="G253" s="78" t="s">
@@ -13116,8 +13138,8 @@
         <v>665</v>
       </c>
       <c r="D254" s="45"/>
-      <c r="E254" s="153"/>
-      <c r="F254" s="147"/>
+      <c r="E254" s="93"/>
+      <c r="F254" s="124"/>
       <c r="G254" s="78" t="s">
         <v>873</v>
       </c>
@@ -13196,11 +13218,11 @@
       <c r="C260" s="18" t="s">
         <v>573</v>
       </c>
-      <c r="E260" s="108" t="s">
+      <c r="E260" s="106" t="s">
         <v>620</v>
       </c>
-      <c r="F260" s="109"/>
-      <c r="G260" s="138" t="s">
+      <c r="F260" s="107"/>
+      <c r="G260" s="155" t="s">
         <v>611</v>
       </c>
     </row>
@@ -13214,9 +13236,9 @@
       <c r="C261" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E261" s="108"/>
-      <c r="F261" s="109"/>
-      <c r="G261" s="139"/>
+      <c r="E261" s="106"/>
+      <c r="F261" s="107"/>
+      <c r="G261" s="156"/>
     </row>
     <row r="262" spans="1:8" x14ac:dyDescent="0.4">
       <c r="C262" s="23"/>
@@ -13254,13 +13276,13 @@
       <c r="D264" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E264" s="156" t="s">
+      <c r="E264" s="96" t="s">
         <v>695</v>
       </c>
       <c r="F264" s="87" t="s">
         <v>787</v>
       </c>
-      <c r="G264" s="157" t="s">
+      <c r="G264" s="97" t="s">
         <v>614</v>
       </c>
     </row>
@@ -13295,7 +13317,7 @@
       <c r="C266" s="18" t="s">
         <v>667</v>
       </c>
-      <c r="E266" s="155" t="s">
+      <c r="E266" s="95" t="s">
         <v>695</v>
       </c>
       <c r="F266" s="78" t="s">
@@ -13336,10 +13358,10 @@
       <c r="C268" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E268" s="118" t="s">
+      <c r="E268" s="105" t="s">
         <v>620</v>
       </c>
-      <c r="F268" s="118"/>
+      <c r="F268" s="105"/>
       <c r="G268" s="26" t="s">
         <v>611</v>
       </c>
@@ -13439,17 +13461,17 @@
       <c r="C275" t="s">
         <v>879</v>
       </c>
-      <c r="D275" s="158" t="s">
+      <c r="D275" s="98" t="s">
         <v>2152</v>
       </c>
-      <c r="E275" s="153"/>
-      <c r="F275" s="160" t="s">
+      <c r="E275" s="93"/>
+      <c r="F275" s="100" t="s">
         <v>964</v>
       </c>
       <c r="G275" s="78" t="s">
         <v>618</v>
       </c>
-      <c r="H275" s="159"/>
+      <c r="H275" s="99"/>
     </row>
     <row r="276" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A276" t="s">
@@ -13464,8 +13486,8 @@
       <c r="D276" s="45" t="s">
         <v>2153</v>
       </c>
-      <c r="E276" s="153"/>
-      <c r="F276" s="160" t="s">
+      <c r="E276" s="93"/>
+      <c r="F276" s="100" t="s">
         <v>965</v>
       </c>
       <c r="G276" s="78" t="s">
@@ -13526,11 +13548,11 @@
         <v>573</v>
       </c>
       <c r="D279" s="45"/>
-      <c r="E279" s="118" t="s">
+      <c r="E279" s="105" t="s">
         <v>620</v>
       </c>
-      <c r="F279" s="118"/>
-      <c r="G279" s="117" t="s">
+      <c r="F279" s="105"/>
+      <c r="G279" s="104" t="s">
         <v>611</v>
       </c>
     </row>
@@ -13545,19 +13567,19 @@
         <v>601</v>
       </c>
       <c r="D280" s="45"/>
-      <c r="E280" s="118"/>
-      <c r="F280" s="118"/>
-      <c r="G280" s="117"/>
+      <c r="E280" s="105"/>
+      <c r="F280" s="105"/>
+      <c r="G280" s="104"/>
     </row>
     <row r="282" spans="1:8" x14ac:dyDescent="0.4">
       <c r="C282" s="23"/>
     </row>
     <row r="283" spans="1:8" x14ac:dyDescent="0.4">
       <c r="C283" s="23"/>
-      <c r="E283" s="106" t="s">
+      <c r="E283" s="122" t="s">
         <v>906</v>
       </c>
-      <c r="F283" s="106"/>
+      <c r="F283" s="122"/>
       <c r="G283" s="28" t="s">
         <v>613</v>
       </c>
@@ -13595,10 +13617,10 @@
       <c r="D285" s="32" t="s">
         <v>621</v>
       </c>
-      <c r="E285" s="153" t="s">
+      <c r="E285" s="93" t="s">
         <v>695</v>
       </c>
-      <c r="F285" s="147" t="s">
+      <c r="F285" s="124" t="s">
         <v>792</v>
       </c>
       <c r="G285" s="78" t="s">
@@ -13618,8 +13640,8 @@
       <c r="C286" s="18" t="s">
         <v>669</v>
       </c>
-      <c r="E286" s="153"/>
-      <c r="F286" s="147"/>
+      <c r="E286" s="93"/>
+      <c r="F286" s="124"/>
       <c r="G286" s="78" t="s">
         <v>611</v>
       </c>
@@ -13637,8 +13659,8 @@
       <c r="D287" s="32" t="s">
         <v>621</v>
       </c>
-      <c r="E287" s="153"/>
-      <c r="F287" s="147" t="s">
+      <c r="E287" s="93"/>
+      <c r="F287" s="124" t="s">
         <v>769</v>
       </c>
       <c r="G287" s="78" t="s">
@@ -13655,8 +13677,8 @@
       <c r="C288" s="18" t="s">
         <v>670</v>
       </c>
-      <c r="E288" s="153"/>
-      <c r="F288" s="147"/>
+      <c r="E288" s="93"/>
+      <c r="F288" s="124"/>
       <c r="G288" s="78" t="s">
         <v>611</v>
       </c>
@@ -13674,8 +13696,8 @@
       <c r="D289" s="32" t="s">
         <v>621</v>
       </c>
-      <c r="E289" s="153"/>
-      <c r="F289" s="147" t="s">
+      <c r="E289" s="93"/>
+      <c r="F289" s="124" t="s">
         <v>770</v>
       </c>
       <c r="G289" s="78" t="s">
@@ -13692,8 +13714,8 @@
       <c r="C290" s="18" t="s">
         <v>671</v>
       </c>
-      <c r="E290" s="153"/>
-      <c r="F290" s="147"/>
+      <c r="E290" s="93"/>
+      <c r="F290" s="124"/>
       <c r="G290" s="78" t="s">
         <v>611</v>
       </c>
@@ -13711,8 +13733,8 @@
       <c r="D291" s="32" t="s">
         <v>622</v>
       </c>
-      <c r="E291" s="153"/>
-      <c r="F291" s="147" t="s">
+      <c r="E291" s="93"/>
+      <c r="F291" s="124" t="s">
         <v>771</v>
       </c>
       <c r="G291" s="78" t="s">
@@ -13729,8 +13751,8 @@
       <c r="C292" s="18" t="s">
         <v>672</v>
       </c>
-      <c r="E292" s="153"/>
-      <c r="F292" s="147"/>
+      <c r="E292" s="93"/>
+      <c r="F292" s="124"/>
       <c r="G292" s="78" t="s">
         <v>614</v>
       </c>
@@ -13748,8 +13770,8 @@
       <c r="D293" s="32" t="s">
         <v>622</v>
       </c>
-      <c r="E293" s="153"/>
-      <c r="F293" s="147" t="s">
+      <c r="E293" s="93"/>
+      <c r="F293" s="124" t="s">
         <v>772</v>
       </c>
       <c r="G293" s="78" t="s">
@@ -13766,8 +13788,8 @@
       <c r="C294" s="18" t="s">
         <v>673</v>
       </c>
-      <c r="E294" s="153"/>
-      <c r="F294" s="147"/>
+      <c r="E294" s="93"/>
+      <c r="F294" s="124"/>
       <c r="G294" s="78" t="s">
         <v>614</v>
       </c>
@@ -13785,8 +13807,8 @@
       <c r="D295" s="32" t="s">
         <v>621</v>
       </c>
-      <c r="E295" s="153"/>
-      <c r="F295" s="147" t="s">
+      <c r="E295" s="93"/>
+      <c r="F295" s="124" t="s">
         <v>773</v>
       </c>
       <c r="G295" s="78" t="s">
@@ -13803,8 +13825,8 @@
       <c r="C296" s="18" t="s">
         <v>674</v>
       </c>
-      <c r="E296" s="153"/>
-      <c r="F296" s="147"/>
+      <c r="E296" s="93"/>
+      <c r="F296" s="124"/>
       <c r="G296" s="78" t="s">
         <v>611</v>
       </c>
@@ -13822,8 +13844,8 @@
       <c r="D297" s="32" t="s">
         <v>621</v>
       </c>
-      <c r="E297" s="153"/>
-      <c r="F297" s="147" t="s">
+      <c r="E297" s="93"/>
+      <c r="F297" s="124" t="s">
         <v>774</v>
       </c>
       <c r="G297" s="78" t="s">
@@ -13840,8 +13862,8 @@
       <c r="C298" s="18" t="s">
         <v>675</v>
       </c>
-      <c r="E298" s="153"/>
-      <c r="F298" s="147"/>
+      <c r="E298" s="93"/>
+      <c r="F298" s="124"/>
       <c r="G298" s="78" t="s">
         <v>611</v>
       </c>
@@ -13859,8 +13881,8 @@
       <c r="D299" s="32" t="s">
         <v>621</v>
       </c>
-      <c r="E299" s="153"/>
-      <c r="F299" s="147" t="s">
+      <c r="E299" s="93"/>
+      <c r="F299" s="124" t="s">
         <v>775</v>
       </c>
       <c r="G299" s="78" t="s">
@@ -13877,8 +13899,8 @@
       <c r="C300" s="18" t="s">
         <v>676</v>
       </c>
-      <c r="E300" s="153"/>
-      <c r="F300" s="147"/>
+      <c r="E300" s="93"/>
+      <c r="F300" s="124"/>
       <c r="G300" s="78" t="s">
         <v>611</v>
       </c>
@@ -13896,8 +13918,8 @@
       <c r="D301" s="32" t="s">
         <v>623</v>
       </c>
-      <c r="E301" s="153"/>
-      <c r="F301" s="147" t="s">
+      <c r="E301" s="93"/>
+      <c r="F301" s="124" t="s">
         <v>776</v>
       </c>
       <c r="G301" s="78" t="s">
@@ -13914,8 +13936,8 @@
       <c r="C302" s="18" t="s">
         <v>677</v>
       </c>
-      <c r="E302" s="153"/>
-      <c r="F302" s="147"/>
+      <c r="E302" s="93"/>
+      <c r="F302" s="124"/>
       <c r="G302" s="78" t="s">
         <v>611</v>
       </c>
@@ -13931,7 +13953,7 @@
         <v>678</v>
       </c>
       <c r="E303" s="77"/>
-      <c r="F303" s="107" t="s">
+      <c r="F303" s="123" t="s">
         <v>777</v>
       </c>
       <c r="G303" s="24" t="s">
@@ -13952,7 +13974,7 @@
         <v>678</v>
       </c>
       <c r="E304" s="77"/>
-      <c r="F304" s="107"/>
+      <c r="F304" s="123"/>
       <c r="G304" s="24" t="s">
         <v>611</v>
       </c>
@@ -13967,8 +13989,8 @@
       <c r="C305" s="18" t="s">
         <v>679</v>
       </c>
-      <c r="E305" s="153"/>
-      <c r="F305" s="147" t="s">
+      <c r="E305" s="93"/>
+      <c r="F305" s="124" t="s">
         <v>778</v>
       </c>
       <c r="G305" s="78" t="s">
@@ -13985,8 +14007,8 @@
       <c r="C306" s="18" t="s">
         <v>679</v>
       </c>
-      <c r="E306" s="153"/>
-      <c r="F306" s="147"/>
+      <c r="E306" s="93"/>
+      <c r="F306" s="124"/>
       <c r="G306" s="78" t="s">
         <v>611</v>
       </c>
@@ -14001,11 +14023,11 @@
       <c r="C307" s="18" t="s">
         <v>680</v>
       </c>
-      <c r="E307" s="153"/>
-      <c r="F307" s="147" t="s">
+      <c r="E307" s="93"/>
+      <c r="F307" s="124" t="s">
         <v>779</v>
       </c>
-      <c r="G307" s="149" t="s">
+      <c r="G307" s="92" t="s">
         <v>618</v>
       </c>
       <c r="H307" s="89" t="s">
@@ -14022,9 +14044,9 @@
       <c r="C308" s="18" t="s">
         <v>680</v>
       </c>
-      <c r="E308" s="153"/>
-      <c r="F308" s="147"/>
-      <c r="G308" s="149" t="s">
+      <c r="E308" s="93"/>
+      <c r="F308" s="124"/>
+      <c r="G308" s="92" t="s">
         <v>618</v>
       </c>
     </row>
@@ -14038,8 +14060,8 @@
       <c r="C309" s="18" t="s">
         <v>682</v>
       </c>
-      <c r="E309" s="153"/>
-      <c r="F309" s="147" t="s">
+      <c r="E309" s="93"/>
+      <c r="F309" s="124" t="s">
         <v>780</v>
       </c>
       <c r="G309" s="78" t="s">
@@ -14056,8 +14078,8 @@
       <c r="C310" s="18" t="s">
         <v>682</v>
       </c>
-      <c r="E310" s="153"/>
-      <c r="F310" s="147"/>
+      <c r="E310" s="93"/>
+      <c r="F310" s="124"/>
       <c r="G310" s="78" t="s">
         <v>611</v>
       </c>
@@ -14072,8 +14094,8 @@
       <c r="C311" s="18" t="s">
         <v>683</v>
       </c>
-      <c r="E311" s="153"/>
-      <c r="F311" s="147" t="s">
+      <c r="E311" s="93"/>
+      <c r="F311" s="124" t="s">
         <v>781</v>
       </c>
       <c r="G311" s="78" t="s">
@@ -14090,8 +14112,8 @@
       <c r="C312" s="18" t="s">
         <v>683</v>
       </c>
-      <c r="E312" s="153"/>
-      <c r="F312" s="147"/>
+      <c r="E312" s="93"/>
+      <c r="F312" s="124"/>
       <c r="G312" s="78" t="s">
         <v>2095</v>
       </c>
@@ -14107,7 +14129,7 @@
         <v>684</v>
       </c>
       <c r="E313" s="77"/>
-      <c r="F313" s="107" t="s">
+      <c r="F313" s="123" t="s">
         <v>782</v>
       </c>
       <c r="G313" s="24" t="s">
@@ -14128,7 +14150,7 @@
         <v>684</v>
       </c>
       <c r="E314" s="77"/>
-      <c r="F314" s="107"/>
+      <c r="F314" s="123"/>
       <c r="G314" s="24" t="s">
         <v>611</v>
       </c>
@@ -14143,8 +14165,8 @@
       <c r="C315" s="18" t="s">
         <v>685</v>
       </c>
-      <c r="E315" s="153"/>
-      <c r="F315" s="147" t="s">
+      <c r="E315" s="93"/>
+      <c r="F315" s="124" t="s">
         <v>783</v>
       </c>
       <c r="G315" s="78" t="s">
@@ -14161,8 +14183,8 @@
       <c r="C316" s="18" t="s">
         <v>685</v>
       </c>
-      <c r="E316" s="153"/>
-      <c r="F316" s="147"/>
+      <c r="E316" s="93"/>
+      <c r="F316" s="124"/>
       <c r="G316" s="78" t="s">
         <v>873</v>
       </c>
@@ -14177,8 +14199,8 @@
       <c r="C317" s="18" t="s">
         <v>686</v>
       </c>
-      <c r="E317" s="153"/>
-      <c r="F317" s="147" t="s">
+      <c r="E317" s="93"/>
+      <c r="F317" s="124" t="s">
         <v>784</v>
       </c>
       <c r="G317" s="78" t="s">
@@ -14195,8 +14217,8 @@
       <c r="C318" s="18" t="s">
         <v>686</v>
       </c>
-      <c r="E318" s="153"/>
-      <c r="F318" s="147"/>
+      <c r="E318" s="93"/>
+      <c r="F318" s="124"/>
       <c r="G318" s="78" t="s">
         <v>873</v>
       </c>
@@ -14211,8 +14233,8 @@
       <c r="C319" s="18" t="s">
         <v>687</v>
       </c>
-      <c r="E319" s="153"/>
-      <c r="F319" s="147" t="s">
+      <c r="E319" s="93"/>
+      <c r="F319" s="124" t="s">
         <v>785</v>
       </c>
       <c r="G319" s="78" t="s">
@@ -14229,8 +14251,8 @@
       <c r="C320" s="18" t="s">
         <v>687</v>
       </c>
-      <c r="E320" s="153"/>
-      <c r="F320" s="147"/>
+      <c r="E320" s="93"/>
+      <c r="F320" s="124"/>
       <c r="G320" s="78" t="s">
         <v>873</v>
       </c>
@@ -14245,8 +14267,8 @@
       <c r="C321" s="18" t="s">
         <v>688</v>
       </c>
-      <c r="E321" s="153"/>
-      <c r="F321" s="147" t="s">
+      <c r="E321" s="93"/>
+      <c r="F321" s="124" t="s">
         <v>786</v>
       </c>
       <c r="G321" s="78" t="s">
@@ -14263,8 +14285,8 @@
       <c r="C322" s="18" t="s">
         <v>688</v>
       </c>
-      <c r="E322" s="153"/>
-      <c r="F322" s="147"/>
+      <c r="E322" s="93"/>
+      <c r="F322" s="124"/>
       <c r="G322" s="78" t="s">
         <v>611</v>
       </c>
@@ -14302,13 +14324,13 @@
       <c r="D326" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E326" s="161" t="s">
+      <c r="E326" s="101" t="s">
         <v>695</v>
       </c>
       <c r="F326" s="87" t="s">
         <v>968</v>
       </c>
-      <c r="G326" s="157" t="s">
+      <c r="G326" s="97" t="s">
         <v>614</v>
       </c>
     </row>
@@ -14325,8 +14347,8 @@
       <c r="D327" s="32" t="s">
         <v>624</v>
       </c>
-      <c r="E327" s="162"/>
-      <c r="F327" s="149" t="s">
+      <c r="E327" s="102"/>
+      <c r="F327" s="92" t="s">
         <v>969</v>
       </c>
       <c r="G327" s="78" t="s">
@@ -14346,7 +14368,7 @@
       <c r="D328" s="32" t="s">
         <v>2065</v>
       </c>
-      <c r="E328" s="154"/>
+      <c r="E328" s="94"/>
       <c r="F328" s="30" t="s">
         <v>970</v>
       </c>
@@ -14364,11 +14386,11 @@
       <c r="C329" s="18" t="s">
         <v>573</v>
       </c>
-      <c r="E329" s="111" t="s">
+      <c r="E329" s="126" t="s">
         <v>620</v>
       </c>
-      <c r="F329" s="112"/>
-      <c r="G329" s="115" t="s">
+      <c r="F329" s="127"/>
+      <c r="G329" s="130" t="s">
         <v>611</v>
       </c>
     </row>
@@ -14382,9 +14404,9 @@
       <c r="C330" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E330" s="113"/>
-      <c r="F330" s="114"/>
-      <c r="G330" s="116"/>
+      <c r="E330" s="128"/>
+      <c r="F330" s="129"/>
+      <c r="G330" s="131"/>
     </row>
     <row r="333" spans="1:7" ht="24.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A333" s="38" t="s">
@@ -14419,13 +14441,13 @@
       <c r="D334" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E334" s="161" t="s">
+      <c r="E334" s="101" t="s">
         <v>695</v>
       </c>
       <c r="F334" s="87" t="s">
         <v>971</v>
       </c>
-      <c r="G334" s="157" t="s">
+      <c r="G334" s="97" t="s">
         <v>614</v>
       </c>
     </row>
@@ -14442,8 +14464,8 @@
       <c r="D335" s="32" t="s">
         <v>2158</v>
       </c>
-      <c r="E335" s="162"/>
-      <c r="F335" s="149" t="s">
+      <c r="E335" s="102"/>
+      <c r="F335" s="92" t="s">
         <v>972</v>
       </c>
       <c r="G335" s="78" t="s">
@@ -14463,7 +14485,7 @@
       <c r="D336" s="32" t="s">
         <v>1016</v>
       </c>
-      <c r="E336" s="154"/>
+      <c r="E336" s="94"/>
       <c r="F336" s="30" t="s">
         <v>973</v>
       </c>
@@ -14481,11 +14503,11 @@
       <c r="C337" s="18" t="s">
         <v>573</v>
       </c>
-      <c r="E337" s="111" t="s">
+      <c r="E337" s="126" t="s">
         <v>620</v>
       </c>
-      <c r="F337" s="112"/>
-      <c r="G337" s="115" t="s">
+      <c r="F337" s="127"/>
+      <c r="G337" s="130" t="s">
         <v>611</v>
       </c>
     </row>
@@ -14499,9 +14521,9 @@
       <c r="C338" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E338" s="113"/>
-      <c r="F338" s="114"/>
-      <c r="G338" s="116"/>
+      <c r="E338" s="128"/>
+      <c r="F338" s="129"/>
+      <c r="G338" s="131"/>
     </row>
   </sheetData>
   <mergeCells count="193">
@@ -14557,6 +14579,7 @@
     <mergeCell ref="E125:E128"/>
     <mergeCell ref="E133:E134"/>
     <mergeCell ref="E198:E199"/>
+    <mergeCell ref="G120:G121"/>
     <mergeCell ref="E4:E7"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="F6:F7"/>
@@ -14600,7 +14623,8 @@
     <mergeCell ref="F31:F32"/>
     <mergeCell ref="F37:F38"/>
     <mergeCell ref="E9:E28"/>
-    <mergeCell ref="G120:G121"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="E29:E30"/>
     <mergeCell ref="G37:G38"/>
     <mergeCell ref="G39:G40"/>
     <mergeCell ref="G41:G42"/>
@@ -14634,18 +14658,6 @@
     <mergeCell ref="F321:F322"/>
     <mergeCell ref="F285:F286"/>
     <mergeCell ref="F287:F288"/>
-    <mergeCell ref="F289:F290"/>
-    <mergeCell ref="F291:F292"/>
-    <mergeCell ref="F293:F294"/>
-    <mergeCell ref="F295:F296"/>
-    <mergeCell ref="F297:F298"/>
-    <mergeCell ref="F299:F300"/>
-    <mergeCell ref="F301:F302"/>
-    <mergeCell ref="F303:F304"/>
-    <mergeCell ref="F305:F306"/>
-    <mergeCell ref="F307:F308"/>
-    <mergeCell ref="F309:F310"/>
-    <mergeCell ref="F311:F312"/>
     <mergeCell ref="F317:F318"/>
     <mergeCell ref="F319:F320"/>
     <mergeCell ref="F237:F238"/>
@@ -14659,11 +14671,24 @@
     <mergeCell ref="E219:E222"/>
     <mergeCell ref="E227:E228"/>
     <mergeCell ref="E231:E232"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="F289:F290"/>
+    <mergeCell ref="F291:F292"/>
+    <mergeCell ref="F293:F294"/>
+    <mergeCell ref="F295:F296"/>
+    <mergeCell ref="F297:F298"/>
+    <mergeCell ref="F299:F300"/>
+    <mergeCell ref="F301:F302"/>
+    <mergeCell ref="F303:F304"/>
+    <mergeCell ref="F305:F306"/>
+    <mergeCell ref="F184:F185"/>
+    <mergeCell ref="F190:F191"/>
+    <mergeCell ref="F192:F193"/>
+    <mergeCell ref="E194:E195"/>
+    <mergeCell ref="E111:F111"/>
+    <mergeCell ref="E120:F121"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="E181:E182"/>
+    <mergeCell ref="F307:F308"/>
     <mergeCell ref="F186:F189"/>
     <mergeCell ref="E283:F283"/>
     <mergeCell ref="F313:F314"/>
@@ -14673,12 +14698,8 @@
     <mergeCell ref="F198:F199"/>
     <mergeCell ref="F200:F201"/>
     <mergeCell ref="F202:F203"/>
-    <mergeCell ref="F184:F185"/>
-    <mergeCell ref="F190:F191"/>
-    <mergeCell ref="F192:F193"/>
-    <mergeCell ref="E194:E195"/>
-    <mergeCell ref="E111:F111"/>
-    <mergeCell ref="E120:F121"/>
+    <mergeCell ref="F309:F310"/>
+    <mergeCell ref="F311:F312"/>
     <mergeCell ref="E56:F56"/>
     <mergeCell ref="E84:F84"/>
     <mergeCell ref="E108:F109"/>
@@ -14688,7 +14709,6 @@
     <mergeCell ref="E151:E155"/>
     <mergeCell ref="E156:E160"/>
     <mergeCell ref="E171:E172"/>
-    <mergeCell ref="E186:E189"/>
     <mergeCell ref="E73:E74"/>
     <mergeCell ref="E86:E88"/>
     <mergeCell ref="E89:E90"/>
@@ -14697,7 +14717,9 @@
     <mergeCell ref="E94:E96"/>
     <mergeCell ref="E78:E79"/>
     <mergeCell ref="E169:E170"/>
-    <mergeCell ref="E181:E182"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E69:E70"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="A1:A123 A135:A1048576">

</xml_diff>

<commit_message>
refactor(m150-onto): - HG/KG updated according to metamodel rework. - Add classes `SpatialEntity` and `InformationEntity` for issues #26 and #20. Subclasses added to consider project-specific data. - Add class `Directionality` for issues #26 and #19. Subclass `FlowingDirection` added.
update(Metamodel): Added more context for `HG008`.
</commit_message>
<xml_diff>
--- a/M150-Onto_Metamodel_Rework.xlsx
+++ b/M150-Onto_Metamodel_Rework.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jluis\GitHub\ICOM\m150-onto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jluis\Repositories\M150-Onto\m150-onto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43ED0766-5420-4B98-8CBB-195F4422D426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D88318-3102-464C-9752-30013A1ADE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="90" yWindow="420" windowWidth="30135" windowHeight="19860" firstSheet="1" activeTab="1" xr2:uid="{FEE85CB8-E22B-44F8-B2C8-C132767C24A8}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{FEE85CB8-E22B-44F8-B2C8-C132767C24A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Template Scoring Matrix" sheetId="8" r:id="rId1"/>
@@ -6601,9 +6601,6 @@
     <t>Create 2 new individuals here named Clockwise, counterclockwise. New class Orientation</t>
   </si>
   <si>
-    <t>Create 2 new individuals here. New class StationingDirection. Type of new class.</t>
-  </si>
-  <si>
     <t>Create new class: Person.</t>
   </si>
   <si>
@@ -6773,6 +6770,9 @@
   </si>
   <si>
     <t>Format Data has been removed from M150-Onto.</t>
+  </si>
+  <si>
+    <t>Create 2 new individuals here. New class FlowingDirection (a subclass of Directionality). Individuals:InFlowingDirection and AgainstFlowingDirection. Both type of FlowingDirection.</t>
   </si>
 </sst>
 </file>
@@ -7617,58 +7617,25 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="3" borderId="7" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="12" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="26" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="27" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="30" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="27" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="31" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="26" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="27" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="32" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="27" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="31" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="31" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="9" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="6" borderId="10" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="3" applyBorder="1" applyAlignment="1">
@@ -7680,7 +7647,106 @@
     <xf numFmtId="49" fontId="6" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="12" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="7" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="19" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="14" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="25" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="12" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="22" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="26" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="27" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="30" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="31" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="29" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="30" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="31" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="7" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="7" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="29" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="29" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="30" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="27" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="31" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="3" borderId="21" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -7707,95 +7773,29 @@
     <xf numFmtId="49" fontId="0" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="27" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="8" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="9" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="10" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="26" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="7" xfId="5" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="27" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="29" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="32" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="29" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="31" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="30" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="30" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="31" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="29" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="7" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="7" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="19" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="14" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="25" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="12" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="22" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -7809,7 +7809,27 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="6" xr:uid="{73184220-ECEF-4E4B-9D39-939CEB9C7E6F}"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -8534,13 +8554,13 @@
       <c r="C4" s="20" t="s">
         <v>1017</v>
       </c>
-      <c r="E4" s="146" t="s">
+      <c r="E4" s="126" t="s">
         <v>695</v>
       </c>
-      <c r="F4" s="147" t="s">
+      <c r="F4" s="127" t="s">
         <v>799</v>
       </c>
-      <c r="G4" s="147" t="s">
+      <c r="G4" s="127" t="s">
         <v>611</v>
       </c>
     </row>
@@ -8554,9 +8574,9 @@
       <c r="C5" s="20" t="s">
         <v>838</v>
       </c>
-      <c r="E5" s="146"/>
-      <c r="F5" s="147"/>
-      <c r="G5" s="147"/>
+      <c r="E5" s="126"/>
+      <c r="F5" s="127"/>
+      <c r="G5" s="127"/>
     </row>
     <row r="6" spans="1:20" ht="30" x14ac:dyDescent="0.4">
       <c r="A6" s="18" t="s">
@@ -8568,11 +8588,11 @@
       <c r="C6" s="20" t="s">
         <v>1018</v>
       </c>
-      <c r="E6" s="146"/>
-      <c r="F6" s="148" t="s">
+      <c r="E6" s="126"/>
+      <c r="F6" s="128" t="s">
         <v>800</v>
       </c>
-      <c r="G6" s="147" t="s">
+      <c r="G6" s="127" t="s">
         <v>611</v>
       </c>
     </row>
@@ -8586,11 +8606,11 @@
       <c r="C7" s="20" t="s">
         <v>839</v>
       </c>
-      <c r="E7" s="146"/>
-      <c r="F7" s="148"/>
-      <c r="G7" s="147"/>
+      <c r="E7" s="126"/>
+      <c r="F7" s="128"/>
+      <c r="G7" s="127"/>
       <c r="N7" t="s">
-        <v>2123</v>
+        <v>2122</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.4">
@@ -8603,20 +8623,20 @@
       <c r="C9" s="20" t="s">
         <v>801</v>
       </c>
-      <c r="D9" s="163" t="s">
+      <c r="D9" s="104" t="s">
         <v>976</v>
       </c>
-      <c r="E9" s="143" t="s">
+      <c r="E9" s="145" t="s">
         <v>694</v>
       </c>
-      <c r="F9" s="136" t="s">
+      <c r="F9" s="143" t="s">
         <v>699</v>
       </c>
-      <c r="G9" s="134" t="s">
+      <c r="G9" s="129" t="s">
         <v>611</v>
       </c>
       <c r="H9" s="89" t="s">
-        <v>2106</v>
+        <v>2105</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -8629,15 +8649,15 @@
       <c r="C10" s="20" t="s">
         <v>801</v>
       </c>
-      <c r="D10" s="163"/>
-      <c r="E10" s="116"/>
-      <c r="F10" s="136"/>
-      <c r="G10" s="134"/>
+      <c r="D10" s="104"/>
+      <c r="E10" s="146"/>
+      <c r="F10" s="144"/>
+      <c r="G10" s="129"/>
       <c r="N10" t="s">
-        <v>2124</v>
+        <v>2123</v>
       </c>
       <c r="T10" t="s">
-        <v>2129</v>
+        <v>2128</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.4">
@@ -8650,18 +8670,18 @@
       <c r="C11" s="20" t="s">
         <v>802</v>
       </c>
-      <c r="E11" s="116"/>
-      <c r="F11" s="136" t="s">
+      <c r="E11" s="146"/>
+      <c r="F11" s="137" t="s">
         <v>698</v>
       </c>
-      <c r="G11" s="134" t="s">
+      <c r="G11" s="129" t="s">
         <v>611</v>
       </c>
       <c r="H11" s="89" t="s">
-        <v>2118</v>
+        <v>2117</v>
       </c>
       <c r="O11" t="s">
-        <v>2107</v>
+        <v>2106</v>
       </c>
     </row>
     <row r="12" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -8674,14 +8694,14 @@
       <c r="C12" s="20" t="s">
         <v>802</v>
       </c>
-      <c r="E12" s="116"/>
-      <c r="F12" s="136"/>
-      <c r="G12" s="134"/>
+      <c r="E12" s="146"/>
+      <c r="F12" s="137"/>
+      <c r="G12" s="129"/>
       <c r="P12" t="s">
-        <v>2119</v>
+        <v>2118</v>
       </c>
       <c r="T12" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.4">
@@ -8694,24 +8714,24 @@
       <c r="C13" s="20" t="s">
         <v>788</v>
       </c>
-      <c r="D13" s="163" t="s">
+      <c r="D13" s="104" t="s">
         <v>977</v>
       </c>
-      <c r="E13" s="116"/>
-      <c r="F13" s="136" t="s">
+      <c r="E13" s="146"/>
+      <c r="F13" s="137" t="s">
         <v>700</v>
       </c>
-      <c r="G13" s="134" t="s">
+      <c r="G13" s="129" t="s">
         <v>611</v>
       </c>
       <c r="H13" s="89" t="s">
-        <v>2116</v>
+        <v>2115</v>
       </c>
       <c r="P13" t="s">
-        <v>2120</v>
+        <v>2119</v>
       </c>
       <c r="T13" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -8724,15 +8744,15 @@
       <c r="C14" s="20" t="s">
         <v>788</v>
       </c>
-      <c r="D14" s="163"/>
-      <c r="E14" s="116"/>
-      <c r="F14" s="136"/>
-      <c r="G14" s="134"/>
+      <c r="D14" s="104"/>
+      <c r="E14" s="146"/>
+      <c r="F14" s="137"/>
+      <c r="G14" s="129"/>
       <c r="P14" t="s">
-        <v>2122</v>
+        <v>2121</v>
       </c>
       <c r="T14" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.4">
@@ -8745,18 +8765,18 @@
       <c r="C15" s="20" t="s">
         <v>803</v>
       </c>
-      <c r="E15" s="116"/>
-      <c r="F15" s="136" t="s">
+      <c r="E15" s="146"/>
+      <c r="F15" s="137" t="s">
         <v>701</v>
       </c>
-      <c r="G15" s="134" t="s">
+      <c r="G15" s="129" t="s">
         <v>611</v>
       </c>
       <c r="H15" s="89" t="s">
-        <v>2115</v>
+        <v>2114</v>
       </c>
       <c r="O15" t="s">
-        <v>2108</v>
+        <v>2107</v>
       </c>
     </row>
     <row r="16" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -8769,14 +8789,14 @@
       <c r="C16" s="20" t="s">
         <v>803</v>
       </c>
-      <c r="E16" s="116"/>
-      <c r="F16" s="136"/>
-      <c r="G16" s="134"/>
+      <c r="E16" s="146"/>
+      <c r="F16" s="137"/>
+      <c r="G16" s="129"/>
       <c r="P16" t="s">
-        <v>2109</v>
+        <v>2108</v>
       </c>
       <c r="T16" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.4">
@@ -8789,24 +8809,24 @@
       <c r="C17" s="20" t="s">
         <v>794</v>
       </c>
-      <c r="D17" s="163" t="s">
+      <c r="D17" s="104" t="s">
         <v>978</v>
       </c>
-      <c r="E17" s="116"/>
-      <c r="F17" s="135" t="s">
+      <c r="E17" s="146"/>
+      <c r="F17" s="138" t="s">
         <v>795</v>
       </c>
-      <c r="G17" s="134" t="s">
+      <c r="G17" s="129" t="s">
         <v>611</v>
       </c>
       <c r="H17" s="89" t="s">
-        <v>2117</v>
+        <v>2116</v>
       </c>
       <c r="P17" t="s">
-        <v>2110</v>
+        <v>2109</v>
       </c>
       <c r="T17" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="18" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -8819,15 +8839,15 @@
       <c r="C18" s="20" t="s">
         <v>794</v>
       </c>
-      <c r="D18" s="163"/>
-      <c r="E18" s="116"/>
-      <c r="F18" s="135"/>
-      <c r="G18" s="134"/>
+      <c r="D18" s="104"/>
+      <c r="E18" s="146"/>
+      <c r="F18" s="138"/>
+      <c r="G18" s="129"/>
       <c r="P18" t="s">
-        <v>2111</v>
+        <v>2110</v>
       </c>
       <c r="T18" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.4">
@@ -8840,24 +8860,24 @@
       <c r="C19" s="20" t="s">
         <v>796</v>
       </c>
-      <c r="D19" s="163" t="s">
+      <c r="D19" s="104" t="s">
         <v>979</v>
       </c>
-      <c r="E19" s="116"/>
-      <c r="F19" s="135" t="s">
+      <c r="E19" s="146"/>
+      <c r="F19" s="138" t="s">
         <v>797</v>
       </c>
-      <c r="G19" s="134" t="s">
+      <c r="G19" s="129" t="s">
         <v>611</v>
       </c>
       <c r="H19" s="89" t="s">
-        <v>2114</v>
+        <v>2113</v>
       </c>
       <c r="P19" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="T19" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="20" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -8870,12 +8890,12 @@
       <c r="C20" s="20" t="s">
         <v>796</v>
       </c>
-      <c r="D20" s="163"/>
-      <c r="E20" s="116"/>
-      <c r="F20" s="135"/>
-      <c r="G20" s="134"/>
+      <c r="D20" s="104"/>
+      <c r="E20" s="146"/>
+      <c r="F20" s="138"/>
+      <c r="G20" s="129"/>
       <c r="O20" t="s">
-        <v>2125</v>
+        <v>2124</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.4">
@@ -8888,27 +8908,27 @@
       <c r="C21" s="20" t="s">
         <v>804</v>
       </c>
-      <c r="D21" s="163" t="s">
+      <c r="D21" s="104" t="s">
         <v>980</v>
       </c>
-      <c r="E21" s="116"/>
-      <c r="F21" s="136" t="s">
+      <c r="E21" s="146"/>
+      <c r="F21" s="137" t="s">
         <v>702</v>
       </c>
-      <c r="G21" s="134" t="s">
+      <c r="G21" s="129" t="s">
         <v>611</v>
       </c>
       <c r="H21" s="89" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="P21" t="s">
+        <v>2125</v>
+      </c>
+      <c r="T21" t="s">
         <v>2126</v>
       </c>
-      <c r="T21" t="s">
+      <c r="U21" t="s">
         <v>2127</v>
-      </c>
-      <c r="U21" t="s">
-        <v>2128</v>
       </c>
     </row>
     <row r="22" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -8921,18 +8941,18 @@
       <c r="C22" s="20" t="s">
         <v>804</v>
       </c>
-      <c r="D22" s="163"/>
-      <c r="E22" s="116"/>
-      <c r="F22" s="136"/>
-      <c r="G22" s="134"/>
+      <c r="D22" s="104"/>
+      <c r="E22" s="146"/>
+      <c r="F22" s="137"/>
+      <c r="G22" s="129"/>
       <c r="P22" t="s">
-        <v>2149</v>
+        <v>2148</v>
       </c>
       <c r="T22" t="s">
+        <v>2129</v>
+      </c>
+      <c r="U22" t="s">
         <v>2130</v>
-      </c>
-      <c r="U22" t="s">
-        <v>2131</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.4">
@@ -8945,21 +8965,21 @@
       <c r="C23" s="20" t="s">
         <v>805</v>
       </c>
-      <c r="D23" s="163" t="s">
+      <c r="D23" s="104" t="s">
         <v>981</v>
       </c>
-      <c r="E23" s="116"/>
-      <c r="F23" s="136" t="s">
+      <c r="E23" s="146"/>
+      <c r="F23" s="137" t="s">
         <v>703</v>
       </c>
-      <c r="G23" s="134" t="s">
+      <c r="G23" s="129" t="s">
         <v>611</v>
       </c>
       <c r="H23" s="89" t="s">
-        <v>2121</v>
+        <v>2120</v>
       </c>
       <c r="O23" t="s">
-        <v>2133</v>
+        <v>2132</v>
       </c>
     </row>
     <row r="24" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -8972,15 +8992,15 @@
       <c r="C24" s="20" t="s">
         <v>805</v>
       </c>
-      <c r="D24" s="163"/>
-      <c r="E24" s="116"/>
-      <c r="F24" s="136"/>
-      <c r="G24" s="134"/>
+      <c r="D24" s="104"/>
+      <c r="E24" s="146"/>
+      <c r="F24" s="137"/>
+      <c r="G24" s="129"/>
       <c r="P24" t="s">
-        <v>2134</v>
+        <v>2133</v>
       </c>
       <c r="T24" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.4">
@@ -8993,21 +9013,21 @@
       <c r="C25" s="20" t="s">
         <v>807</v>
       </c>
-      <c r="D25" s="163" t="s">
+      <c r="D25" s="104" t="s">
         <v>982</v>
       </c>
-      <c r="E25" s="116"/>
-      <c r="F25" s="136" t="s">
+      <c r="E25" s="146"/>
+      <c r="F25" s="137" t="s">
         <v>704</v>
       </c>
-      <c r="G25" s="134" t="s">
+      <c r="G25" s="129" t="s">
         <v>611</v>
       </c>
       <c r="P25" t="s">
-        <v>2135</v>
+        <v>2134</v>
       </c>
       <c r="T25" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="26" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -9020,12 +9040,12 @@
       <c r="C26" s="20" t="s">
         <v>807</v>
       </c>
-      <c r="D26" s="163"/>
-      <c r="E26" s="116"/>
-      <c r="F26" s="136"/>
-      <c r="G26" s="134"/>
+      <c r="D26" s="104"/>
+      <c r="E26" s="146"/>
+      <c r="F26" s="137"/>
+      <c r="G26" s="129"/>
       <c r="O26" t="s">
-        <v>2136</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.4">
@@ -9038,21 +9058,21 @@
       <c r="C27" s="20" t="s">
         <v>808</v>
       </c>
-      <c r="D27" s="163" t="s">
+      <c r="D27" s="104" t="s">
         <v>983</v>
       </c>
-      <c r="E27" s="116"/>
-      <c r="F27" s="136" t="s">
+      <c r="E27" s="146"/>
+      <c r="F27" s="137" t="s">
         <v>2080</v>
       </c>
-      <c r="G27" s="134" t="s">
+      <c r="G27" s="129" t="s">
         <v>611</v>
       </c>
       <c r="P27" t="s">
         <v>626</v>
       </c>
       <c r="T27" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="28" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -9065,15 +9085,15 @@
       <c r="C28" s="20" t="s">
         <v>808</v>
       </c>
-      <c r="D28" s="163"/>
-      <c r="E28" s="117"/>
-      <c r="F28" s="136"/>
-      <c r="G28" s="134"/>
+      <c r="D28" s="104"/>
+      <c r="E28" s="147"/>
+      <c r="F28" s="137"/>
+      <c r="G28" s="129"/>
       <c r="P28" t="s">
         <v>643</v>
       </c>
       <c r="T28" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.4">
@@ -9086,13 +9106,13 @@
       <c r="C29" s="20" t="s">
         <v>809</v>
       </c>
-      <c r="E29" s="144" t="s">
+      <c r="E29" s="130" t="s">
         <v>695</v>
       </c>
-      <c r="F29" s="139" t="s">
+      <c r="F29" s="141" t="s">
         <v>705</v>
       </c>
-      <c r="G29" s="153" t="s">
+      <c r="G29" s="135" t="s">
         <v>873</v>
       </c>
       <c r="P29" t="s">
@@ -9109,9 +9129,9 @@
       <c r="C30" s="20" t="s">
         <v>809</v>
       </c>
-      <c r="E30" s="145"/>
-      <c r="F30" s="140"/>
-      <c r="G30" s="154"/>
+      <c r="E30" s="131"/>
+      <c r="F30" s="142"/>
+      <c r="G30" s="136"/>
       <c r="P30" t="s">
         <v>653</v>
       </c>
@@ -9126,16 +9146,16 @@
       <c r="C31" s="20" t="s">
         <v>810</v>
       </c>
-      <c r="D31" s="163" t="s">
+      <c r="D31" s="104" t="s">
         <v>984</v>
       </c>
-      <c r="E31" s="143" t="s">
+      <c r="E31" s="145" t="s">
         <v>694</v>
       </c>
-      <c r="F31" s="141" t="s">
+      <c r="F31" s="143" t="s">
         <v>706</v>
       </c>
-      <c r="G31" s="151" t="s">
+      <c r="G31" s="133" t="s">
         <v>611</v>
       </c>
       <c r="P31" t="s">
@@ -9152,10 +9172,10 @@
       <c r="C32" s="20" t="s">
         <v>810</v>
       </c>
-      <c r="D32" s="163"/>
-      <c r="E32" s="117"/>
-      <c r="F32" s="142"/>
-      <c r="G32" s="152"/>
+      <c r="D32" s="104"/>
+      <c r="E32" s="147"/>
+      <c r="F32" s="144"/>
+      <c r="G32" s="134"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A34" s="18" t="s">
@@ -9170,13 +9190,13 @@
       <c r="D34" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E34" s="144" t="s">
+      <c r="E34" s="130" t="s">
         <v>695</v>
       </c>
-      <c r="F34" s="149" t="s">
+      <c r="F34" s="116" t="s">
         <v>709</v>
       </c>
-      <c r="G34" s="150" t="s">
+      <c r="G34" s="132" t="s">
         <v>614</v>
       </c>
     </row>
@@ -9190,9 +9210,9 @@
       <c r="C35" s="20" t="s">
         <v>806</v>
       </c>
-      <c r="E35" s="145"/>
-      <c r="F35" s="149"/>
-      <c r="G35" s="150"/>
+      <c r="E35" s="131"/>
+      <c r="F35" s="116"/>
+      <c r="G35" s="132"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A37" s="18" t="s">
@@ -9204,16 +9224,16 @@
       <c r="C37" s="20" t="s">
         <v>831</v>
       </c>
-      <c r="D37" s="163" t="s">
+      <c r="D37" s="104" t="s">
         <v>993</v>
       </c>
-      <c r="E37" s="137" t="s">
+      <c r="E37" s="139" t="s">
         <v>694</v>
       </c>
-      <c r="F37" s="136" t="s">
+      <c r="F37" s="137" t="s">
         <v>711</v>
       </c>
-      <c r="G37" s="134" t="s">
+      <c r="G37" s="129" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9227,10 +9247,10 @@
       <c r="C38" s="20" t="s">
         <v>831</v>
       </c>
-      <c r="D38" s="163"/>
-      <c r="E38" s="138"/>
-      <c r="F38" s="136"/>
-      <c r="G38" s="134"/>
+      <c r="D38" s="104"/>
+      <c r="E38" s="140"/>
+      <c r="F38" s="137"/>
+      <c r="G38" s="129"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A39" s="18" t="s">
@@ -9242,14 +9262,14 @@
       <c r="C39" s="20" t="s">
         <v>566</v>
       </c>
-      <c r="D39" s="163" t="s">
+      <c r="D39" s="104" t="s">
         <v>994</v>
       </c>
-      <c r="E39" s="138"/>
-      <c r="F39" s="136" t="s">
+      <c r="E39" s="140"/>
+      <c r="F39" s="137" t="s">
         <v>712</v>
       </c>
-      <c r="G39" s="134" t="s">
+      <c r="G39" s="129" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9263,10 +9283,10 @@
       <c r="C40" s="20" t="s">
         <v>566</v>
       </c>
-      <c r="D40" s="163"/>
-      <c r="E40" s="138"/>
-      <c r="F40" s="136"/>
-      <c r="G40" s="134"/>
+      <c r="D40" s="104"/>
+      <c r="E40" s="140"/>
+      <c r="F40" s="137"/>
+      <c r="G40" s="129"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A41" s="18" t="s">
@@ -9278,14 +9298,14 @@
       <c r="C41" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="D41" s="163" t="s">
+      <c r="D41" s="104" t="s">
         <v>995</v>
       </c>
-      <c r="E41" s="138"/>
-      <c r="F41" s="136" t="s">
+      <c r="E41" s="140"/>
+      <c r="F41" s="137" t="s">
         <v>717</v>
       </c>
-      <c r="G41" s="134" t="s">
+      <c r="G41" s="129" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9299,10 +9319,10 @@
       <c r="C42" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="D42" s="163"/>
-      <c r="E42" s="138"/>
-      <c r="F42" s="136"/>
-      <c r="G42" s="134"/>
+      <c r="D42" s="104"/>
+      <c r="E42" s="140"/>
+      <c r="F42" s="137"/>
+      <c r="G42" s="129"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A43" s="18" t="s">
@@ -9314,14 +9334,14 @@
       <c r="C43" s="20" t="s">
         <v>833</v>
       </c>
-      <c r="D43" s="163" t="s">
+      <c r="D43" s="104" t="s">
         <v>996</v>
       </c>
-      <c r="E43" s="138"/>
-      <c r="F43" s="136" t="s">
+      <c r="E43" s="140"/>
+      <c r="F43" s="137" t="s">
         <v>713</v>
       </c>
-      <c r="G43" s="134" t="s">
+      <c r="G43" s="129" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9335,10 +9355,10 @@
       <c r="C44" s="20" t="s">
         <v>833</v>
       </c>
-      <c r="D44" s="163"/>
-      <c r="E44" s="138"/>
-      <c r="F44" s="136"/>
-      <c r="G44" s="134"/>
+      <c r="D44" s="104"/>
+      <c r="E44" s="140"/>
+      <c r="F44" s="137"/>
+      <c r="G44" s="129"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A45" s="18" t="s">
@@ -9350,14 +9370,14 @@
       <c r="C45" s="20" t="s">
         <v>834</v>
       </c>
-      <c r="D45" s="163" t="s">
+      <c r="D45" s="104" t="s">
         <v>997</v>
       </c>
-      <c r="E45" s="138"/>
-      <c r="F45" s="136" t="s">
+      <c r="E45" s="140"/>
+      <c r="F45" s="137" t="s">
         <v>714</v>
       </c>
-      <c r="G45" s="134" t="s">
+      <c r="G45" s="129" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9371,10 +9391,10 @@
       <c r="C46" s="20" t="s">
         <v>834</v>
       </c>
-      <c r="D46" s="163"/>
-      <c r="E46" s="138"/>
-      <c r="F46" s="136"/>
-      <c r="G46" s="134"/>
+      <c r="D46" s="104"/>
+      <c r="E46" s="140"/>
+      <c r="F46" s="137"/>
+      <c r="G46" s="129"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A47" s="18" t="s">
@@ -9386,14 +9406,14 @@
       <c r="C47" s="20" t="s">
         <v>835</v>
       </c>
-      <c r="D47" s="163" t="s">
+      <c r="D47" s="104" t="s">
         <v>998</v>
       </c>
-      <c r="E47" s="138"/>
-      <c r="F47" s="136" t="s">
+      <c r="E47" s="140"/>
+      <c r="F47" s="137" t="s">
         <v>864</v>
       </c>
-      <c r="G47" s="134" t="s">
+      <c r="G47" s="129" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9407,10 +9427,10 @@
       <c r="C48" s="20" t="s">
         <v>835</v>
       </c>
-      <c r="D48" s="163"/>
-      <c r="E48" s="138"/>
-      <c r="F48" s="136"/>
-      <c r="G48" s="134"/>
+      <c r="D48" s="104"/>
+      <c r="E48" s="140"/>
+      <c r="F48" s="137"/>
+      <c r="G48" s="129"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A49" s="18" t="s">
@@ -9422,14 +9442,14 @@
       <c r="C49" s="20" t="s">
         <v>836</v>
       </c>
-      <c r="D49" s="163" t="s">
+      <c r="D49" s="104" t="s">
         <v>999</v>
       </c>
-      <c r="E49" s="138"/>
-      <c r="F49" s="136" t="s">
+      <c r="E49" s="140"/>
+      <c r="F49" s="137" t="s">
         <v>715</v>
       </c>
-      <c r="G49" s="134" t="s">
+      <c r="G49" s="129" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9443,10 +9463,10 @@
       <c r="C50" s="20" t="s">
         <v>836</v>
       </c>
-      <c r="D50" s="163"/>
-      <c r="E50" s="138"/>
-      <c r="F50" s="136"/>
-      <c r="G50" s="134"/>
+      <c r="D50" s="104"/>
+      <c r="E50" s="140"/>
+      <c r="F50" s="137"/>
+      <c r="G50" s="129"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A51" s="18" t="s">
@@ -9458,14 +9478,14 @@
       <c r="C51" s="20" t="s">
         <v>860</v>
       </c>
-      <c r="D51" s="163" t="s">
+      <c r="D51" s="104" t="s">
         <v>1000</v>
       </c>
-      <c r="E51" s="138"/>
-      <c r="F51" s="135" t="s">
+      <c r="E51" s="140"/>
+      <c r="F51" s="138" t="s">
         <v>798</v>
       </c>
-      <c r="G51" s="134" t="s">
+      <c r="G51" s="129" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9479,10 +9499,10 @@
       <c r="C52" s="20" t="s">
         <v>860</v>
       </c>
-      <c r="D52" s="163"/>
-      <c r="E52" s="138"/>
-      <c r="F52" s="135"/>
-      <c r="G52" s="134"/>
+      <c r="D52" s="104"/>
+      <c r="E52" s="140"/>
+      <c r="F52" s="138"/>
+      <c r="G52" s="129"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A53" s="18" t="s">
@@ -9494,14 +9514,14 @@
       <c r="C53" s="20" t="s">
         <v>837</v>
       </c>
-      <c r="D53" s="163" t="s">
+      <c r="D53" s="104" t="s">
         <v>1001</v>
       </c>
-      <c r="E53" s="138"/>
-      <c r="F53" s="136" t="s">
+      <c r="E53" s="140"/>
+      <c r="F53" s="137" t="s">
         <v>716</v>
       </c>
-      <c r="G53" s="134" t="s">
+      <c r="G53" s="129" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9515,16 +9535,16 @@
       <c r="C54" s="20" t="s">
         <v>837</v>
       </c>
-      <c r="D54" s="163"/>
-      <c r="E54" s="138"/>
-      <c r="F54" s="136"/>
-      <c r="G54" s="134"/>
+      <c r="D54" s="104"/>
+      <c r="E54" s="140"/>
+      <c r="F54" s="137"/>
+      <c r="G54" s="129"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="E56" s="104" t="s">
+      <c r="E56" s="108" t="s">
         <v>790</v>
       </c>
-      <c r="F56" s="104"/>
+      <c r="F56" s="108"/>
       <c r="G56" s="28" t="s">
         <v>613</v>
       </c>
@@ -9560,7 +9580,7 @@
       <c r="D58" s="32" t="s">
         <v>616</v>
       </c>
-      <c r="E58" s="108" t="s">
+      <c r="E58" s="160" t="s">
         <v>694</v>
       </c>
       <c r="F58" s="61" t="s">
@@ -9581,7 +9601,7 @@
       <c r="D59" s="32" t="s">
         <v>616</v>
       </c>
-      <c r="E59" s="109"/>
+      <c r="E59" s="161"/>
       <c r="F59" s="63" t="s">
         <v>2098</v>
       </c>
@@ -9600,7 +9620,7 @@
       <c r="D60" s="32" t="s">
         <v>616</v>
       </c>
-      <c r="E60" s="109"/>
+      <c r="E60" s="161"/>
       <c r="F60" s="65" t="s">
         <v>2099</v>
       </c>
@@ -9619,7 +9639,7 @@
       <c r="D61" s="32" t="s">
         <v>2052</v>
       </c>
-      <c r="E61" s="118"/>
+      <c r="E61" s="163"/>
       <c r="F61" s="27" t="s">
         <v>923</v>
       </c>
@@ -9673,7 +9693,7 @@
         <v>611</v>
       </c>
       <c r="H63" s="90" t="s">
-        <v>2104</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="24.75" thickBot="1" x14ac:dyDescent="0.45">
@@ -9752,7 +9772,7 @@
       <c r="C67" s="20" t="s">
         <v>567</v>
       </c>
-      <c r="E67" s="108" t="s">
+      <c r="E67" s="160" t="s">
         <v>694</v>
       </c>
       <c r="F67" s="34" t="s">
@@ -9773,7 +9793,7 @@
       <c r="D68" s="32" t="s">
         <v>2054</v>
       </c>
-      <c r="E68" s="109"/>
+      <c r="E68" s="161"/>
       <c r="F68" s="27" t="s">
         <v>929</v>
       </c>
@@ -9794,7 +9814,7 @@
       <c r="D69" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E69" s="110" t="s">
+      <c r="E69" s="124" t="s">
         <v>695</v>
       </c>
       <c r="F69" s="73" t="s">
@@ -9817,7 +9837,7 @@
       <c r="D70" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E70" s="111"/>
+      <c r="E70" s="156"/>
       <c r="F70" s="73" t="s">
         <v>931</v>
       </c>
@@ -9838,7 +9858,7 @@
       <c r="D71" s="32" t="s">
         <v>2055</v>
       </c>
-      <c r="E71" s="108" t="s">
+      <c r="E71" s="160" t="s">
         <v>694</v>
       </c>
       <c r="F71" s="27" t="s">
@@ -9861,7 +9881,7 @@
       <c r="D72" s="32" t="s">
         <v>984</v>
       </c>
-      <c r="E72" s="109"/>
+      <c r="E72" s="161"/>
       <c r="F72" s="27" t="s">
         <v>933</v>
       </c>
@@ -9882,7 +9902,7 @@
       <c r="D73" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E73" s="110" t="s">
+      <c r="E73" s="124" t="s">
         <v>695</v>
       </c>
       <c r="F73" s="73" t="s">
@@ -9905,7 +9925,7 @@
       <c r="D74" s="32" t="s">
         <v>605</v>
       </c>
-      <c r="E74" s="111"/>
+      <c r="E74" s="156"/>
       <c r="F74" s="73" t="s">
         <v>708</v>
       </c>
@@ -9992,7 +10012,7 @@
       <c r="C78" s="20" t="s">
         <v>859</v>
       </c>
-      <c r="E78" s="110" t="s">
+      <c r="E78" s="124" t="s">
         <v>695</v>
       </c>
       <c r="F78" s="73" t="s">
@@ -10015,7 +10035,7 @@
       <c r="D79" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E79" s="115"/>
+      <c r="E79" s="162"/>
       <c r="F79" s="73" t="s">
         <v>936</v>
       </c>
@@ -10056,11 +10076,11 @@
       <c r="C81" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E81" s="105" t="s">
+      <c r="E81" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F81" s="105"/>
-      <c r="G81" s="104" t="s">
+      <c r="F81" s="107"/>
+      <c r="G81" s="108" t="s">
         <v>611</v>
       </c>
     </row>
@@ -10074,9 +10094,9 @@
       <c r="C82" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E82" s="106"/>
-      <c r="F82" s="107"/>
-      <c r="G82" s="125"/>
+      <c r="E82" s="114"/>
+      <c r="F82" s="115"/>
+      <c r="G82" s="109"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E83" s="54"/>
@@ -10084,10 +10104,10 @@
       <c r="G83" s="23"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E84" s="104" t="s">
+      <c r="E84" s="108" t="s">
         <v>868</v>
       </c>
-      <c r="F84" s="104"/>
+      <c r="F84" s="108"/>
       <c r="G84" s="28" t="s">
         <v>613</v>
       </c>
@@ -10123,7 +10143,7 @@
       <c r="D86" s="32" t="s">
         <v>985</v>
       </c>
-      <c r="E86" s="113" t="s">
+      <c r="E86" s="122" t="s">
         <v>694</v>
       </c>
       <c r="F86" s="27" t="s">
@@ -10146,7 +10166,7 @@
       <c r="D87" s="32" t="s">
         <v>986</v>
       </c>
-      <c r="E87" s="116"/>
+      <c r="E87" s="146"/>
       <c r="F87" s="27" t="s">
         <v>939</v>
       </c>
@@ -10167,7 +10187,7 @@
       <c r="D88" s="32" t="s">
         <v>987</v>
       </c>
-      <c r="E88" s="116"/>
+      <c r="E88" s="146"/>
       <c r="F88" s="27" t="s">
         <v>940</v>
       </c>
@@ -10188,7 +10208,7 @@
       <c r="D89" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E89" s="110" t="s">
+      <c r="E89" s="124" t="s">
         <v>695</v>
       </c>
       <c r="F89" s="73" t="s">
@@ -10211,7 +10231,7 @@
       <c r="D90" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E90" s="111"/>
+      <c r="E90" s="156"/>
       <c r="F90" s="73" t="s">
         <v>942</v>
       </c>
@@ -10232,7 +10252,7 @@
       <c r="D91" s="32" t="s">
         <v>987</v>
       </c>
-      <c r="E91" s="113" t="s">
+      <c r="E91" s="122" t="s">
         <v>694</v>
       </c>
       <c r="F91" s="27" t="s">
@@ -10255,7 +10275,7 @@
       <c r="D92" s="32" t="s">
         <v>984</v>
       </c>
-      <c r="E92" s="116"/>
+      <c r="E92" s="146"/>
       <c r="F92" s="27" t="s">
         <v>944</v>
       </c>
@@ -10276,7 +10296,7 @@
       <c r="D93" s="32" t="s">
         <v>988</v>
       </c>
-      <c r="E93" s="116"/>
+      <c r="E93" s="146"/>
       <c r="F93" s="27" t="s">
         <v>2067</v>
       </c>
@@ -10297,7 +10317,7 @@
       <c r="D94" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E94" s="110" t="s">
+      <c r="E94" s="124" t="s">
         <v>695</v>
       </c>
       <c r="F94" s="73" t="s">
@@ -10320,7 +10340,7 @@
       <c r="D95" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E95" s="111"/>
+      <c r="E95" s="156"/>
       <c r="F95" s="73" t="s">
         <v>946</v>
       </c>
@@ -10338,7 +10358,7 @@
       <c r="C96" s="20" t="s">
         <v>819</v>
       </c>
-      <c r="E96" s="111"/>
+      <c r="E96" s="156"/>
       <c r="F96" s="73" t="s">
         <v>947</v>
       </c>
@@ -10401,7 +10421,7 @@
       <c r="D99" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E99" s="110" t="s">
+      <c r="E99" s="124" t="s">
         <v>695</v>
       </c>
       <c r="F99" s="73" t="s">
@@ -10424,7 +10444,7 @@
       <c r="D100" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E100" s="111"/>
+      <c r="E100" s="156"/>
       <c r="F100" s="73" t="s">
         <v>951</v>
       </c>
@@ -10588,11 +10608,11 @@
       <c r="C108" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E108" s="105" t="s">
+      <c r="E108" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F108" s="105"/>
-      <c r="G108" s="104" t="s">
+      <c r="F108" s="107"/>
+      <c r="G108" s="108" t="s">
         <v>611</v>
       </c>
     </row>
@@ -10606,15 +10626,15 @@
       <c r="C109" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E109" s="106"/>
-      <c r="F109" s="107"/>
-      <c r="G109" s="125"/>
+      <c r="E109" s="114"/>
+      <c r="F109" s="115"/>
+      <c r="G109" s="109"/>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="E111" s="104" t="s">
+      <c r="E111" s="108" t="s">
         <v>868</v>
       </c>
-      <c r="F111" s="104"/>
+      <c r="F111" s="108"/>
       <c r="G111" s="28" t="s">
         <v>613</v>
       </c>
@@ -10691,7 +10711,7 @@
       <c r="C115" s="20" t="s">
         <v>914</v>
       </c>
-      <c r="E115" s="110" t="s">
+      <c r="E115" s="124" t="s">
         <v>695</v>
       </c>
       <c r="F115" s="78" t="s">
@@ -10714,7 +10734,7 @@
       <c r="D116" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E116" s="111"/>
+      <c r="E116" s="156"/>
       <c r="F116" s="78" t="s">
         <v>919</v>
       </c>
@@ -10735,7 +10755,7 @@
       <c r="D117" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E117" s="111"/>
+      <c r="E117" s="156"/>
       <c r="F117" s="78" t="s">
         <v>920</v>
       </c>
@@ -10756,7 +10776,7 @@
       <c r="D118" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E118" s="112"/>
+      <c r="E118" s="125"/>
       <c r="F118" s="78" t="s">
         <v>921</v>
       </c>
@@ -10795,11 +10815,11 @@
       <c r="C120" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E120" s="105" t="s">
+      <c r="E120" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F120" s="105"/>
-      <c r="G120" s="104" t="s">
+      <c r="F120" s="107"/>
+      <c r="G120" s="108" t="s">
         <v>611</v>
       </c>
     </row>
@@ -10813,9 +10833,9 @@
       <c r="C121" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E121" s="105"/>
-      <c r="F121" s="105"/>
-      <c r="G121" s="104"/>
+      <c r="E121" s="107"/>
+      <c r="F121" s="107"/>
+      <c r="G121" s="108"/>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.4">
       <c r="E122" s="55"/>
@@ -10856,7 +10876,7 @@
         <v>1021</v>
       </c>
       <c r="D125" s="45"/>
-      <c r="E125" s="160" t="s">
+      <c r="E125" s="119" t="s">
         <v>694</v>
       </c>
       <c r="F125" s="24" t="s">
@@ -10877,7 +10897,7 @@
         <v>1022</v>
       </c>
       <c r="D126" s="45"/>
-      <c r="E126" s="161"/>
+      <c r="E126" s="120"/>
       <c r="F126" s="51" t="s">
         <v>1028</v>
       </c>
@@ -10885,7 +10905,7 @@
         <v>611</v>
       </c>
       <c r="H126" s="89" t="s">
-        <v>2160</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.4">
@@ -10899,7 +10919,7 @@
         <v>1023</v>
       </c>
       <c r="D127" s="45"/>
-      <c r="E127" s="161"/>
+      <c r="E127" s="120"/>
       <c r="F127" s="24" t="s">
         <v>1029</v>
       </c>
@@ -10918,7 +10938,7 @@
         <v>1024</v>
       </c>
       <c r="D128" s="45"/>
-      <c r="E128" s="162"/>
+      <c r="E128" s="121"/>
       <c r="F128" s="24" t="s">
         <v>1030</v>
       </c>
@@ -10937,10 +10957,10 @@
         <v>601</v>
       </c>
       <c r="D129" s="45"/>
-      <c r="E129" s="158" t="s">
+      <c r="E129" s="117" t="s">
         <v>620</v>
       </c>
-      <c r="F129" s="159"/>
+      <c r="F129" s="118"/>
       <c r="G129" s="26" t="s">
         <v>611</v>
       </c>
@@ -10996,7 +11016,7 @@
         <v>1025</v>
       </c>
       <c r="D133" s="45"/>
-      <c r="E133" s="113" t="s">
+      <c r="E133" s="122" t="s">
         <v>694</v>
       </c>
       <c r="F133" s="24" t="s">
@@ -11006,7 +11026,7 @@
         <v>611</v>
       </c>
       <c r="H133" s="89" t="s">
-        <v>2161</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.4">
@@ -11020,7 +11040,7 @@
         <v>1026</v>
       </c>
       <c r="D134" s="45"/>
-      <c r="E134" s="114"/>
+      <c r="E134" s="123"/>
       <c r="F134" s="24" t="s">
         <v>2068</v>
       </c>
@@ -11039,10 +11059,10 @@
       <c r="H136" s="91"/>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="E138" s="157" t="s">
+      <c r="E138" s="110" t="s">
         <v>907</v>
       </c>
-      <c r="F138" s="157"/>
+      <c r="F138" s="110"/>
       <c r="G138" s="28" t="s">
         <v>613</v>
       </c>
@@ -11100,7 +11120,7 @@
       <c r="D141" s="32" t="s">
         <v>2058</v>
       </c>
-      <c r="E141" s="113" t="s">
+      <c r="E141" s="122" t="s">
         <v>694</v>
       </c>
       <c r="F141" s="27" t="s">
@@ -11123,7 +11143,7 @@
       <c r="D142" s="32" t="s">
         <v>2059</v>
       </c>
-      <c r="E142" s="114"/>
+      <c r="E142" s="123"/>
       <c r="F142" s="27" t="s">
         <v>719</v>
       </c>
@@ -11141,11 +11161,11 @@
       <c r="C143" s="20" t="s">
         <v>589</v>
       </c>
-      <c r="E143" s="105" t="s">
+      <c r="E143" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F143" s="105"/>
-      <c r="G143" s="104" t="s">
+      <c r="F143" s="107"/>
+      <c r="G143" s="108" t="s">
         <v>611</v>
       </c>
     </row>
@@ -11159,9 +11179,9 @@
       <c r="C144" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E144" s="105"/>
-      <c r="F144" s="105"/>
-      <c r="G144" s="104"/>
+      <c r="E144" s="107"/>
+      <c r="F144" s="107"/>
+      <c r="G144" s="108"/>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A145" s="18" t="s">
@@ -11173,15 +11193,15 @@
       <c r="C145" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E145" s="105"/>
-      <c r="F145" s="105"/>
-      <c r="G145" s="104"/>
+      <c r="E145" s="107"/>
+      <c r="F145" s="107"/>
+      <c r="G145" s="108"/>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="E147" s="157" t="s">
+      <c r="E147" s="110" t="s">
         <v>908</v>
       </c>
-      <c r="F147" s="157"/>
+      <c r="F147" s="110"/>
       <c r="G147" s="28" t="s">
         <v>613</v>
       </c>
@@ -11257,7 +11277,7 @@
       <c r="C151" s="20" t="s">
         <v>590</v>
       </c>
-      <c r="E151" s="110" t="s">
+      <c r="E151" s="124" t="s">
         <v>695</v>
       </c>
       <c r="F151" s="78" t="s">
@@ -11277,7 +11297,7 @@
       <c r="C152" s="20" t="s">
         <v>591</v>
       </c>
-      <c r="E152" s="111"/>
+      <c r="E152" s="156"/>
       <c r="F152" s="78" t="s">
         <v>722</v>
       </c>
@@ -11295,7 +11315,7 @@
       <c r="C153" s="20" t="s">
         <v>596</v>
       </c>
-      <c r="E153" s="111"/>
+      <c r="E153" s="156"/>
       <c r="F153" s="78" t="s">
         <v>723</v>
       </c>
@@ -11313,7 +11333,7 @@
       <c r="C154" s="20" t="s">
         <v>597</v>
       </c>
-      <c r="E154" s="111"/>
+      <c r="E154" s="156"/>
       <c r="F154" s="78" t="s">
         <v>724</v>
       </c>
@@ -11331,7 +11351,7 @@
       <c r="C155" s="20" t="s">
         <v>592</v>
       </c>
-      <c r="E155" s="115"/>
+      <c r="E155" s="162"/>
       <c r="F155" s="78" t="s">
         <v>725</v>
       </c>
@@ -11352,7 +11372,7 @@
       <c r="D156" s="32" t="s">
         <v>2060</v>
       </c>
-      <c r="E156" s="113" t="s">
+      <c r="E156" s="122" t="s">
         <v>694</v>
       </c>
       <c r="F156" s="24" t="s">
@@ -11375,7 +11395,7 @@
       <c r="D157" s="32" t="s">
         <v>2061</v>
       </c>
-      <c r="E157" s="116"/>
+      <c r="E157" s="146"/>
       <c r="F157" s="24" t="s">
         <v>727</v>
       </c>
@@ -11396,7 +11416,7 @@
       <c r="D158" s="32" t="s">
         <v>2062</v>
       </c>
-      <c r="E158" s="116"/>
+      <c r="E158" s="146"/>
       <c r="F158" s="24" t="s">
         <v>728</v>
       </c>
@@ -11417,7 +11437,7 @@
       <c r="D159" s="32" t="s">
         <v>2063</v>
       </c>
-      <c r="E159" s="116"/>
+      <c r="E159" s="146"/>
       <c r="F159" s="24" t="s">
         <v>729</v>
       </c>
@@ -11438,7 +11458,7 @@
       <c r="D160" s="33" t="s">
         <v>2101</v>
       </c>
-      <c r="E160" s="117"/>
+      <c r="E160" s="147"/>
       <c r="F160" s="24" t="s">
         <v>730</v>
       </c>
@@ -11459,10 +11479,10 @@
       <c r="C161" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E161" s="105" t="s">
+      <c r="E161" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F161" s="105"/>
+      <c r="F161" s="107"/>
       <c r="G161" s="26" t="s">
         <v>611</v>
       </c>
@@ -11487,10 +11507,10 @@
       <c r="G164"/>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="E165" s="122" t="s">
+      <c r="E165" s="111" t="s">
         <v>2089</v>
       </c>
-      <c r="F165" s="122"/>
+      <c r="F165" s="111"/>
       <c r="G165" s="28" t="s">
         <v>613</v>
       </c>
@@ -11528,14 +11548,14 @@
       <c r="E167" s="77" t="s">
         <v>694</v>
       </c>
-      <c r="F167" s="123" t="s">
+      <c r="F167" s="112" t="s">
         <v>732</v>
       </c>
       <c r="G167" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H167" s="90" t="s">
-        <v>2105</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.4">
@@ -11550,7 +11570,7 @@
       </c>
       <c r="D168" s="45"/>
       <c r="E168" s="77"/>
-      <c r="F168" s="123"/>
+      <c r="F168" s="112"/>
       <c r="G168" s="24" t="s">
         <v>611</v>
       </c>
@@ -11565,10 +11585,10 @@
       <c r="C169" s="18" t="s">
         <v>627</v>
       </c>
-      <c r="E169" s="110" t="s">
+      <c r="E169" s="124" t="s">
         <v>695</v>
       </c>
-      <c r="F169" s="124" t="s">
+      <c r="F169" s="113" t="s">
         <v>733</v>
       </c>
       <c r="G169" s="78" t="s">
@@ -11587,8 +11607,8 @@
         <v>627</v>
       </c>
       <c r="D170" s="45"/>
-      <c r="E170" s="112"/>
-      <c r="F170" s="124"/>
+      <c r="E170" s="125"/>
+      <c r="F170" s="113"/>
       <c r="G170" s="78" t="s">
         <v>611</v>
       </c>
@@ -11603,10 +11623,10 @@
       <c r="C171" s="18" t="s">
         <v>628</v>
       </c>
-      <c r="E171" s="110" t="s">
+      <c r="E171" s="124" t="s">
         <v>695</v>
       </c>
-      <c r="F171" s="149" t="s">
+      <c r="F171" s="116" t="s">
         <v>791</v>
       </c>
       <c r="G171" s="72" t="s">
@@ -11624,8 +11644,8 @@
         <v>628</v>
       </c>
       <c r="D172" s="45"/>
-      <c r="E172" s="112"/>
-      <c r="F172" s="149"/>
+      <c r="E172" s="125"/>
+      <c r="F172" s="116"/>
       <c r="G172" s="72" t="s">
         <v>873</v>
       </c>
@@ -11640,11 +11660,11 @@
       <c r="C173" s="18" t="s">
         <v>874</v>
       </c>
-      <c r="D173" s="163" t="s">
+      <c r="D173" s="104" t="s">
         <v>1003</v>
       </c>
       <c r="E173" s="77"/>
-      <c r="F173" s="123" t="s">
+      <c r="F173" s="112" t="s">
         <v>883</v>
       </c>
       <c r="G173" s="24" t="s">
@@ -11661,9 +11681,9 @@
       <c r="C174" t="s">
         <v>874</v>
       </c>
-      <c r="D174" s="163"/>
+      <c r="D174" s="104"/>
       <c r="E174" s="77"/>
-      <c r="F174" s="123"/>
+      <c r="F174" s="112"/>
       <c r="G174" s="24" t="s">
         <v>611</v>
       </c>
@@ -11678,11 +11698,11 @@
       <c r="C175" s="18" t="s">
         <v>629</v>
       </c>
-      <c r="D175" s="163" t="s">
+      <c r="D175" s="104" t="s">
         <v>1004</v>
       </c>
       <c r="E175" s="77"/>
-      <c r="F175" s="123" t="s">
+      <c r="F175" s="112" t="s">
         <v>734</v>
       </c>
       <c r="G175" s="24" t="s">
@@ -11699,9 +11719,9 @@
       <c r="C176" t="s">
         <v>629</v>
       </c>
-      <c r="D176" s="163"/>
+      <c r="D176" s="104"/>
       <c r="E176" s="77"/>
-      <c r="F176" s="123"/>
+      <c r="F176" s="112"/>
       <c r="G176" s="24" t="s">
         <v>611</v>
       </c>
@@ -11717,14 +11737,14 @@
         <v>630</v>
       </c>
       <c r="E177" s="77"/>
-      <c r="F177" s="123" t="s">
+      <c r="F177" s="112" t="s">
         <v>735</v>
       </c>
       <c r="G177" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H177" s="89" t="s">
-        <v>2137</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.4">
@@ -11739,7 +11759,7 @@
       </c>
       <c r="D178" s="45"/>
       <c r="E178" s="77"/>
-      <c r="F178" s="123"/>
+      <c r="F178" s="112"/>
       <c r="G178" s="24" t="s">
         <v>611</v>
       </c>
@@ -11754,11 +11774,11 @@
       <c r="C179" s="18" t="s">
         <v>631</v>
       </c>
-      <c r="D179" s="163" t="s">
+      <c r="D179" s="104" t="s">
         <v>1005</v>
       </c>
       <c r="E179" s="77"/>
-      <c r="F179" s="123" t="s">
+      <c r="F179" s="112" t="s">
         <v>736</v>
       </c>
       <c r="G179" s="24" t="s">
@@ -11775,9 +11795,9 @@
       <c r="C180" t="s">
         <v>631</v>
       </c>
-      <c r="D180" s="163"/>
+      <c r="D180" s="104"/>
       <c r="E180" s="77"/>
-      <c r="F180" s="123"/>
+      <c r="F180" s="112"/>
       <c r="G180" s="24" t="s">
         <v>611</v>
       </c>
@@ -11792,10 +11812,10 @@
       <c r="C181" s="18" t="s">
         <v>632</v>
       </c>
-      <c r="E181" s="110" t="s">
+      <c r="E181" s="124" t="s">
         <v>695</v>
       </c>
-      <c r="F181" s="124" t="s">
+      <c r="F181" s="113" t="s">
         <v>737</v>
       </c>
       <c r="G181" s="78" t="s">
@@ -11813,8 +11833,8 @@
         <v>632</v>
       </c>
       <c r="D182" s="45"/>
-      <c r="E182" s="112"/>
-      <c r="F182" s="124"/>
+      <c r="E182" s="125"/>
+      <c r="F182" s="113"/>
       <c r="G182" s="78" t="s">
         <v>611</v>
       </c>
@@ -11829,13 +11849,13 @@
       <c r="C184" s="18" t="s">
         <v>635</v>
       </c>
-      <c r="D184" s="163" t="s">
+      <c r="D184" s="104" t="s">
         <v>1008</v>
       </c>
       <c r="E184" s="79" t="s">
         <v>694</v>
       </c>
-      <c r="F184" s="123" t="s">
+      <c r="F184" s="112" t="s">
         <v>890</v>
       </c>
       <c r="G184" s="24" t="s">
@@ -11852,9 +11872,9 @@
       <c r="C185" t="s">
         <v>635</v>
       </c>
-      <c r="D185" s="163"/>
+      <c r="D185" s="104"/>
       <c r="E185" s="77"/>
-      <c r="F185" s="123"/>
+      <c r="F185" s="112"/>
       <c r="G185" s="24" t="s">
         <v>611</v>
       </c>
@@ -11869,10 +11889,10 @@
       <c r="C186" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="E186" s="110" t="s">
+      <c r="E186" s="124" t="s">
         <v>695</v>
       </c>
-      <c r="F186" s="119" t="s">
+      <c r="F186" s="157" t="s">
         <v>2094</v>
       </c>
       <c r="G186" s="92" t="s">
@@ -11890,8 +11910,8 @@
         <v>636</v>
       </c>
       <c r="D187" s="45"/>
-      <c r="E187" s="111"/>
-      <c r="F187" s="120"/>
+      <c r="E187" s="156"/>
+      <c r="F187" s="158"/>
       <c r="G187" s="92" t="s">
         <v>2095</v>
       </c>
@@ -11906,8 +11926,8 @@
       <c r="C188" s="18" t="s">
         <v>637</v>
       </c>
-      <c r="E188" s="111"/>
-      <c r="F188" s="120"/>
+      <c r="E188" s="156"/>
+      <c r="F188" s="158"/>
       <c r="G188" s="92" t="s">
         <v>2095</v>
       </c>
@@ -11923,8 +11943,8 @@
         <v>637</v>
       </c>
       <c r="D189" s="45"/>
-      <c r="E189" s="112"/>
-      <c r="F189" s="121"/>
+      <c r="E189" s="125"/>
+      <c r="F189" s="159"/>
       <c r="G189" s="92" t="s">
         <v>2095</v>
       </c>
@@ -11939,11 +11959,11 @@
       <c r="C190" s="18" t="s">
         <v>638</v>
       </c>
-      <c r="D190" s="163" t="s">
+      <c r="D190" s="104" t="s">
         <v>1009</v>
       </c>
       <c r="E190" s="77"/>
-      <c r="F190" s="123" t="s">
+      <c r="F190" s="112" t="s">
         <v>738</v>
       </c>
       <c r="G190" s="24" t="s">
@@ -11960,9 +11980,9 @@
       <c r="C191" t="s">
         <v>638</v>
       </c>
-      <c r="D191" s="163"/>
+      <c r="D191" s="104"/>
       <c r="E191" s="77"/>
-      <c r="F191" s="123"/>
+      <c r="F191" s="112"/>
       <c r="G191" s="24" t="s">
         <v>611</v>
       </c>
@@ -11977,11 +11997,11 @@
       <c r="C192" s="18" t="s">
         <v>639</v>
       </c>
-      <c r="D192" s="163" t="s">
+      <c r="D192" s="104" t="s">
         <v>1010</v>
       </c>
       <c r="E192" s="77"/>
-      <c r="F192" s="123" t="s">
+      <c r="F192" s="112" t="s">
         <v>739</v>
       </c>
       <c r="G192" s="24" t="s">
@@ -11998,9 +12018,9 @@
       <c r="C193" t="s">
         <v>639</v>
       </c>
-      <c r="D193" s="163"/>
+      <c r="D193" s="104"/>
       <c r="E193" s="77"/>
-      <c r="F193" s="123"/>
+      <c r="F193" s="112"/>
       <c r="G193" s="24" t="s">
         <v>611</v>
       </c>
@@ -12015,13 +12035,13 @@
       <c r="C194" s="18" t="s">
         <v>640</v>
       </c>
-      <c r="D194" s="163" t="s">
+      <c r="D194" s="104" t="s">
         <v>606</v>
       </c>
-      <c r="E194" s="110" t="s">
+      <c r="E194" s="124" t="s">
         <v>695</v>
       </c>
-      <c r="F194" s="124" t="s">
+      <c r="F194" s="113" t="s">
         <v>740</v>
       </c>
       <c r="G194" s="78" t="s">
@@ -12038,9 +12058,9 @@
       <c r="C195" t="s">
         <v>640</v>
       </c>
-      <c r="D195" s="163"/>
-      <c r="E195" s="112"/>
-      <c r="F195" s="124"/>
+      <c r="D195" s="104"/>
+      <c r="E195" s="125"/>
+      <c r="F195" s="113"/>
       <c r="G195" s="78" t="s">
         <v>873</v>
       </c>
@@ -12055,11 +12075,11 @@
       <c r="C196" s="18" t="s">
         <v>877</v>
       </c>
-      <c r="D196" s="163" t="s">
+      <c r="D196" s="104" t="s">
         <v>1011</v>
       </c>
       <c r="E196" s="77"/>
-      <c r="F196" s="123" t="s">
+      <c r="F196" s="112" t="s">
         <v>741</v>
       </c>
       <c r="G196" s="24" t="s">
@@ -12076,9 +12096,9 @@
       <c r="C197" t="s">
         <v>877</v>
       </c>
-      <c r="D197" s="163"/>
+      <c r="D197" s="104"/>
       <c r="E197" s="77"/>
-      <c r="F197" s="123"/>
+      <c r="F197" s="112"/>
       <c r="G197" s="24" t="s">
         <v>611</v>
       </c>
@@ -12093,10 +12113,10 @@
       <c r="C198" s="18" t="s">
         <v>641</v>
       </c>
-      <c r="E198" s="110" t="s">
+      <c r="E198" s="124" t="s">
         <v>695</v>
       </c>
-      <c r="F198" s="124" t="s">
+      <c r="F198" s="113" t="s">
         <v>742</v>
       </c>
       <c r="G198" s="78" t="s">
@@ -12114,8 +12134,8 @@
         <v>641</v>
       </c>
       <c r="D199" s="45"/>
-      <c r="E199" s="112"/>
-      <c r="F199" s="124"/>
+      <c r="E199" s="125"/>
+      <c r="F199" s="113"/>
       <c r="G199" s="78" t="s">
         <v>873</v>
       </c>
@@ -12131,14 +12151,14 @@
         <v>642</v>
       </c>
       <c r="E200" s="77"/>
-      <c r="F200" s="123" t="s">
+      <c r="F200" s="112" t="s">
         <v>743</v>
       </c>
       <c r="G200" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H200" s="89" t="s">
-        <v>2139</v>
+        <v>2138</v>
       </c>
     </row>
     <row r="201" spans="1:8" x14ac:dyDescent="0.4">
@@ -12153,7 +12173,7 @@
       </c>
       <c r="D201" s="45"/>
       <c r="E201" s="77"/>
-      <c r="F201" s="123"/>
+      <c r="F201" s="112"/>
       <c r="G201" s="24" t="s">
         <v>611</v>
       </c>
@@ -12169,14 +12189,14 @@
         <v>643</v>
       </c>
       <c r="E202" s="77"/>
-      <c r="F202" s="123" t="s">
+      <c r="F202" s="112" t="s">
         <v>744</v>
       </c>
       <c r="G202" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H202" s="89" t="s">
-        <v>2138</v>
+        <v>2137</v>
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.4">
@@ -12191,7 +12211,7 @@
       </c>
       <c r="D203" s="45"/>
       <c r="E203" s="77"/>
-      <c r="F203" s="123"/>
+      <c r="F203" s="112"/>
       <c r="G203" s="24" t="s">
         <v>611</v>
       </c>
@@ -12207,7 +12227,7 @@
         <v>644</v>
       </c>
       <c r="E204" s="77"/>
-      <c r="F204" s="123" t="s">
+      <c r="F204" s="112" t="s">
         <v>745</v>
       </c>
       <c r="G204" s="24" t="s">
@@ -12226,7 +12246,7 @@
       </c>
       <c r="D205" s="45"/>
       <c r="E205" s="77"/>
-      <c r="F205" s="123"/>
+      <c r="F205" s="112"/>
       <c r="G205" s="24" t="s">
         <v>611</v>
       </c>
@@ -12241,11 +12261,11 @@
       <c r="C206" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="D206" s="163" t="s">
+      <c r="D206" s="104" t="s">
         <v>1012</v>
       </c>
       <c r="E206" s="77"/>
-      <c r="F206" s="123" t="s">
+      <c r="F206" s="112" t="s">
         <v>746</v>
       </c>
       <c r="G206" s="24" t="s">
@@ -12262,9 +12282,9 @@
       <c r="C207" t="s">
         <v>645</v>
       </c>
-      <c r="D207" s="163"/>
+      <c r="D207" s="104"/>
       <c r="E207" s="77"/>
-      <c r="F207" s="123"/>
+      <c r="F207" s="112"/>
       <c r="G207" s="24" t="s">
         <v>611</v>
       </c>
@@ -12280,14 +12300,14 @@
         <v>646</v>
       </c>
       <c r="E208" s="77"/>
-      <c r="F208" s="123" t="s">
+      <c r="F208" s="112" t="s">
         <v>891</v>
       </c>
       <c r="G208" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H208" s="89" t="s">
-        <v>2140</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="209" spans="1:8" x14ac:dyDescent="0.4">
@@ -12302,12 +12322,12 @@
       </c>
       <c r="D209" s="45"/>
       <c r="E209" s="77"/>
-      <c r="F209" s="123"/>
+      <c r="F209" s="112"/>
       <c r="G209" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H209" s="89" t="s">
-        <v>2141</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.4">
@@ -12321,14 +12341,14 @@
         <v>647</v>
       </c>
       <c r="E210" s="77"/>
-      <c r="F210" s="123" t="s">
+      <c r="F210" s="112" t="s">
         <v>892</v>
       </c>
       <c r="G210" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H210" s="89" t="s">
-        <v>2142</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.4">
@@ -12343,7 +12363,7 @@
       </c>
       <c r="D211" s="45"/>
       <c r="E211" s="77"/>
-      <c r="F211" s="123"/>
+      <c r="F211" s="112"/>
       <c r="G211" s="24" t="s">
         <v>611</v>
       </c>
@@ -12358,11 +12378,11 @@
       <c r="C212" s="18" t="s">
         <v>648</v>
       </c>
-      <c r="D212" s="163" t="s">
+      <c r="D212" s="104" t="s">
         <v>1013</v>
       </c>
       <c r="E212" s="77"/>
-      <c r="F212" s="123" t="s">
+      <c r="F212" s="112" t="s">
         <v>747</v>
       </c>
       <c r="G212" s="24" t="s">
@@ -12379,9 +12399,9 @@
       <c r="C213" t="s">
         <v>648</v>
       </c>
-      <c r="D213" s="163"/>
+      <c r="D213" s="104"/>
       <c r="E213" s="77"/>
-      <c r="F213" s="123"/>
+      <c r="F213" s="112"/>
       <c r="G213" s="24" t="s">
         <v>611</v>
       </c>
@@ -12405,13 +12425,13 @@
       <c r="C215" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="D215" s="163" t="s">
+      <c r="D215" s="104" t="s">
         <v>1015</v>
       </c>
       <c r="E215" s="77" t="s">
         <v>695</v>
       </c>
-      <c r="F215" s="132" t="s">
+      <c r="F215" s="154" t="s">
         <v>748</v>
       </c>
       <c r="G215" s="24" t="s">
@@ -12428,9 +12448,9 @@
       <c r="C216" t="s">
         <v>649</v>
       </c>
-      <c r="D216" s="163"/>
+      <c r="D216" s="104"/>
       <c r="E216" s="77"/>
-      <c r="F216" s="132"/>
+      <c r="F216" s="154"/>
       <c r="G216" s="24" t="s">
         <v>611</v>
       </c>
@@ -12445,9 +12465,9 @@
       <c r="C217" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="D217" s="163"/>
+      <c r="D217" s="104"/>
       <c r="E217" s="77"/>
-      <c r="F217" s="132"/>
+      <c r="F217" s="154"/>
       <c r="G217" s="24" t="s">
         <v>611</v>
       </c>
@@ -12462,9 +12482,9 @@
       <c r="C218" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="D218" s="163"/>
+      <c r="D218" s="104"/>
       <c r="E218" s="77"/>
-      <c r="F218" s="132"/>
+      <c r="F218" s="154"/>
       <c r="G218" s="24" t="s">
         <v>611</v>
       </c>
@@ -12479,10 +12499,10 @@
       <c r="C219" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="E219" s="110" t="s">
+      <c r="E219" s="124" t="s">
         <v>695</v>
       </c>
-      <c r="F219" s="133" t="s">
+      <c r="F219" s="155" t="s">
         <v>749</v>
       </c>
       <c r="G219" s="92" t="s">
@@ -12500,8 +12520,8 @@
         <v>650</v>
       </c>
       <c r="D220" s="45"/>
-      <c r="E220" s="111"/>
-      <c r="F220" s="133"/>
+      <c r="E220" s="156"/>
+      <c r="F220" s="155"/>
       <c r="G220" s="92" t="s">
         <v>2095</v>
       </c>
@@ -12516,8 +12536,8 @@
       <c r="C221" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="E221" s="111"/>
-      <c r="F221" s="133"/>
+      <c r="E221" s="156"/>
+      <c r="F221" s="155"/>
       <c r="G221" s="92" t="s">
         <v>2095</v>
       </c>
@@ -12532,8 +12552,8 @@
       <c r="C222" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="E222" s="112"/>
-      <c r="F222" s="133"/>
+      <c r="E222" s="125"/>
+      <c r="F222" s="155"/>
       <c r="G222" s="92" t="s">
         <v>2095</v>
       </c>
@@ -12549,14 +12569,14 @@
         <v>651</v>
       </c>
       <c r="E223" s="77"/>
-      <c r="F223" s="132" t="s">
+      <c r="F223" s="154" t="s">
         <v>750</v>
       </c>
       <c r="G223" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H223" s="89" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
     </row>
     <row r="224" spans="1:8" x14ac:dyDescent="0.4">
@@ -12571,12 +12591,12 @@
       </c>
       <c r="D224" s="45"/>
       <c r="E224" s="77"/>
-      <c r="F224" s="132"/>
+      <c r="F224" s="154"/>
       <c r="G224" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H224" s="89" t="s">
-        <v>2144</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="225" spans="1:8" x14ac:dyDescent="0.4">
@@ -12590,7 +12610,7 @@
         <v>651</v>
       </c>
       <c r="E225" s="77"/>
-      <c r="F225" s="132"/>
+      <c r="F225" s="154"/>
       <c r="G225" s="24" t="s">
         <v>611</v>
       </c>
@@ -12606,7 +12626,7 @@
         <v>651</v>
       </c>
       <c r="E226" s="77"/>
-      <c r="F226" s="132"/>
+      <c r="F226" s="154"/>
       <c r="G226" s="24" t="s">
         <v>611</v>
       </c>
@@ -12621,10 +12641,10 @@
       <c r="C227" s="18" t="s">
         <v>652</v>
       </c>
-      <c r="E227" s="110" t="s">
+      <c r="E227" s="124" t="s">
         <v>695</v>
       </c>
-      <c r="F227" s="124" t="s">
+      <c r="F227" s="113" t="s">
         <v>751</v>
       </c>
       <c r="G227" s="78" t="s">
@@ -12642,8 +12662,8 @@
         <v>652</v>
       </c>
       <c r="D228" s="45"/>
-      <c r="E228" s="112"/>
-      <c r="F228" s="124"/>
+      <c r="E228" s="125"/>
+      <c r="F228" s="113"/>
       <c r="G228" s="78" t="s">
         <v>2095</v>
       </c>
@@ -12659,14 +12679,14 @@
         <v>653</v>
       </c>
       <c r="E229" s="77"/>
-      <c r="F229" s="123" t="s">
+      <c r="F229" s="112" t="s">
         <v>752</v>
       </c>
       <c r="G229" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H229" s="89" t="s">
-        <v>2145</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="230" spans="1:8" x14ac:dyDescent="0.4">
@@ -12681,7 +12701,7 @@
       </c>
       <c r="D230" s="45"/>
       <c r="E230" s="77"/>
-      <c r="F230" s="123"/>
+      <c r="F230" s="112"/>
       <c r="G230" s="24" t="s">
         <v>611</v>
       </c>
@@ -12699,17 +12719,17 @@
       <c r="D231" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E231" s="110" t="s">
+      <c r="E231" s="124" t="s">
         <v>695</v>
       </c>
-      <c r="F231" s="124" t="s">
+      <c r="F231" s="113" t="s">
         <v>753</v>
       </c>
       <c r="G231" s="78" t="s">
         <v>873</v>
       </c>
       <c r="H231" s="89" t="s">
-        <v>2146</v>
+        <v>2145</v>
       </c>
     </row>
     <row r="232" spans="1:8" x14ac:dyDescent="0.4">
@@ -12723,8 +12743,8 @@
         <v>654</v>
       </c>
       <c r="D232" s="45"/>
-      <c r="E232" s="112"/>
-      <c r="F232" s="124"/>
+      <c r="E232" s="125"/>
+      <c r="F232" s="113"/>
       <c r="G232" s="78" t="s">
         <v>873</v>
       </c>
@@ -12743,7 +12763,7 @@
         <v>625</v>
       </c>
       <c r="E233" s="93"/>
-      <c r="F233" s="124" t="s">
+      <c r="F233" s="113" t="s">
         <v>754</v>
       </c>
       <c r="G233" s="78" t="s">
@@ -12762,7 +12782,7 @@
       </c>
       <c r="D234" s="45"/>
       <c r="E234" s="93"/>
-      <c r="F234" s="124"/>
+      <c r="F234" s="113"/>
       <c r="G234" s="78" t="s">
         <v>873</v>
       </c>
@@ -12781,7 +12801,7 @@
         <v>625</v>
       </c>
       <c r="E235" s="93"/>
-      <c r="F235" s="124" t="s">
+      <c r="F235" s="113" t="s">
         <v>755</v>
       </c>
       <c r="G235" s="78" t="s">
@@ -12800,7 +12820,7 @@
       </c>
       <c r="D236" s="45"/>
       <c r="E236" s="93"/>
-      <c r="F236" s="124"/>
+      <c r="F236" s="113"/>
       <c r="G236" s="78" t="s">
         <v>873</v>
       </c>
@@ -12819,7 +12839,7 @@
         <v>625</v>
       </c>
       <c r="E237" s="93"/>
-      <c r="F237" s="124" t="s">
+      <c r="F237" s="113" t="s">
         <v>756</v>
       </c>
       <c r="G237" s="78" t="s">
@@ -12838,7 +12858,7 @@
       </c>
       <c r="D238" s="45"/>
       <c r="E238" s="93"/>
-      <c r="F238" s="124"/>
+      <c r="F238" s="113"/>
       <c r="G238" s="78" t="s">
         <v>873</v>
       </c>
@@ -12857,7 +12877,7 @@
         <v>625</v>
       </c>
       <c r="E239" s="93"/>
-      <c r="F239" s="124" t="s">
+      <c r="F239" s="113" t="s">
         <v>757</v>
       </c>
       <c r="G239" s="78" t="s">
@@ -12876,7 +12896,7 @@
       </c>
       <c r="D240" s="45"/>
       <c r="E240" s="93"/>
-      <c r="F240" s="124"/>
+      <c r="F240" s="113"/>
       <c r="G240" s="78" t="s">
         <v>873</v>
       </c>
@@ -12895,7 +12915,7 @@
         <v>625</v>
       </c>
       <c r="E241" s="93"/>
-      <c r="F241" s="124" t="s">
+      <c r="F241" s="113" t="s">
         <v>758</v>
       </c>
       <c r="G241" s="78" t="s">
@@ -12914,7 +12934,7 @@
       </c>
       <c r="D242" s="45"/>
       <c r="E242" s="93"/>
-      <c r="F242" s="124"/>
+      <c r="F242" s="113"/>
       <c r="G242" s="78" t="s">
         <v>873</v>
       </c>
@@ -12933,7 +12953,7 @@
         <v>625</v>
       </c>
       <c r="E243" s="93"/>
-      <c r="F243" s="124" t="s">
+      <c r="F243" s="113" t="s">
         <v>759</v>
       </c>
       <c r="G243" s="78" t="s">
@@ -12952,7 +12972,7 @@
       </c>
       <c r="D244" s="45"/>
       <c r="E244" s="93"/>
-      <c r="F244" s="124"/>
+      <c r="F244" s="113"/>
       <c r="G244" s="78" t="s">
         <v>873</v>
       </c>
@@ -12971,7 +12991,7 @@
         <v>625</v>
       </c>
       <c r="E245" s="93"/>
-      <c r="F245" s="124" t="s">
+      <c r="F245" s="113" t="s">
         <v>760</v>
       </c>
       <c r="G245" s="78" t="s">
@@ -12990,7 +13010,7 @@
       </c>
       <c r="D246" s="45"/>
       <c r="E246" s="93"/>
-      <c r="F246" s="124"/>
+      <c r="F246" s="113"/>
       <c r="G246" s="78" t="s">
         <v>873</v>
       </c>
@@ -13009,7 +13029,7 @@
         <v>625</v>
       </c>
       <c r="E247" s="93"/>
-      <c r="F247" s="124" t="s">
+      <c r="F247" s="113" t="s">
         <v>761</v>
       </c>
       <c r="G247" s="78" t="s">
@@ -13028,7 +13048,7 @@
       </c>
       <c r="D248" s="45"/>
       <c r="E248" s="93"/>
-      <c r="F248" s="124"/>
+      <c r="F248" s="113"/>
       <c r="G248" s="78" t="s">
         <v>873</v>
       </c>
@@ -13047,7 +13067,7 @@
         <v>625</v>
       </c>
       <c r="E249" s="93"/>
-      <c r="F249" s="124" t="s">
+      <c r="F249" s="113" t="s">
         <v>2072</v>
       </c>
       <c r="G249" s="78" t="s">
@@ -13066,7 +13086,7 @@
       </c>
       <c r="D250" s="45"/>
       <c r="E250" s="93"/>
-      <c r="F250" s="124"/>
+      <c r="F250" s="113"/>
       <c r="G250" s="78" t="s">
         <v>873</v>
       </c>
@@ -13085,7 +13105,7 @@
         <v>625</v>
       </c>
       <c r="E251" s="93"/>
-      <c r="F251" s="124" t="s">
+      <c r="F251" s="113" t="s">
         <v>762</v>
       </c>
       <c r="G251" s="78" t="s">
@@ -13104,7 +13124,7 @@
       </c>
       <c r="D252" s="45"/>
       <c r="E252" s="93"/>
-      <c r="F252" s="124"/>
+      <c r="F252" s="113"/>
       <c r="G252" s="78" t="s">
         <v>873</v>
       </c>
@@ -13120,7 +13140,7 @@
         <v>665</v>
       </c>
       <c r="E253" s="93"/>
-      <c r="F253" s="124" t="s">
+      <c r="F253" s="113" t="s">
         <v>763</v>
       </c>
       <c r="G253" s="78" t="s">
@@ -13139,7 +13159,7 @@
       </c>
       <c r="D254" s="45"/>
       <c r="E254" s="93"/>
-      <c r="F254" s="124"/>
+      <c r="F254" s="113"/>
       <c r="G254" s="78" t="s">
         <v>873</v>
       </c>
@@ -13175,7 +13195,7 @@
         <v>633</v>
       </c>
       <c r="D258" s="32" t="s">
-        <v>2147</v>
+        <v>2146</v>
       </c>
       <c r="E258" s="76" t="s">
         <v>694</v>
@@ -13187,7 +13207,7 @@
         <v>611</v>
       </c>
       <c r="H258" s="89" t="s">
-        <v>2148</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="259" spans="1:8" x14ac:dyDescent="0.4">
@@ -13218,11 +13238,11 @@
       <c r="C260" s="18" t="s">
         <v>573</v>
       </c>
-      <c r="E260" s="106" t="s">
+      <c r="E260" s="114" t="s">
         <v>620</v>
       </c>
-      <c r="F260" s="107"/>
-      <c r="G260" s="155" t="s">
+      <c r="F260" s="115"/>
+      <c r="G260" s="105" t="s">
         <v>611</v>
       </c>
     </row>
@@ -13236,9 +13256,9 @@
       <c r="C261" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E261" s="106"/>
-      <c r="F261" s="107"/>
-      <c r="G261" s="156"/>
+      <c r="E261" s="114"/>
+      <c r="F261" s="115"/>
+      <c r="G261" s="106"/>
     </row>
     <row r="262" spans="1:8" x14ac:dyDescent="0.4">
       <c r="C262" s="23"/>
@@ -13345,7 +13365,7 @@
         <v>611</v>
       </c>
       <c r="H267" s="89" t="s">
-        <v>2150</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="268" spans="1:8" x14ac:dyDescent="0.4">
@@ -13358,10 +13378,10 @@
       <c r="C268" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E268" s="105" t="s">
+      <c r="E268" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F268" s="105"/>
+      <c r="F268" s="107"/>
       <c r="G268" s="26" t="s">
         <v>611</v>
       </c>
@@ -13448,7 +13468,7 @@
         <v>611</v>
       </c>
       <c r="H274" s="89" t="s">
-        <v>2151</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="275" spans="1:8" x14ac:dyDescent="0.4">
@@ -13462,7 +13482,7 @@
         <v>879</v>
       </c>
       <c r="D275" s="98" t="s">
-        <v>2152</v>
+        <v>2151</v>
       </c>
       <c r="E275" s="93"/>
       <c r="F275" s="100" t="s">
@@ -13484,7 +13504,7 @@
         <v>880</v>
       </c>
       <c r="D276" s="45" t="s">
-        <v>2153</v>
+        <v>2152</v>
       </c>
       <c r="E276" s="93"/>
       <c r="F276" s="100" t="s">
@@ -13534,7 +13554,7 @@
         <v>611</v>
       </c>
       <c r="H278" s="89" t="s">
-        <v>2154</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="279" spans="1:8" x14ac:dyDescent="0.4">
@@ -13548,11 +13568,11 @@
         <v>573</v>
       </c>
       <c r="D279" s="45"/>
-      <c r="E279" s="105" t="s">
+      <c r="E279" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F279" s="105"/>
-      <c r="G279" s="104" t="s">
+      <c r="F279" s="107"/>
+      <c r="G279" s="108" t="s">
         <v>611</v>
       </c>
     </row>
@@ -13567,19 +13587,19 @@
         <v>601</v>
       </c>
       <c r="D280" s="45"/>
-      <c r="E280" s="105"/>
-      <c r="F280" s="105"/>
-      <c r="G280" s="104"/>
+      <c r="E280" s="107"/>
+      <c r="F280" s="107"/>
+      <c r="G280" s="108"/>
     </row>
     <row r="282" spans="1:8" x14ac:dyDescent="0.4">
       <c r="C282" s="23"/>
     </row>
     <row r="283" spans="1:8" x14ac:dyDescent="0.4">
       <c r="C283" s="23"/>
-      <c r="E283" s="122" t="s">
+      <c r="E283" s="111" t="s">
         <v>906</v>
       </c>
-      <c r="F283" s="122"/>
+      <c r="F283" s="111"/>
       <c r="G283" s="28" t="s">
         <v>613</v>
       </c>
@@ -13620,14 +13640,14 @@
       <c r="E285" s="93" t="s">
         <v>695</v>
       </c>
-      <c r="F285" s="124" t="s">
+      <c r="F285" s="113" t="s">
         <v>792</v>
       </c>
       <c r="G285" s="78" t="s">
         <v>611</v>
       </c>
       <c r="H285" s="89" t="s">
-        <v>2155</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="286" spans="1:8" x14ac:dyDescent="0.4">
@@ -13641,7 +13661,7 @@
         <v>669</v>
       </c>
       <c r="E286" s="93"/>
-      <c r="F286" s="124"/>
+      <c r="F286" s="113"/>
       <c r="G286" s="78" t="s">
         <v>611</v>
       </c>
@@ -13660,7 +13680,7 @@
         <v>621</v>
       </c>
       <c r="E287" s="93"/>
-      <c r="F287" s="124" t="s">
+      <c r="F287" s="113" t="s">
         <v>769</v>
       </c>
       <c r="G287" s="78" t="s">
@@ -13678,7 +13698,7 @@
         <v>670</v>
       </c>
       <c r="E288" s="93"/>
-      <c r="F288" s="124"/>
+      <c r="F288" s="113"/>
       <c r="G288" s="78" t="s">
         <v>611</v>
       </c>
@@ -13697,7 +13717,7 @@
         <v>621</v>
       </c>
       <c r="E289" s="93"/>
-      <c r="F289" s="124" t="s">
+      <c r="F289" s="113" t="s">
         <v>770</v>
       </c>
       <c r="G289" s="78" t="s">
@@ -13715,7 +13735,7 @@
         <v>671</v>
       </c>
       <c r="E290" s="93"/>
-      <c r="F290" s="124"/>
+      <c r="F290" s="113"/>
       <c r="G290" s="78" t="s">
         <v>611</v>
       </c>
@@ -13734,7 +13754,7 @@
         <v>622</v>
       </c>
       <c r="E291" s="93"/>
-      <c r="F291" s="124" t="s">
+      <c r="F291" s="113" t="s">
         <v>771</v>
       </c>
       <c r="G291" s="78" t="s">
@@ -13752,7 +13772,7 @@
         <v>672</v>
       </c>
       <c r="E292" s="93"/>
-      <c r="F292" s="124"/>
+      <c r="F292" s="113"/>
       <c r="G292" s="78" t="s">
         <v>614</v>
       </c>
@@ -13771,7 +13791,7 @@
         <v>622</v>
       </c>
       <c r="E293" s="93"/>
-      <c r="F293" s="124" t="s">
+      <c r="F293" s="113" t="s">
         <v>772</v>
       </c>
       <c r="G293" s="78" t="s">
@@ -13789,7 +13809,7 @@
         <v>673</v>
       </c>
       <c r="E294" s="93"/>
-      <c r="F294" s="124"/>
+      <c r="F294" s="113"/>
       <c r="G294" s="78" t="s">
         <v>614</v>
       </c>
@@ -13808,7 +13828,7 @@
         <v>621</v>
       </c>
       <c r="E295" s="93"/>
-      <c r="F295" s="124" t="s">
+      <c r="F295" s="113" t="s">
         <v>773</v>
       </c>
       <c r="G295" s="78" t="s">
@@ -13826,7 +13846,7 @@
         <v>674</v>
       </c>
       <c r="E296" s="93"/>
-      <c r="F296" s="124"/>
+      <c r="F296" s="113"/>
       <c r="G296" s="78" t="s">
         <v>611</v>
       </c>
@@ -13845,7 +13865,7 @@
         <v>621</v>
       </c>
       <c r="E297" s="93"/>
-      <c r="F297" s="124" t="s">
+      <c r="F297" s="113" t="s">
         <v>774</v>
       </c>
       <c r="G297" s="78" t="s">
@@ -13863,7 +13883,7 @@
         <v>675</v>
       </c>
       <c r="E298" s="93"/>
-      <c r="F298" s="124"/>
+      <c r="F298" s="113"/>
       <c r="G298" s="78" t="s">
         <v>611</v>
       </c>
@@ -13882,7 +13902,7 @@
         <v>621</v>
       </c>
       <c r="E299" s="93"/>
-      <c r="F299" s="124" t="s">
+      <c r="F299" s="113" t="s">
         <v>775</v>
       </c>
       <c r="G299" s="78" t="s">
@@ -13900,7 +13920,7 @@
         <v>676</v>
       </c>
       <c r="E300" s="93"/>
-      <c r="F300" s="124"/>
+      <c r="F300" s="113"/>
       <c r="G300" s="78" t="s">
         <v>611</v>
       </c>
@@ -13919,7 +13939,7 @@
         <v>623</v>
       </c>
       <c r="E301" s="93"/>
-      <c r="F301" s="124" t="s">
+      <c r="F301" s="113" t="s">
         <v>776</v>
       </c>
       <c r="G301" s="78" t="s">
@@ -13937,7 +13957,7 @@
         <v>677</v>
       </c>
       <c r="E302" s="93"/>
-      <c r="F302" s="124"/>
+      <c r="F302" s="113"/>
       <c r="G302" s="78" t="s">
         <v>611</v>
       </c>
@@ -13953,14 +13973,14 @@
         <v>678</v>
       </c>
       <c r="E303" s="77"/>
-      <c r="F303" s="123" t="s">
+      <c r="F303" s="112" t="s">
         <v>777</v>
       </c>
       <c r="G303" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H303" s="89" t="s">
-        <v>2156</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="304" spans="1:8" x14ac:dyDescent="0.4">
@@ -13974,7 +13994,7 @@
         <v>678</v>
       </c>
       <c r="E304" s="77"/>
-      <c r="F304" s="123"/>
+      <c r="F304" s="112"/>
       <c r="G304" s="24" t="s">
         <v>611</v>
       </c>
@@ -13990,7 +14010,7 @@
         <v>679</v>
       </c>
       <c r="E305" s="93"/>
-      <c r="F305" s="124" t="s">
+      <c r="F305" s="113" t="s">
         <v>778</v>
       </c>
       <c r="G305" s="78" t="s">
@@ -14008,7 +14028,7 @@
         <v>679</v>
       </c>
       <c r="E306" s="93"/>
-      <c r="F306" s="124"/>
+      <c r="F306" s="113"/>
       <c r="G306" s="78" t="s">
         <v>611</v>
       </c>
@@ -14024,14 +14044,14 @@
         <v>680</v>
       </c>
       <c r="E307" s="93"/>
-      <c r="F307" s="124" t="s">
+      <c r="F307" s="113" t="s">
         <v>779</v>
       </c>
       <c r="G307" s="92" t="s">
         <v>618</v>
       </c>
       <c r="H307" s="89" t="s">
-        <v>2157</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="308" spans="1:8" x14ac:dyDescent="0.4">
@@ -14045,7 +14065,7 @@
         <v>680</v>
       </c>
       <c r="E308" s="93"/>
-      <c r="F308" s="124"/>
+      <c r="F308" s="113"/>
       <c r="G308" s="92" t="s">
         <v>618</v>
       </c>
@@ -14061,7 +14081,7 @@
         <v>682</v>
       </c>
       <c r="E309" s="93"/>
-      <c r="F309" s="124" t="s">
+      <c r="F309" s="113" t="s">
         <v>780</v>
       </c>
       <c r="G309" s="78" t="s">
@@ -14079,7 +14099,7 @@
         <v>682</v>
       </c>
       <c r="E310" s="93"/>
-      <c r="F310" s="124"/>
+      <c r="F310" s="113"/>
       <c r="G310" s="78" t="s">
         <v>611</v>
       </c>
@@ -14095,7 +14115,7 @@
         <v>683</v>
       </c>
       <c r="E311" s="93"/>
-      <c r="F311" s="124" t="s">
+      <c r="F311" s="113" t="s">
         <v>781</v>
       </c>
       <c r="G311" s="78" t="s">
@@ -14113,7 +14133,7 @@
         <v>683</v>
       </c>
       <c r="E312" s="93"/>
-      <c r="F312" s="124"/>
+      <c r="F312" s="113"/>
       <c r="G312" s="78" t="s">
         <v>2095</v>
       </c>
@@ -14129,14 +14149,14 @@
         <v>684</v>
       </c>
       <c r="E313" s="77"/>
-      <c r="F313" s="123" t="s">
+      <c r="F313" s="112" t="s">
         <v>782</v>
       </c>
       <c r="G313" s="24" t="s">
         <v>611</v>
       </c>
       <c r="H313" s="89" t="s">
-        <v>2159</v>
+        <v>2158</v>
       </c>
     </row>
     <row r="314" spans="1:8" x14ac:dyDescent="0.4">
@@ -14150,7 +14170,7 @@
         <v>684</v>
       </c>
       <c r="E314" s="77"/>
-      <c r="F314" s="123"/>
+      <c r="F314" s="112"/>
       <c r="G314" s="24" t="s">
         <v>611</v>
       </c>
@@ -14166,7 +14186,7 @@
         <v>685</v>
       </c>
       <c r="E315" s="93"/>
-      <c r="F315" s="124" t="s">
+      <c r="F315" s="113" t="s">
         <v>783</v>
       </c>
       <c r="G315" s="78" t="s">
@@ -14184,7 +14204,7 @@
         <v>685</v>
       </c>
       <c r="E316" s="93"/>
-      <c r="F316" s="124"/>
+      <c r="F316" s="113"/>
       <c r="G316" s="78" t="s">
         <v>873</v>
       </c>
@@ -14200,7 +14220,7 @@
         <v>686</v>
       </c>
       <c r="E317" s="93"/>
-      <c r="F317" s="124" t="s">
+      <c r="F317" s="113" t="s">
         <v>784</v>
       </c>
       <c r="G317" s="78" t="s">
@@ -14218,7 +14238,7 @@
         <v>686</v>
       </c>
       <c r="E318" s="93"/>
-      <c r="F318" s="124"/>
+      <c r="F318" s="113"/>
       <c r="G318" s="78" t="s">
         <v>873</v>
       </c>
@@ -14234,7 +14254,7 @@
         <v>687</v>
       </c>
       <c r="E319" s="93"/>
-      <c r="F319" s="124" t="s">
+      <c r="F319" s="113" t="s">
         <v>785</v>
       </c>
       <c r="G319" s="78" t="s">
@@ -14252,7 +14272,7 @@
         <v>687</v>
       </c>
       <c r="E320" s="93"/>
-      <c r="F320" s="124"/>
+      <c r="F320" s="113"/>
       <c r="G320" s="78" t="s">
         <v>873</v>
       </c>
@@ -14268,7 +14288,7 @@
         <v>688</v>
       </c>
       <c r="E321" s="93"/>
-      <c r="F321" s="124" t="s">
+      <c r="F321" s="155" t="s">
         <v>786</v>
       </c>
       <c r="G321" s="78" t="s">
@@ -14286,7 +14306,7 @@
         <v>688</v>
       </c>
       <c r="E322" s="93"/>
-      <c r="F322" s="124"/>
+      <c r="F322" s="113"/>
       <c r="G322" s="78" t="s">
         <v>611</v>
       </c>
@@ -14386,11 +14406,11 @@
       <c r="C329" s="18" t="s">
         <v>573</v>
       </c>
-      <c r="E329" s="126" t="s">
+      <c r="E329" s="148" t="s">
         <v>620</v>
       </c>
-      <c r="F329" s="127"/>
-      <c r="G329" s="130" t="s">
+      <c r="F329" s="149"/>
+      <c r="G329" s="152" t="s">
         <v>611</v>
       </c>
     </row>
@@ -14404,9 +14424,9 @@
       <c r="C330" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E330" s="128"/>
-      <c r="F330" s="129"/>
-      <c r="G330" s="131"/>
+      <c r="E330" s="150"/>
+      <c r="F330" s="151"/>
+      <c r="G330" s="153"/>
     </row>
     <row r="333" spans="1:7" ht="24.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A333" s="38" t="s">
@@ -14462,7 +14482,7 @@
         <v>893</v>
       </c>
       <c r="D335" s="32" t="s">
-        <v>2158</v>
+        <v>2157</v>
       </c>
       <c r="E335" s="102"/>
       <c r="F335" s="92" t="s">
@@ -14503,11 +14523,11 @@
       <c r="C337" s="18" t="s">
         <v>573</v>
       </c>
-      <c r="E337" s="126" t="s">
+      <c r="E337" s="148" t="s">
         <v>620</v>
       </c>
-      <c r="F337" s="127"/>
-      <c r="G337" s="130" t="s">
+      <c r="F337" s="149"/>
+      <c r="G337" s="152" t="s">
         <v>611</v>
       </c>
     </row>
@@ -14521,41 +14541,152 @@
       <c r="C338" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E338" s="128"/>
-      <c r="F338" s="129"/>
-      <c r="G338" s="131"/>
+      <c r="E338" s="150"/>
+      <c r="F338" s="151"/>
+      <c r="G338" s="153"/>
     </row>
   </sheetData>
   <mergeCells count="193">
-    <mergeCell ref="D212:D213"/>
-    <mergeCell ref="D215:D218"/>
-    <mergeCell ref="D173:D174"/>
-    <mergeCell ref="D175:D176"/>
-    <mergeCell ref="D179:D180"/>
-    <mergeCell ref="D184:D185"/>
-    <mergeCell ref="D190:D191"/>
-    <mergeCell ref="D192:D193"/>
-    <mergeCell ref="D194:D195"/>
-    <mergeCell ref="D196:D197"/>
-    <mergeCell ref="D206:D207"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="D39:D40"/>
-    <mergeCell ref="D41:D42"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="D45:D46"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="D51:D52"/>
-    <mergeCell ref="D53:D54"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="F309:F310"/>
+    <mergeCell ref="F311:F312"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="E84:F84"/>
+    <mergeCell ref="E108:F109"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="E115:E118"/>
+    <mergeCell ref="E141:E142"/>
+    <mergeCell ref="E151:E155"/>
+    <mergeCell ref="E156:E160"/>
+    <mergeCell ref="E171:E172"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="E86:E88"/>
+    <mergeCell ref="E89:E90"/>
+    <mergeCell ref="E91:E93"/>
+    <mergeCell ref="E99:E100"/>
+    <mergeCell ref="E94:E96"/>
+    <mergeCell ref="E78:E79"/>
+    <mergeCell ref="E169:E170"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="F184:F185"/>
+    <mergeCell ref="F190:F191"/>
+    <mergeCell ref="F192:F193"/>
+    <mergeCell ref="E194:E195"/>
+    <mergeCell ref="E111:F111"/>
+    <mergeCell ref="E120:F121"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="E181:E182"/>
+    <mergeCell ref="F307:F308"/>
+    <mergeCell ref="F186:F189"/>
+    <mergeCell ref="E283:F283"/>
+    <mergeCell ref="F194:F195"/>
+    <mergeCell ref="F196:F197"/>
+    <mergeCell ref="F198:F199"/>
+    <mergeCell ref="F200:F201"/>
+    <mergeCell ref="F202:F203"/>
+    <mergeCell ref="F317:F318"/>
+    <mergeCell ref="F319:F320"/>
+    <mergeCell ref="F237:F238"/>
+    <mergeCell ref="F239:F240"/>
+    <mergeCell ref="F204:F205"/>
+    <mergeCell ref="F206:F207"/>
+    <mergeCell ref="F208:F209"/>
+    <mergeCell ref="F210:F211"/>
+    <mergeCell ref="F212:F213"/>
+    <mergeCell ref="E260:F261"/>
+    <mergeCell ref="E219:E222"/>
+    <mergeCell ref="E227:E228"/>
+    <mergeCell ref="E231:E232"/>
+    <mergeCell ref="F289:F290"/>
+    <mergeCell ref="F291:F292"/>
+    <mergeCell ref="F293:F294"/>
+    <mergeCell ref="F295:F296"/>
+    <mergeCell ref="F297:F298"/>
+    <mergeCell ref="F299:F300"/>
+    <mergeCell ref="F301:F302"/>
+    <mergeCell ref="F303:F304"/>
+    <mergeCell ref="F305:F306"/>
+    <mergeCell ref="F313:F314"/>
+    <mergeCell ref="F315:F316"/>
+    <mergeCell ref="G108:G109"/>
+    <mergeCell ref="E329:F330"/>
+    <mergeCell ref="G329:G330"/>
+    <mergeCell ref="E337:F338"/>
+    <mergeCell ref="G337:G338"/>
+    <mergeCell ref="G279:G280"/>
+    <mergeCell ref="F251:F252"/>
+    <mergeCell ref="F253:F254"/>
+    <mergeCell ref="E279:F280"/>
+    <mergeCell ref="F215:F218"/>
+    <mergeCell ref="F219:F222"/>
+    <mergeCell ref="F223:F226"/>
+    <mergeCell ref="F227:F228"/>
+    <mergeCell ref="F229:F230"/>
+    <mergeCell ref="F241:F242"/>
+    <mergeCell ref="F243:F244"/>
+    <mergeCell ref="F245:F246"/>
+    <mergeCell ref="F247:F248"/>
+    <mergeCell ref="F249:F250"/>
+    <mergeCell ref="F231:F232"/>
+    <mergeCell ref="F233:F234"/>
+    <mergeCell ref="F321:F322"/>
+    <mergeCell ref="F285:F286"/>
+    <mergeCell ref="F287:F288"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="G41:G42"/>
+    <mergeCell ref="G43:G44"/>
+    <mergeCell ref="G45:G46"/>
+    <mergeCell ref="G47:G48"/>
+    <mergeCell ref="G49:G50"/>
+    <mergeCell ref="G51:G52"/>
+    <mergeCell ref="G53:G54"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="E37:E54"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="E9:E28"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E4:E7"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="G34:G35"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
     <mergeCell ref="G260:G261"/>
     <mergeCell ref="E268:F268"/>
     <mergeCell ref="G81:G82"/>
@@ -14580,186 +14711,75 @@
     <mergeCell ref="E133:E134"/>
     <mergeCell ref="E198:E199"/>
     <mergeCell ref="G120:G121"/>
-    <mergeCell ref="E4:E7"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="F34:F35"/>
-    <mergeCell ref="G34:G35"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F51:F52"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="E37:E54"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="E9:E28"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="G37:G38"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="G41:G42"/>
-    <mergeCell ref="G43:G44"/>
-    <mergeCell ref="G45:G46"/>
-    <mergeCell ref="G47:G48"/>
-    <mergeCell ref="G49:G50"/>
-    <mergeCell ref="G51:G52"/>
-    <mergeCell ref="G53:G54"/>
-    <mergeCell ref="G108:G109"/>
-    <mergeCell ref="E329:F330"/>
-    <mergeCell ref="G329:G330"/>
-    <mergeCell ref="E337:F338"/>
-    <mergeCell ref="G337:G338"/>
-    <mergeCell ref="G279:G280"/>
-    <mergeCell ref="F251:F252"/>
-    <mergeCell ref="F253:F254"/>
-    <mergeCell ref="E279:F280"/>
-    <mergeCell ref="F215:F218"/>
-    <mergeCell ref="F219:F222"/>
-    <mergeCell ref="F223:F226"/>
-    <mergeCell ref="F227:F228"/>
-    <mergeCell ref="F229:F230"/>
-    <mergeCell ref="F241:F242"/>
-    <mergeCell ref="F243:F244"/>
-    <mergeCell ref="F245:F246"/>
-    <mergeCell ref="F247:F248"/>
-    <mergeCell ref="F249:F250"/>
-    <mergeCell ref="F231:F232"/>
-    <mergeCell ref="F233:F234"/>
-    <mergeCell ref="F321:F322"/>
-    <mergeCell ref="F285:F286"/>
-    <mergeCell ref="F287:F288"/>
-    <mergeCell ref="F317:F318"/>
-    <mergeCell ref="F319:F320"/>
-    <mergeCell ref="F237:F238"/>
-    <mergeCell ref="F239:F240"/>
-    <mergeCell ref="F204:F205"/>
-    <mergeCell ref="F206:F207"/>
-    <mergeCell ref="F208:F209"/>
-    <mergeCell ref="F210:F211"/>
-    <mergeCell ref="F212:F213"/>
-    <mergeCell ref="E260:F261"/>
-    <mergeCell ref="E219:E222"/>
-    <mergeCell ref="E227:E228"/>
-    <mergeCell ref="E231:E232"/>
-    <mergeCell ref="F289:F290"/>
-    <mergeCell ref="F291:F292"/>
-    <mergeCell ref="F293:F294"/>
-    <mergeCell ref="F295:F296"/>
-    <mergeCell ref="F297:F298"/>
-    <mergeCell ref="F299:F300"/>
-    <mergeCell ref="F301:F302"/>
-    <mergeCell ref="F303:F304"/>
-    <mergeCell ref="F305:F306"/>
-    <mergeCell ref="F184:F185"/>
-    <mergeCell ref="F190:F191"/>
-    <mergeCell ref="F192:F193"/>
-    <mergeCell ref="E194:E195"/>
-    <mergeCell ref="E111:F111"/>
-    <mergeCell ref="E120:F121"/>
-    <mergeCell ref="E186:E189"/>
-    <mergeCell ref="E181:E182"/>
-    <mergeCell ref="F307:F308"/>
-    <mergeCell ref="F186:F189"/>
-    <mergeCell ref="E283:F283"/>
-    <mergeCell ref="F313:F314"/>
-    <mergeCell ref="F315:F316"/>
-    <mergeCell ref="F194:F195"/>
-    <mergeCell ref="F196:F197"/>
-    <mergeCell ref="F198:F199"/>
-    <mergeCell ref="F200:F201"/>
-    <mergeCell ref="F202:F203"/>
-    <mergeCell ref="F309:F310"/>
-    <mergeCell ref="F311:F312"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="E84:F84"/>
-    <mergeCell ref="E108:F109"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="E115:E118"/>
-    <mergeCell ref="E141:E142"/>
-    <mergeCell ref="E151:E155"/>
-    <mergeCell ref="E156:E160"/>
-    <mergeCell ref="E171:E172"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="E86:E88"/>
-    <mergeCell ref="E89:E90"/>
-    <mergeCell ref="E91:E93"/>
-    <mergeCell ref="E99:E100"/>
-    <mergeCell ref="E94:E96"/>
-    <mergeCell ref="E78:E79"/>
-    <mergeCell ref="E169:E170"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="D45:D46"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="D51:D52"/>
+    <mergeCell ref="D53:D54"/>
+    <mergeCell ref="D212:D213"/>
+    <mergeCell ref="D215:D218"/>
+    <mergeCell ref="D173:D174"/>
+    <mergeCell ref="D175:D176"/>
+    <mergeCell ref="D179:D180"/>
+    <mergeCell ref="D184:D185"/>
+    <mergeCell ref="D190:D191"/>
+    <mergeCell ref="D192:D193"/>
+    <mergeCell ref="D194:D195"/>
+    <mergeCell ref="D196:D197"/>
+    <mergeCell ref="D206:D207"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="A1:A123 A135:A1048576">
-    <cfRule type="containsText" dxfId="13" priority="19" operator="containsText" text="K">
+    <cfRule type="containsText" dxfId="15" priority="19" operator="containsText" text="K">
       <formula>NOT(ISERROR(SEARCH("K",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="20" operator="containsText" text="H">
+    <cfRule type="containsText" dxfId="14" priority="20" operator="containsText" text="H">
       <formula>NOT(ISERROR(SEARCH("H",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B135:B1048576 B1:B123">
-    <cfRule type="duplicateValues" dxfId="11" priority="10333"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="10333"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C135:C1048576 C1:C129">
-    <cfRule type="duplicateValues" dxfId="10" priority="10337"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="10337"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E125">
-    <cfRule type="duplicateValues" dxfId="9" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E133">
-    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E141">
-    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E156">
-    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F31 F33:F66 F190:F1048576 F115:F128 F133:F186 F68:F113 F67:G67">
-    <cfRule type="duplicateValues" dxfId="5" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F112">
-    <cfRule type="duplicateValues" dxfId="4" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F124">
-    <cfRule type="duplicateValues" dxfId="3" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F132">
-    <cfRule type="duplicateValues" dxfId="2" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F351:F358 F257:F259 F279:F280 F215 F235 F253 F251 F249 F247 F245 F243 F241 F239 F237 F233 F231 F229 F227 F212 F186 F184 F181 F202 F210 F208 F206 F204 F200 F198 F196 F194 F192 F190 F179 F177 F175 F173 F171 F169 F34 F37 F9 F6 F11 F13 F15 F17 F19 F21 F23 F25 F27 F29 F31 F39 F41 F43 F45 F47 F49 F51 F53 F1:F4 F56:F58 F61:F66 F165:F167 F372:F1048576 F325:F328 F219 F223 F331:F336 F287 F289 F291 F293 F295 F297 F299 F301 F303 F305 F307 F309 F311 F313 F315 F317 F319 F321 F282:F285 F262:F268 F138:F161 F68:F109 F67:G67">
     <cfRule type="duplicateValues" dxfId="0" priority="10363"/>

</xml_diff>

<commit_message>
refactor(m150-onto.rdf): Remove ranges due to OntoParser not converting float values correctly (See issue #30 and #27).
Will have to be corrected in the future.
</commit_message>
<xml_diff>
--- a/M150-Onto_Metamodel_Rework.xlsx
+++ b/M150-Onto_Metamodel_Rework.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jluis\Repositories\M150-Onto\m150-onto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E04D1B3A-3D3A-4806-BA98-11395F45F976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80884029-4A41-4A9F-8573-28C390E54F76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="1" activeTab="1" xr2:uid="{FEE85CB8-E22B-44F8-B2C8-C132767C24A8}"/>
   </bookViews>
@@ -6709,9 +6709,6 @@
     <t>Create new individuals. Type of VideoStorageMedium.</t>
   </si>
   <si>
-    <t>Not a new class.</t>
-  </si>
-  <si>
     <t>Create new class: VideoFile. New individuals type of VideoFile.</t>
   </si>
   <si>
@@ -6773,6 +6770,9 @@
   </si>
   <si>
     <t>This could be an object property with a New class: MeasurementUnit. New individuals. Data property for now.</t>
+  </si>
+  <si>
+    <t>Not a new class. Check RT207.</t>
   </si>
 </sst>
 </file>
@@ -8948,7 +8948,7 @@
       <c r="G22" s="134"/>
       <c r="H22" s="164"/>
       <c r="P22" t="s">
-        <v>2148</v>
+        <v>2147</v>
       </c>
       <c r="T22" t="s">
         <v>2129</v>
@@ -9695,7 +9695,7 @@
         <v>611</v>
       </c>
       <c r="H63" s="164" t="s">
-        <v>2160</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="24" thickBot="1" x14ac:dyDescent="0.5">
@@ -10907,7 +10907,7 @@
         <v>611</v>
       </c>
       <c r="H126" s="89" t="s">
-        <v>2158</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.45">
@@ -11028,7 +11028,7 @@
         <v>611</v>
       </c>
       <c r="H133" s="89" t="s">
-        <v>2159</v>
+        <v>2158</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.45">
@@ -12308,7 +12308,7 @@
       <c r="G208" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H208" s="89" t="s">
+      <c r="H208" s="90" t="s">
         <v>2139</v>
       </c>
     </row>
@@ -12328,8 +12328,8 @@
       <c r="G209" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H209" s="89" t="s">
-        <v>2140</v>
+      <c r="H209" s="90" t="s">
+        <v>2161</v>
       </c>
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.45">
@@ -12350,7 +12350,7 @@
         <v>611</v>
       </c>
       <c r="H210" s="89" t="s">
-        <v>2141</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.45">
@@ -12578,7 +12578,7 @@
         <v>611</v>
       </c>
       <c r="H223" s="89" t="s">
-        <v>2142</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="224" spans="1:8" x14ac:dyDescent="0.45">
@@ -12598,7 +12598,7 @@
         <v>611</v>
       </c>
       <c r="H224" s="89" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
     </row>
     <row r="225" spans="1:8" x14ac:dyDescent="0.45">
@@ -12688,7 +12688,7 @@
         <v>611</v>
       </c>
       <c r="H229" s="89" t="s">
-        <v>2144</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="230" spans="1:8" x14ac:dyDescent="0.45">
@@ -12731,7 +12731,7 @@
         <v>873</v>
       </c>
       <c r="H231" s="89" t="s">
-        <v>2145</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="232" spans="1:8" x14ac:dyDescent="0.45">
@@ -13197,7 +13197,7 @@
         <v>633</v>
       </c>
       <c r="D258" s="32" t="s">
-        <v>2146</v>
+        <v>2145</v>
       </c>
       <c r="E258" s="76" t="s">
         <v>694</v>
@@ -13209,7 +13209,7 @@
         <v>611</v>
       </c>
       <c r="H258" s="89" t="s">
-        <v>2147</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="259" spans="1:8" x14ac:dyDescent="0.45">
@@ -13369,7 +13369,7 @@
         <v>611</v>
       </c>
       <c r="H267" s="89" t="s">
-        <v>2161</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="268" spans="1:8" x14ac:dyDescent="0.45">
@@ -13472,7 +13472,7 @@
         <v>611</v>
       </c>
       <c r="H274" s="89" t="s">
-        <v>2149</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="275" spans="1:8" x14ac:dyDescent="0.45">
@@ -13486,7 +13486,7 @@
         <v>879</v>
       </c>
       <c r="D275" s="98" t="s">
-        <v>2150</v>
+        <v>2149</v>
       </c>
       <c r="E275" s="93"/>
       <c r="F275" s="100" t="s">
@@ -13508,7 +13508,7 @@
         <v>880</v>
       </c>
       <c r="D276" s="45" t="s">
-        <v>2151</v>
+        <v>2150</v>
       </c>
       <c r="E276" s="93"/>
       <c r="F276" s="100" t="s">
@@ -13558,7 +13558,7 @@
         <v>611</v>
       </c>
       <c r="H278" s="89" t="s">
-        <v>2152</v>
+        <v>2151</v>
       </c>
     </row>
     <row r="279" spans="1:8" x14ac:dyDescent="0.45">
@@ -13651,7 +13651,7 @@
         <v>611</v>
       </c>
       <c r="H285" s="89" t="s">
-        <v>2153</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="286" spans="1:8" x14ac:dyDescent="0.45">
@@ -13984,7 +13984,7 @@
         <v>611</v>
       </c>
       <c r="H303" s="89" t="s">
-        <v>2154</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="304" spans="1:8" x14ac:dyDescent="0.45">
@@ -14055,7 +14055,7 @@
         <v>618</v>
       </c>
       <c r="H307" s="89" t="s">
-        <v>2155</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="308" spans="1:8" x14ac:dyDescent="0.45">
@@ -14160,7 +14160,7 @@
         <v>611</v>
       </c>
       <c r="H313" s="89" t="s">
-        <v>2157</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="314" spans="1:8" x14ac:dyDescent="0.45">
@@ -14486,7 +14486,7 @@
         <v>893</v>
       </c>
       <c r="D335" s="32" t="s">
-        <v>2156</v>
+        <v>2155</v>
       </c>
       <c r="E335" s="102"/>
       <c r="F335" s="92" t="s">

</xml_diff>

<commit_message>
feat(ontology): restore rdfs:range axioms on all data properties
Add Scripts/5_add_datatype_property_ranges.py driven by the new
Scripts/dataproperties.csv (79 property → XSD-type mappings).
65 ranges inserted into m150-onto.rdf; 14 pre-existing ranges left
untouched. Decimal-valued properties use xsd:decimal to match
owlready2 serialization. Partly resolves issue #27 and closes #30.
</commit_message>
<xml_diff>
--- a/M150-Onto_Metamodel_Rework.xlsx
+++ b/M150-Onto_Metamodel_Rework.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jluis\Repositories\M150-Onto\m150-onto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80884029-4A41-4A9F-8573-28C390E54F76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FF8D4B-BE8D-4A21-9C3A-8A7C5BCE24E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="1" activeTab="1" xr2:uid="{FEE85CB8-E22B-44F8-B2C8-C132767C24A8}"/>
   </bookViews>
@@ -19,6 +19,7 @@
     <sheet name="Type Z Raw Data" sheetId="5" r:id="rId4"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'M150-Onto'!$A$184:$H$213</definedName>
     <definedName name="TypZ" localSheetId="3">'Type Z Raw Data'!$A$1:$Y$349</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -6779,7 +6780,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6926,8 +6927,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6977,6 +6985,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -7357,7 +7370,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="10">
+  <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -7368,8 +7381,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="165">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -7630,6 +7644,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="9"/>
     <xf numFmtId="49" fontId="6" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -7810,9 +7825,9 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="9"/>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" xfId="10"/>
   </cellXfs>
-  <cellStyles count="10">
+  <cellStyles count="11">
     <cellStyle name="20% - Accent1" xfId="4" builtinId="30"/>
     <cellStyle name="40% - Accent1" xfId="5" builtinId="31"/>
     <cellStyle name="Accent1" xfId="3" builtinId="29"/>
@@ -7821,6 +7836,7 @@
     <cellStyle name="Good" xfId="9" builtinId="26"/>
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="7" builtinId="17"/>
+    <cellStyle name="Neutral" xfId="10" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="6" xr:uid="{73184220-ECEF-4E4B-9D39-939CEB9C7E6F}"/>
   </cellStyles>
@@ -8291,6 +8307,26 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="645" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{5067DCF1-AA0F-46D2-920D-68C150BE6311}">
+  <we:reference id="WA200010725" version="1.0.0.1" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010725" version="1.0.0.1" store="WA200010725" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{655DA492-23D4-4B0E-933F-AB627B415EAD}">
   <dimension ref="B2:F15"/>
@@ -8549,13 +8585,13 @@
       <c r="C4" s="20" t="s">
         <v>1017</v>
       </c>
-      <c r="E4" s="146" t="s">
+      <c r="E4" s="147" t="s">
         <v>695</v>
       </c>
-      <c r="F4" s="147" t="s">
+      <c r="F4" s="148" t="s">
         <v>799</v>
       </c>
-      <c r="G4" s="147" t="s">
+      <c r="G4" s="148" t="s">
         <v>611</v>
       </c>
     </row>
@@ -8569,9 +8605,9 @@
       <c r="C5" s="20" t="s">
         <v>838</v>
       </c>
-      <c r="E5" s="146"/>
-      <c r="F5" s="147"/>
-      <c r="G5" s="147"/>
+      <c r="E5" s="147"/>
+      <c r="F5" s="148"/>
+      <c r="G5" s="148"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A6" s="18" t="s">
@@ -8583,11 +8619,11 @@
       <c r="C6" s="20" t="s">
         <v>1018</v>
       </c>
-      <c r="E6" s="146"/>
-      <c r="F6" s="148" t="s">
+      <c r="E6" s="147"/>
+      <c r="F6" s="149" t="s">
         <v>800</v>
       </c>
-      <c r="G6" s="147" t="s">
+      <c r="G6" s="148" t="s">
         <v>611</v>
       </c>
     </row>
@@ -8601,9 +8637,9 @@
       <c r="C7" s="20" t="s">
         <v>839</v>
       </c>
-      <c r="E7" s="146"/>
-      <c r="F7" s="148"/>
-      <c r="G7" s="147"/>
+      <c r="E7" s="147"/>
+      <c r="F7" s="149"/>
+      <c r="G7" s="148"/>
       <c r="N7" t="s">
         <v>2122</v>
       </c>
@@ -8618,19 +8654,19 @@
       <c r="C9" s="20" t="s">
         <v>801</v>
       </c>
-      <c r="D9" s="163" t="s">
+      <c r="D9" s="164" t="s">
         <v>976</v>
       </c>
-      <c r="E9" s="143" t="s">
+      <c r="E9" s="144" t="s">
         <v>694</v>
       </c>
-      <c r="F9" s="141" t="s">
+      <c r="F9" s="142" t="s">
         <v>699</v>
       </c>
-      <c r="G9" s="134" t="s">
+      <c r="G9" s="135" t="s">
         <v>611</v>
       </c>
-      <c r="H9" s="164" t="s">
+      <c r="H9" s="104" t="s">
         <v>2105</v>
       </c>
     </row>
@@ -8644,11 +8680,11 @@
       <c r="C10" s="20" t="s">
         <v>801</v>
       </c>
-      <c r="D10" s="163"/>
-      <c r="E10" s="117"/>
-      <c r="F10" s="142"/>
-      <c r="G10" s="134"/>
-      <c r="H10" s="164"/>
+      <c r="D10" s="164"/>
+      <c r="E10" s="118"/>
+      <c r="F10" s="143"/>
+      <c r="G10" s="135"/>
+      <c r="H10" s="104"/>
       <c r="N10" t="s">
         <v>2123</v>
       </c>
@@ -8666,14 +8702,14 @@
       <c r="C11" s="20" t="s">
         <v>802</v>
       </c>
-      <c r="E11" s="117"/>
-      <c r="F11" s="136" t="s">
+      <c r="E11" s="118"/>
+      <c r="F11" s="137" t="s">
         <v>698</v>
       </c>
-      <c r="G11" s="134" t="s">
+      <c r="G11" s="135" t="s">
         <v>611</v>
       </c>
-      <c r="H11" s="164" t="s">
+      <c r="H11" s="104" t="s">
         <v>2117</v>
       </c>
       <c r="O11" t="s">
@@ -8690,10 +8726,10 @@
       <c r="C12" s="20" t="s">
         <v>802</v>
       </c>
-      <c r="E12" s="117"/>
-      <c r="F12" s="136"/>
-      <c r="G12" s="134"/>
-      <c r="H12" s="164"/>
+      <c r="E12" s="118"/>
+      <c r="F12" s="137"/>
+      <c r="G12" s="135"/>
+      <c r="H12" s="104"/>
       <c r="P12" t="s">
         <v>2118</v>
       </c>
@@ -8711,17 +8747,17 @@
       <c r="C13" s="20" t="s">
         <v>788</v>
       </c>
-      <c r="D13" s="163" t="s">
+      <c r="D13" s="164" t="s">
         <v>977</v>
       </c>
-      <c r="E13" s="117"/>
-      <c r="F13" s="136" t="s">
+      <c r="E13" s="118"/>
+      <c r="F13" s="137" t="s">
         <v>700</v>
       </c>
-      <c r="G13" s="134" t="s">
+      <c r="G13" s="135" t="s">
         <v>611</v>
       </c>
-      <c r="H13" s="164" t="s">
+      <c r="H13" s="104" t="s">
         <v>2115</v>
       </c>
       <c r="P13" t="s">
@@ -8741,11 +8777,11 @@
       <c r="C14" s="20" t="s">
         <v>788</v>
       </c>
-      <c r="D14" s="163"/>
-      <c r="E14" s="117"/>
-      <c r="F14" s="136"/>
-      <c r="G14" s="134"/>
-      <c r="H14" s="164"/>
+      <c r="D14" s="164"/>
+      <c r="E14" s="118"/>
+      <c r="F14" s="137"/>
+      <c r="G14" s="135"/>
+      <c r="H14" s="104"/>
       <c r="P14" t="s">
         <v>2121</v>
       </c>
@@ -8763,14 +8799,14 @@
       <c r="C15" s="20" t="s">
         <v>803</v>
       </c>
-      <c r="E15" s="117"/>
-      <c r="F15" s="136" t="s">
+      <c r="E15" s="118"/>
+      <c r="F15" s="137" t="s">
         <v>701</v>
       </c>
-      <c r="G15" s="134" t="s">
+      <c r="G15" s="135" t="s">
         <v>611</v>
       </c>
-      <c r="H15" s="164" t="s">
+      <c r="H15" s="104" t="s">
         <v>2114</v>
       </c>
       <c r="O15" t="s">
@@ -8787,10 +8823,10 @@
       <c r="C16" s="20" t="s">
         <v>803</v>
       </c>
-      <c r="E16" s="117"/>
-      <c r="F16" s="136"/>
-      <c r="G16" s="134"/>
-      <c r="H16" s="164"/>
+      <c r="E16" s="118"/>
+      <c r="F16" s="137"/>
+      <c r="G16" s="135"/>
+      <c r="H16" s="104"/>
       <c r="P16" t="s">
         <v>2108</v>
       </c>
@@ -8808,17 +8844,17 @@
       <c r="C17" s="20" t="s">
         <v>794</v>
       </c>
-      <c r="D17" s="163" t="s">
+      <c r="D17" s="164" t="s">
         <v>978</v>
       </c>
-      <c r="E17" s="117"/>
-      <c r="F17" s="135" t="s">
+      <c r="E17" s="118"/>
+      <c r="F17" s="136" t="s">
         <v>795</v>
       </c>
-      <c r="G17" s="134" t="s">
+      <c r="G17" s="135" t="s">
         <v>611</v>
       </c>
-      <c r="H17" s="164" t="s">
+      <c r="H17" s="104" t="s">
         <v>2116</v>
       </c>
       <c r="P17" t="s">
@@ -8838,11 +8874,11 @@
       <c r="C18" s="20" t="s">
         <v>794</v>
       </c>
-      <c r="D18" s="163"/>
-      <c r="E18" s="117"/>
-      <c r="F18" s="135"/>
-      <c r="G18" s="134"/>
-      <c r="H18" s="164"/>
+      <c r="D18" s="164"/>
+      <c r="E18" s="118"/>
+      <c r="F18" s="136"/>
+      <c r="G18" s="135"/>
+      <c r="H18" s="104"/>
       <c r="P18" t="s">
         <v>2110</v>
       </c>
@@ -8860,17 +8896,17 @@
       <c r="C19" s="20" t="s">
         <v>796</v>
       </c>
-      <c r="D19" s="163" t="s">
+      <c r="D19" s="164" t="s">
         <v>979</v>
       </c>
-      <c r="E19" s="117"/>
-      <c r="F19" s="135" t="s">
+      <c r="E19" s="118"/>
+      <c r="F19" s="136" t="s">
         <v>797</v>
       </c>
-      <c r="G19" s="134" t="s">
+      <c r="G19" s="135" t="s">
         <v>611</v>
       </c>
-      <c r="H19" s="164" t="s">
+      <c r="H19" s="104" t="s">
         <v>2113</v>
       </c>
       <c r="P19" t="s">
@@ -8890,11 +8926,11 @@
       <c r="C20" s="20" t="s">
         <v>796</v>
       </c>
-      <c r="D20" s="163"/>
-      <c r="E20" s="117"/>
-      <c r="F20" s="135"/>
-      <c r="G20" s="134"/>
-      <c r="H20" s="164"/>
+      <c r="D20" s="164"/>
+      <c r="E20" s="118"/>
+      <c r="F20" s="136"/>
+      <c r="G20" s="135"/>
+      <c r="H20" s="104"/>
       <c r="O20" t="s">
         <v>2124</v>
       </c>
@@ -8909,17 +8945,17 @@
       <c r="C21" s="20" t="s">
         <v>804</v>
       </c>
-      <c r="D21" s="163" t="s">
+      <c r="D21" s="164" t="s">
         <v>980</v>
       </c>
-      <c r="E21" s="117"/>
-      <c r="F21" s="136" t="s">
+      <c r="E21" s="118"/>
+      <c r="F21" s="137" t="s">
         <v>702</v>
       </c>
-      <c r="G21" s="134" t="s">
+      <c r="G21" s="135" t="s">
         <v>611</v>
       </c>
-      <c r="H21" s="164" t="s">
+      <c r="H21" s="104" t="s">
         <v>2112</v>
       </c>
       <c r="P21" t="s">
@@ -8942,11 +8978,11 @@
       <c r="C22" s="20" t="s">
         <v>804</v>
       </c>
-      <c r="D22" s="163"/>
-      <c r="E22" s="117"/>
-      <c r="F22" s="136"/>
-      <c r="G22" s="134"/>
-      <c r="H22" s="164"/>
+      <c r="D22" s="164"/>
+      <c r="E22" s="118"/>
+      <c r="F22" s="137"/>
+      <c r="G22" s="135"/>
+      <c r="H22" s="104"/>
       <c r="P22" t="s">
         <v>2147</v>
       </c>
@@ -8967,17 +9003,17 @@
       <c r="C23" s="20" t="s">
         <v>805</v>
       </c>
-      <c r="D23" s="163" t="s">
+      <c r="D23" s="164" t="s">
         <v>981</v>
       </c>
-      <c r="E23" s="117"/>
-      <c r="F23" s="136" t="s">
+      <c r="E23" s="118"/>
+      <c r="F23" s="137" t="s">
         <v>703</v>
       </c>
-      <c r="G23" s="134" t="s">
+      <c r="G23" s="135" t="s">
         <v>611</v>
       </c>
-      <c r="H23" s="164" t="s">
+      <c r="H23" s="104" t="s">
         <v>2120</v>
       </c>
       <c r="O23" t="s">
@@ -8994,10 +9030,10 @@
       <c r="C24" s="20" t="s">
         <v>805</v>
       </c>
-      <c r="D24" s="163"/>
-      <c r="E24" s="117"/>
-      <c r="F24" s="136"/>
-      <c r="G24" s="134"/>
+      <c r="D24" s="164"/>
+      <c r="E24" s="118"/>
+      <c r="F24" s="137"/>
+      <c r="G24" s="135"/>
       <c r="P24" t="s">
         <v>2133</v>
       </c>
@@ -9015,14 +9051,14 @@
       <c r="C25" s="20" t="s">
         <v>807</v>
       </c>
-      <c r="D25" s="163" t="s">
+      <c r="D25" s="164" t="s">
         <v>982</v>
       </c>
-      <c r="E25" s="117"/>
-      <c r="F25" s="136" t="s">
+      <c r="E25" s="118"/>
+      <c r="F25" s="137" t="s">
         <v>704</v>
       </c>
-      <c r="G25" s="134" t="s">
+      <c r="G25" s="135" t="s">
         <v>611</v>
       </c>
       <c r="P25" t="s">
@@ -9042,10 +9078,10 @@
       <c r="C26" s="20" t="s">
         <v>807</v>
       </c>
-      <c r="D26" s="163"/>
-      <c r="E26" s="117"/>
-      <c r="F26" s="136"/>
-      <c r="G26" s="134"/>
+      <c r="D26" s="164"/>
+      <c r="E26" s="118"/>
+      <c r="F26" s="137"/>
+      <c r="G26" s="135"/>
       <c r="O26" t="s">
         <v>2135</v>
       </c>
@@ -9060,14 +9096,14 @@
       <c r="C27" s="20" t="s">
         <v>808</v>
       </c>
-      <c r="D27" s="163" t="s">
+      <c r="D27" s="164" t="s">
         <v>983</v>
       </c>
-      <c r="E27" s="117"/>
-      <c r="F27" s="136" t="s">
+      <c r="E27" s="118"/>
+      <c r="F27" s="137" t="s">
         <v>2080</v>
       </c>
-      <c r="G27" s="134" t="s">
+      <c r="G27" s="135" t="s">
         <v>611</v>
       </c>
       <c r="P27" t="s">
@@ -9087,10 +9123,10 @@
       <c r="C28" s="20" t="s">
         <v>808</v>
       </c>
-      <c r="D28" s="163"/>
-      <c r="E28" s="118"/>
-      <c r="F28" s="136"/>
-      <c r="G28" s="134"/>
+      <c r="D28" s="164"/>
+      <c r="E28" s="119"/>
+      <c r="F28" s="137"/>
+      <c r="G28" s="135"/>
       <c r="P28" t="s">
         <v>643</v>
       </c>
@@ -9108,13 +9144,13 @@
       <c r="C29" s="20" t="s">
         <v>809</v>
       </c>
-      <c r="E29" s="144" t="s">
+      <c r="E29" s="145" t="s">
         <v>695</v>
       </c>
-      <c r="F29" s="139" t="s">
+      <c r="F29" s="140" t="s">
         <v>705</v>
       </c>
-      <c r="G29" s="153" t="s">
+      <c r="G29" s="154" t="s">
         <v>873</v>
       </c>
       <c r="P29" t="s">
@@ -9131,9 +9167,9 @@
       <c r="C30" s="20" t="s">
         <v>809</v>
       </c>
-      <c r="E30" s="145"/>
-      <c r="F30" s="140"/>
-      <c r="G30" s="154"/>
+      <c r="E30" s="146"/>
+      <c r="F30" s="141"/>
+      <c r="G30" s="155"/>
       <c r="P30" t="s">
         <v>653</v>
       </c>
@@ -9148,16 +9184,16 @@
       <c r="C31" s="20" t="s">
         <v>810</v>
       </c>
-      <c r="D31" s="163" t="s">
+      <c r="D31" s="164" t="s">
         <v>984</v>
       </c>
-      <c r="E31" s="143" t="s">
+      <c r="E31" s="144" t="s">
         <v>694</v>
       </c>
-      <c r="F31" s="141" t="s">
+      <c r="F31" s="142" t="s">
         <v>706</v>
       </c>
-      <c r="G31" s="151" t="s">
+      <c r="G31" s="152" t="s">
         <v>611</v>
       </c>
       <c r="P31" t="s">
@@ -9174,10 +9210,10 @@
       <c r="C32" s="20" t="s">
         <v>810</v>
       </c>
-      <c r="D32" s="163"/>
-      <c r="E32" s="118"/>
-      <c r="F32" s="142"/>
-      <c r="G32" s="152"/>
+      <c r="D32" s="164"/>
+      <c r="E32" s="119"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="153"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="18" t="s">
@@ -9192,13 +9228,13 @@
       <c r="D34" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E34" s="144" t="s">
+      <c r="E34" s="145" t="s">
         <v>695</v>
       </c>
-      <c r="F34" s="149" t="s">
+      <c r="F34" s="150" t="s">
         <v>709</v>
       </c>
-      <c r="G34" s="150" t="s">
+      <c r="G34" s="151" t="s">
         <v>614</v>
       </c>
     </row>
@@ -9212,9 +9248,9 @@
       <c r="C35" s="20" t="s">
         <v>806</v>
       </c>
-      <c r="E35" s="145"/>
-      <c r="F35" s="149"/>
-      <c r="G35" s="150"/>
+      <c r="E35" s="146"/>
+      <c r="F35" s="150"/>
+      <c r="G35" s="151"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="18" t="s">
@@ -9226,16 +9262,16 @@
       <c r="C37" s="20" t="s">
         <v>831</v>
       </c>
-      <c r="D37" s="163" t="s">
+      <c r="D37" s="164" t="s">
         <v>993</v>
       </c>
-      <c r="E37" s="137" t="s">
+      <c r="E37" s="138" t="s">
         <v>694</v>
       </c>
-      <c r="F37" s="136" t="s">
+      <c r="F37" s="137" t="s">
         <v>711</v>
       </c>
-      <c r="G37" s="134" t="s">
+      <c r="G37" s="135" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9249,10 +9285,10 @@
       <c r="C38" s="20" t="s">
         <v>831</v>
       </c>
-      <c r="D38" s="163"/>
-      <c r="E38" s="138"/>
-      <c r="F38" s="136"/>
-      <c r="G38" s="134"/>
+      <c r="D38" s="164"/>
+      <c r="E38" s="139"/>
+      <c r="F38" s="137"/>
+      <c r="G38" s="135"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="18" t="s">
@@ -9264,14 +9300,14 @@
       <c r="C39" s="20" t="s">
         <v>566</v>
       </c>
-      <c r="D39" s="163" t="s">
+      <c r="D39" s="164" t="s">
         <v>994</v>
       </c>
-      <c r="E39" s="138"/>
-      <c r="F39" s="136" t="s">
+      <c r="E39" s="139"/>
+      <c r="F39" s="137" t="s">
         <v>712</v>
       </c>
-      <c r="G39" s="134" t="s">
+      <c r="G39" s="135" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9285,10 +9321,10 @@
       <c r="C40" s="20" t="s">
         <v>566</v>
       </c>
-      <c r="D40" s="163"/>
-      <c r="E40" s="138"/>
-      <c r="F40" s="136"/>
-      <c r="G40" s="134"/>
+      <c r="D40" s="164"/>
+      <c r="E40" s="139"/>
+      <c r="F40" s="137"/>
+      <c r="G40" s="135"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="18" t="s">
@@ -9300,14 +9336,14 @@
       <c r="C41" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="D41" s="163" t="s">
+      <c r="D41" s="164" t="s">
         <v>995</v>
       </c>
-      <c r="E41" s="138"/>
-      <c r="F41" s="136" t="s">
+      <c r="E41" s="139"/>
+      <c r="F41" s="137" t="s">
         <v>717</v>
       </c>
-      <c r="G41" s="134" t="s">
+      <c r="G41" s="135" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9321,10 +9357,10 @@
       <c r="C42" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="D42" s="163"/>
-      <c r="E42" s="138"/>
-      <c r="F42" s="136"/>
-      <c r="G42" s="134"/>
+      <c r="D42" s="164"/>
+      <c r="E42" s="139"/>
+      <c r="F42" s="137"/>
+      <c r="G42" s="135"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="18" t="s">
@@ -9336,14 +9372,14 @@
       <c r="C43" s="20" t="s">
         <v>833</v>
       </c>
-      <c r="D43" s="163" t="s">
+      <c r="D43" s="164" t="s">
         <v>996</v>
       </c>
-      <c r="E43" s="138"/>
-      <c r="F43" s="136" t="s">
+      <c r="E43" s="139"/>
+      <c r="F43" s="137" t="s">
         <v>713</v>
       </c>
-      <c r="G43" s="134" t="s">
+      <c r="G43" s="135" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9357,10 +9393,10 @@
       <c r="C44" s="20" t="s">
         <v>833</v>
       </c>
-      <c r="D44" s="163"/>
-      <c r="E44" s="138"/>
-      <c r="F44" s="136"/>
-      <c r="G44" s="134"/>
+      <c r="D44" s="164"/>
+      <c r="E44" s="139"/>
+      <c r="F44" s="137"/>
+      <c r="G44" s="135"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="18" t="s">
@@ -9372,14 +9408,14 @@
       <c r="C45" s="20" t="s">
         <v>834</v>
       </c>
-      <c r="D45" s="163" t="s">
+      <c r="D45" s="164" t="s">
         <v>997</v>
       </c>
-      <c r="E45" s="138"/>
-      <c r="F45" s="136" t="s">
+      <c r="E45" s="139"/>
+      <c r="F45" s="137" t="s">
         <v>714</v>
       </c>
-      <c r="G45" s="134" t="s">
+      <c r="G45" s="135" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9393,10 +9429,10 @@
       <c r="C46" s="20" t="s">
         <v>834</v>
       </c>
-      <c r="D46" s="163"/>
-      <c r="E46" s="138"/>
-      <c r="F46" s="136"/>
-      <c r="G46" s="134"/>
+      <c r="D46" s="164"/>
+      <c r="E46" s="139"/>
+      <c r="F46" s="137"/>
+      <c r="G46" s="135"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A47" s="18" t="s">
@@ -9408,14 +9444,14 @@
       <c r="C47" s="20" t="s">
         <v>835</v>
       </c>
-      <c r="D47" s="163" t="s">
+      <c r="D47" s="164" t="s">
         <v>998</v>
       </c>
-      <c r="E47" s="138"/>
-      <c r="F47" s="136" t="s">
+      <c r="E47" s="139"/>
+      <c r="F47" s="137" t="s">
         <v>864</v>
       </c>
-      <c r="G47" s="134" t="s">
+      <c r="G47" s="135" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9429,10 +9465,10 @@
       <c r="C48" s="20" t="s">
         <v>835</v>
       </c>
-      <c r="D48" s="163"/>
-      <c r="E48" s="138"/>
-      <c r="F48" s="136"/>
-      <c r="G48" s="134"/>
+      <c r="D48" s="164"/>
+      <c r="E48" s="139"/>
+      <c r="F48" s="137"/>
+      <c r="G48" s="135"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A49" s="18" t="s">
@@ -9444,14 +9480,14 @@
       <c r="C49" s="20" t="s">
         <v>836</v>
       </c>
-      <c r="D49" s="163" t="s">
+      <c r="D49" s="164" t="s">
         <v>999</v>
       </c>
-      <c r="E49" s="138"/>
-      <c r="F49" s="136" t="s">
+      <c r="E49" s="139"/>
+      <c r="F49" s="137" t="s">
         <v>715</v>
       </c>
-      <c r="G49" s="134" t="s">
+      <c r="G49" s="135" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9465,10 +9501,10 @@
       <c r="C50" s="20" t="s">
         <v>836</v>
       </c>
-      <c r="D50" s="163"/>
-      <c r="E50" s="138"/>
-      <c r="F50" s="136"/>
-      <c r="G50" s="134"/>
+      <c r="D50" s="164"/>
+      <c r="E50" s="139"/>
+      <c r="F50" s="137"/>
+      <c r="G50" s="135"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A51" s="18" t="s">
@@ -9480,14 +9516,14 @@
       <c r="C51" s="20" t="s">
         <v>860</v>
       </c>
-      <c r="D51" s="163" t="s">
+      <c r="D51" s="164" t="s">
         <v>1000</v>
       </c>
-      <c r="E51" s="138"/>
-      <c r="F51" s="135" t="s">
+      <c r="E51" s="139"/>
+      <c r="F51" s="136" t="s">
         <v>798</v>
       </c>
-      <c r="G51" s="134" t="s">
+      <c r="G51" s="135" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9501,10 +9537,10 @@
       <c r="C52" s="20" t="s">
         <v>860</v>
       </c>
-      <c r="D52" s="163"/>
-      <c r="E52" s="138"/>
-      <c r="F52" s="135"/>
-      <c r="G52" s="134"/>
+      <c r="D52" s="164"/>
+      <c r="E52" s="139"/>
+      <c r="F52" s="136"/>
+      <c r="G52" s="135"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A53" s="18" t="s">
@@ -9516,14 +9552,14 @@
       <c r="C53" s="20" t="s">
         <v>837</v>
       </c>
-      <c r="D53" s="163" t="s">
+      <c r="D53" s="164" t="s">
         <v>1001</v>
       </c>
-      <c r="E53" s="138"/>
-      <c r="F53" s="136" t="s">
+      <c r="E53" s="139"/>
+      <c r="F53" s="137" t="s">
         <v>716</v>
       </c>
-      <c r="G53" s="134" t="s">
+      <c r="G53" s="135" t="s">
         <v>611</v>
       </c>
     </row>
@@ -9537,16 +9573,16 @@
       <c r="C54" s="20" t="s">
         <v>837</v>
       </c>
-      <c r="D54" s="163"/>
-      <c r="E54" s="138"/>
-      <c r="F54" s="136"/>
-      <c r="G54" s="134"/>
+      <c r="D54" s="164"/>
+      <c r="E54" s="139"/>
+      <c r="F54" s="137"/>
+      <c r="G54" s="135"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="E56" s="105" t="s">
+      <c r="E56" s="106" t="s">
         <v>790</v>
       </c>
-      <c r="F56" s="105"/>
+      <c r="F56" s="106"/>
       <c r="G56" s="28" t="s">
         <v>613</v>
       </c>
@@ -9582,7 +9618,7 @@
       <c r="D58" s="32" t="s">
         <v>616</v>
       </c>
-      <c r="E58" s="109" t="s">
+      <c r="E58" s="110" t="s">
         <v>694</v>
       </c>
       <c r="F58" s="61" t="s">
@@ -9603,7 +9639,7 @@
       <c r="D59" s="32" t="s">
         <v>616</v>
       </c>
-      <c r="E59" s="110"/>
+      <c r="E59" s="111"/>
       <c r="F59" s="63" t="s">
         <v>2098</v>
       </c>
@@ -9622,7 +9658,7 @@
       <c r="D60" s="32" t="s">
         <v>616</v>
       </c>
-      <c r="E60" s="110"/>
+      <c r="E60" s="111"/>
       <c r="F60" s="65" t="s">
         <v>2099</v>
       </c>
@@ -9641,7 +9677,7 @@
       <c r="D61" s="32" t="s">
         <v>2052</v>
       </c>
-      <c r="E61" s="119"/>
+      <c r="E61" s="120"/>
       <c r="F61" s="27" t="s">
         <v>923</v>
       </c>
@@ -9694,7 +9730,7 @@
       <c r="G63" s="25" t="s">
         <v>611</v>
       </c>
-      <c r="H63" s="164" t="s">
+      <c r="H63" s="104" t="s">
         <v>2159</v>
       </c>
     </row>
@@ -9774,7 +9810,7 @@
       <c r="C67" s="20" t="s">
         <v>567</v>
       </c>
-      <c r="E67" s="109" t="s">
+      <c r="E67" s="110" t="s">
         <v>694</v>
       </c>
       <c r="F67" s="34" t="s">
@@ -9795,7 +9831,7 @@
       <c r="D68" s="32" t="s">
         <v>2054</v>
       </c>
-      <c r="E68" s="110"/>
+      <c r="E68" s="111"/>
       <c r="F68" s="27" t="s">
         <v>929</v>
       </c>
@@ -9816,7 +9852,7 @@
       <c r="D69" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E69" s="111" t="s">
+      <c r="E69" s="112" t="s">
         <v>695</v>
       </c>
       <c r="F69" s="73" t="s">
@@ -9839,7 +9875,7 @@
       <c r="D70" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E70" s="112"/>
+      <c r="E70" s="113"/>
       <c r="F70" s="73" t="s">
         <v>931</v>
       </c>
@@ -9860,7 +9896,7 @@
       <c r="D71" s="32" t="s">
         <v>2055</v>
       </c>
-      <c r="E71" s="109" t="s">
+      <c r="E71" s="110" t="s">
         <v>694</v>
       </c>
       <c r="F71" s="27" t="s">
@@ -9883,7 +9919,7 @@
       <c r="D72" s="32" t="s">
         <v>984</v>
       </c>
-      <c r="E72" s="110"/>
+      <c r="E72" s="111"/>
       <c r="F72" s="27" t="s">
         <v>933</v>
       </c>
@@ -9904,7 +9940,7 @@
       <c r="D73" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E73" s="111" t="s">
+      <c r="E73" s="112" t="s">
         <v>695</v>
       </c>
       <c r="F73" s="73" t="s">
@@ -9927,7 +9963,7 @@
       <c r="D74" s="32" t="s">
         <v>605</v>
       </c>
-      <c r="E74" s="112"/>
+      <c r="E74" s="113"/>
       <c r="F74" s="73" t="s">
         <v>708</v>
       </c>
@@ -10014,7 +10050,7 @@
       <c r="C78" s="20" t="s">
         <v>859</v>
       </c>
-      <c r="E78" s="111" t="s">
+      <c r="E78" s="112" t="s">
         <v>695</v>
       </c>
       <c r="F78" s="73" t="s">
@@ -10037,7 +10073,7 @@
       <c r="D79" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E79" s="116"/>
+      <c r="E79" s="117"/>
       <c r="F79" s="73" t="s">
         <v>936</v>
       </c>
@@ -10078,11 +10114,11 @@
       <c r="C81" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E81" s="106" t="s">
+      <c r="E81" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F81" s="106"/>
-      <c r="G81" s="105" t="s">
+      <c r="F81" s="107"/>
+      <c r="G81" s="106" t="s">
         <v>611</v>
       </c>
     </row>
@@ -10096,9 +10132,9 @@
       <c r="C82" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E82" s="107"/>
-      <c r="F82" s="108"/>
-      <c r="G82" s="125"/>
+      <c r="E82" s="108"/>
+      <c r="F82" s="109"/>
+      <c r="G82" s="126"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.45">
       <c r="E83" s="54"/>
@@ -10106,10 +10142,10 @@
       <c r="G83" s="23"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="E84" s="105" t="s">
+      <c r="E84" s="106" t="s">
         <v>868</v>
       </c>
-      <c r="F84" s="105"/>
+      <c r="F84" s="106"/>
       <c r="G84" s="28" t="s">
         <v>613</v>
       </c>
@@ -10145,7 +10181,7 @@
       <c r="D86" s="32" t="s">
         <v>985</v>
       </c>
-      <c r="E86" s="114" t="s">
+      <c r="E86" s="115" t="s">
         <v>694</v>
       </c>
       <c r="F86" s="27" t="s">
@@ -10168,7 +10204,7 @@
       <c r="D87" s="32" t="s">
         <v>986</v>
       </c>
-      <c r="E87" s="117"/>
+      <c r="E87" s="118"/>
       <c r="F87" s="27" t="s">
         <v>939</v>
       </c>
@@ -10189,7 +10225,7 @@
       <c r="D88" s="32" t="s">
         <v>987</v>
       </c>
-      <c r="E88" s="117"/>
+      <c r="E88" s="118"/>
       <c r="F88" s="27" t="s">
         <v>940</v>
       </c>
@@ -10210,7 +10246,7 @@
       <c r="D89" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E89" s="111" t="s">
+      <c r="E89" s="112" t="s">
         <v>695</v>
       </c>
       <c r="F89" s="73" t="s">
@@ -10233,7 +10269,7 @@
       <c r="D90" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E90" s="112"/>
+      <c r="E90" s="113"/>
       <c r="F90" s="73" t="s">
         <v>942</v>
       </c>
@@ -10254,7 +10290,7 @@
       <c r="D91" s="32" t="s">
         <v>987</v>
       </c>
-      <c r="E91" s="114" t="s">
+      <c r="E91" s="115" t="s">
         <v>694</v>
       </c>
       <c r="F91" s="27" t="s">
@@ -10277,7 +10313,7 @@
       <c r="D92" s="32" t="s">
         <v>984</v>
       </c>
-      <c r="E92" s="117"/>
+      <c r="E92" s="118"/>
       <c r="F92" s="27" t="s">
         <v>944</v>
       </c>
@@ -10298,7 +10334,7 @@
       <c r="D93" s="32" t="s">
         <v>988</v>
       </c>
-      <c r="E93" s="117"/>
+      <c r="E93" s="118"/>
       <c r="F93" s="27" t="s">
         <v>2067</v>
       </c>
@@ -10319,7 +10355,7 @@
       <c r="D94" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E94" s="111" t="s">
+      <c r="E94" s="112" t="s">
         <v>695</v>
       </c>
       <c r="F94" s="73" t="s">
@@ -10342,7 +10378,7 @@
       <c r="D95" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E95" s="112"/>
+      <c r="E95" s="113"/>
       <c r="F95" s="73" t="s">
         <v>946</v>
       </c>
@@ -10360,7 +10396,7 @@
       <c r="C96" s="20" t="s">
         <v>819</v>
       </c>
-      <c r="E96" s="112"/>
+      <c r="E96" s="113"/>
       <c r="F96" s="73" t="s">
         <v>947</v>
       </c>
@@ -10423,7 +10459,7 @@
       <c r="D99" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E99" s="111" t="s">
+      <c r="E99" s="112" t="s">
         <v>695</v>
       </c>
       <c r="F99" s="73" t="s">
@@ -10446,7 +10482,7 @@
       <c r="D100" s="32" t="s">
         <v>604</v>
       </c>
-      <c r="E100" s="112"/>
+      <c r="E100" s="113"/>
       <c r="F100" s="73" t="s">
         <v>951</v>
       </c>
@@ -10610,11 +10646,11 @@
       <c r="C108" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E108" s="106" t="s">
+      <c r="E108" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F108" s="106"/>
-      <c r="G108" s="105" t="s">
+      <c r="F108" s="107"/>
+      <c r="G108" s="106" t="s">
         <v>611</v>
       </c>
     </row>
@@ -10628,15 +10664,15 @@
       <c r="C109" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E109" s="107"/>
-      <c r="F109" s="108"/>
-      <c r="G109" s="125"/>
+      <c r="E109" s="108"/>
+      <c r="F109" s="109"/>
+      <c r="G109" s="126"/>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="E111" s="105" t="s">
+      <c r="E111" s="106" t="s">
         <v>868</v>
       </c>
-      <c r="F111" s="105"/>
+      <c r="F111" s="106"/>
       <c r="G111" s="28" t="s">
         <v>613</v>
       </c>
@@ -10713,7 +10749,7 @@
       <c r="C115" s="20" t="s">
         <v>914</v>
       </c>
-      <c r="E115" s="111" t="s">
+      <c r="E115" s="112" t="s">
         <v>695</v>
       </c>
       <c r="F115" s="78" t="s">
@@ -10736,7 +10772,7 @@
       <c r="D116" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E116" s="112"/>
+      <c r="E116" s="113"/>
       <c r="F116" s="78" t="s">
         <v>919</v>
       </c>
@@ -10757,7 +10793,7 @@
       <c r="D117" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E117" s="112"/>
+      <c r="E117" s="113"/>
       <c r="F117" s="78" t="s">
         <v>920</v>
       </c>
@@ -10778,7 +10814,7 @@
       <c r="D118" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="E118" s="113"/>
+      <c r="E118" s="114"/>
       <c r="F118" s="78" t="s">
         <v>921</v>
       </c>
@@ -10817,11 +10853,11 @@
       <c r="C120" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E120" s="106" t="s">
+      <c r="E120" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F120" s="106"/>
-      <c r="G120" s="105" t="s">
+      <c r="F120" s="107"/>
+      <c r="G120" s="106" t="s">
         <v>611</v>
       </c>
     </row>
@@ -10835,9 +10871,9 @@
       <c r="C121" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E121" s="106"/>
-      <c r="F121" s="106"/>
-      <c r="G121" s="105"/>
+      <c r="E121" s="107"/>
+      <c r="F121" s="107"/>
+      <c r="G121" s="106"/>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.45">
       <c r="E122" s="55"/>
@@ -10878,7 +10914,7 @@
         <v>1021</v>
       </c>
       <c r="D125" s="45"/>
-      <c r="E125" s="160" t="s">
+      <c r="E125" s="161" t="s">
         <v>694</v>
       </c>
       <c r="F125" s="24" t="s">
@@ -10899,7 +10935,7 @@
         <v>1022</v>
       </c>
       <c r="D126" s="45"/>
-      <c r="E126" s="161"/>
+      <c r="E126" s="162"/>
       <c r="F126" s="51" t="s">
         <v>1028</v>
       </c>
@@ -10921,7 +10957,7 @@
         <v>1023</v>
       </c>
       <c r="D127" s="45"/>
-      <c r="E127" s="161"/>
+      <c r="E127" s="162"/>
       <c r="F127" s="24" t="s">
         <v>1029</v>
       </c>
@@ -10940,7 +10976,7 @@
         <v>1024</v>
       </c>
       <c r="D128" s="45"/>
-      <c r="E128" s="162"/>
+      <c r="E128" s="163"/>
       <c r="F128" s="24" t="s">
         <v>1030</v>
       </c>
@@ -10959,10 +10995,10 @@
         <v>601</v>
       </c>
       <c r="D129" s="45"/>
-      <c r="E129" s="158" t="s">
+      <c r="E129" s="159" t="s">
         <v>620</v>
       </c>
-      <c r="F129" s="159"/>
+      <c r="F129" s="160"/>
       <c r="G129" s="26" t="s">
         <v>611</v>
       </c>
@@ -11018,7 +11054,7 @@
         <v>1025</v>
       </c>
       <c r="D133" s="45"/>
-      <c r="E133" s="114" t="s">
+      <c r="E133" s="115" t="s">
         <v>694</v>
       </c>
       <c r="F133" s="24" t="s">
@@ -11042,7 +11078,7 @@
         <v>1026</v>
       </c>
       <c r="D134" s="45"/>
-      <c r="E134" s="115"/>
+      <c r="E134" s="116"/>
       <c r="F134" s="24" t="s">
         <v>2068</v>
       </c>
@@ -11061,10 +11097,10 @@
       <c r="H136" s="91"/>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="E138" s="157" t="s">
+      <c r="E138" s="158" t="s">
         <v>907</v>
       </c>
-      <c r="F138" s="157"/>
+      <c r="F138" s="158"/>
       <c r="G138" s="28" t="s">
         <v>613</v>
       </c>
@@ -11122,7 +11158,7 @@
       <c r="D141" s="32" t="s">
         <v>2058</v>
       </c>
-      <c r="E141" s="114" t="s">
+      <c r="E141" s="115" t="s">
         <v>694</v>
       </c>
       <c r="F141" s="27" t="s">
@@ -11145,7 +11181,7 @@
       <c r="D142" s="32" t="s">
         <v>2059</v>
       </c>
-      <c r="E142" s="115"/>
+      <c r="E142" s="116"/>
       <c r="F142" s="27" t="s">
         <v>719</v>
       </c>
@@ -11163,11 +11199,11 @@
       <c r="C143" s="20" t="s">
         <v>589</v>
       </c>
-      <c r="E143" s="106" t="s">
+      <c r="E143" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F143" s="106"/>
-      <c r="G143" s="105" t="s">
+      <c r="F143" s="107"/>
+      <c r="G143" s="106" t="s">
         <v>611</v>
       </c>
     </row>
@@ -11181,9 +11217,9 @@
       <c r="C144" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="E144" s="106"/>
-      <c r="F144" s="106"/>
-      <c r="G144" s="105"/>
+      <c r="E144" s="107"/>
+      <c r="F144" s="107"/>
+      <c r="G144" s="106"/>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A145" s="18" t="s">
@@ -11195,15 +11231,15 @@
       <c r="C145" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E145" s="106"/>
-      <c r="F145" s="106"/>
-      <c r="G145" s="105"/>
+      <c r="E145" s="107"/>
+      <c r="F145" s="107"/>
+      <c r="G145" s="106"/>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="E147" s="157" t="s">
+      <c r="E147" s="158" t="s">
         <v>908</v>
       </c>
-      <c r="F147" s="157"/>
+      <c r="F147" s="158"/>
       <c r="G147" s="28" t="s">
         <v>613</v>
       </c>
@@ -11279,7 +11315,7 @@
       <c r="C151" s="20" t="s">
         <v>590</v>
       </c>
-      <c r="E151" s="111" t="s">
+      <c r="E151" s="112" t="s">
         <v>695</v>
       </c>
       <c r="F151" s="78" t="s">
@@ -11299,7 +11335,7 @@
       <c r="C152" s="20" t="s">
         <v>591</v>
       </c>
-      <c r="E152" s="112"/>
+      <c r="E152" s="113"/>
       <c r="F152" s="78" t="s">
         <v>722</v>
       </c>
@@ -11317,7 +11353,7 @@
       <c r="C153" s="20" t="s">
         <v>596</v>
       </c>
-      <c r="E153" s="112"/>
+      <c r="E153" s="113"/>
       <c r="F153" s="78" t="s">
         <v>723</v>
       </c>
@@ -11335,7 +11371,7 @@
       <c r="C154" s="20" t="s">
         <v>597</v>
       </c>
-      <c r="E154" s="112"/>
+      <c r="E154" s="113"/>
       <c r="F154" s="78" t="s">
         <v>724</v>
       </c>
@@ -11353,7 +11389,7 @@
       <c r="C155" s="20" t="s">
         <v>592</v>
       </c>
-      <c r="E155" s="116"/>
+      <c r="E155" s="117"/>
       <c r="F155" s="78" t="s">
         <v>725</v>
       </c>
@@ -11374,7 +11410,7 @@
       <c r="D156" s="32" t="s">
         <v>2060</v>
       </c>
-      <c r="E156" s="114" t="s">
+      <c r="E156" s="115" t="s">
         <v>694</v>
       </c>
       <c r="F156" s="24" t="s">
@@ -11397,7 +11433,7 @@
       <c r="D157" s="32" t="s">
         <v>2061</v>
       </c>
-      <c r="E157" s="117"/>
+      <c r="E157" s="118"/>
       <c r="F157" s="24" t="s">
         <v>727</v>
       </c>
@@ -11418,7 +11454,7 @@
       <c r="D158" s="32" t="s">
         <v>2062</v>
       </c>
-      <c r="E158" s="117"/>
+      <c r="E158" s="118"/>
       <c r="F158" s="24" t="s">
         <v>728</v>
       </c>
@@ -11439,7 +11475,7 @@
       <c r="D159" s="32" t="s">
         <v>2063</v>
       </c>
-      <c r="E159" s="117"/>
+      <c r="E159" s="118"/>
       <c r="F159" s="24" t="s">
         <v>729</v>
       </c>
@@ -11460,14 +11496,14 @@
       <c r="D160" s="33" t="s">
         <v>2101</v>
       </c>
-      <c r="E160" s="118"/>
+      <c r="E160" s="119"/>
       <c r="F160" s="24" t="s">
         <v>730</v>
       </c>
       <c r="G160" s="25" t="s">
         <v>611</v>
       </c>
-      <c r="H160" s="164" t="s">
+      <c r="H160" s="104" t="s">
         <v>2103</v>
       </c>
     </row>
@@ -11481,10 +11517,10 @@
       <c r="C161" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E161" s="106" t="s">
+      <c r="E161" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F161" s="106"/>
+      <c r="F161" s="107"/>
       <c r="G161" s="26" t="s">
         <v>611</v>
       </c>
@@ -11509,10 +11545,10 @@
       <c r="G164"/>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="E165" s="124" t="s">
+      <c r="E165" s="125" t="s">
         <v>2089</v>
       </c>
-      <c r="F165" s="124"/>
+      <c r="F165" s="125"/>
       <c r="G165" s="28" t="s">
         <v>613</v>
       </c>
@@ -11537,7 +11573,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="167" spans="1:8" ht="24" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A167" s="18" t="s">
         <v>129</v>
       </c>
@@ -11550,13 +11586,13 @@
       <c r="E167" s="77" t="s">
         <v>694</v>
       </c>
-      <c r="F167" s="120" t="s">
+      <c r="F167" s="121" t="s">
         <v>732</v>
       </c>
       <c r="G167" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H167" s="90" t="s">
+      <c r="H167" s="104" t="s">
         <v>2104</v>
       </c>
     </row>
@@ -11572,7 +11608,7 @@
       </c>
       <c r="D168" s="45"/>
       <c r="E168" s="77"/>
-      <c r="F168" s="120"/>
+      <c r="F168" s="121"/>
       <c r="G168" s="24" t="s">
         <v>611</v>
       </c>
@@ -11587,10 +11623,10 @@
       <c r="C169" s="18" t="s">
         <v>627</v>
       </c>
-      <c r="E169" s="111" t="s">
+      <c r="E169" s="112" t="s">
         <v>695</v>
       </c>
-      <c r="F169" s="104" t="s">
+      <c r="F169" s="105" t="s">
         <v>733</v>
       </c>
       <c r="G169" s="78" t="s">
@@ -11609,8 +11645,8 @@
         <v>627</v>
       </c>
       <c r="D170" s="45"/>
-      <c r="E170" s="113"/>
-      <c r="F170" s="104"/>
+      <c r="E170" s="114"/>
+      <c r="F170" s="105"/>
       <c r="G170" s="78" t="s">
         <v>611</v>
       </c>
@@ -11625,10 +11661,10 @@
       <c r="C171" s="18" t="s">
         <v>628</v>
       </c>
-      <c r="E171" s="111" t="s">
+      <c r="E171" s="112" t="s">
         <v>695</v>
       </c>
-      <c r="F171" s="149" t="s">
+      <c r="F171" s="150" t="s">
         <v>791</v>
       </c>
       <c r="G171" s="72" t="s">
@@ -11646,8 +11682,8 @@
         <v>628</v>
       </c>
       <c r="D172" s="45"/>
-      <c r="E172" s="113"/>
-      <c r="F172" s="149"/>
+      <c r="E172" s="114"/>
+      <c r="F172" s="150"/>
       <c r="G172" s="72" t="s">
         <v>873</v>
       </c>
@@ -11662,11 +11698,11 @@
       <c r="C173" s="18" t="s">
         <v>874</v>
       </c>
-      <c r="D173" s="163" t="s">
+      <c r="D173" s="164" t="s">
         <v>1003</v>
       </c>
       <c r="E173" s="77"/>
-      <c r="F173" s="120" t="s">
+      <c r="F173" s="121" t="s">
         <v>883</v>
       </c>
       <c r="G173" s="24" t="s">
@@ -11683,9 +11719,9 @@
       <c r="C174" t="s">
         <v>874</v>
       </c>
-      <c r="D174" s="163"/>
+      <c r="D174" s="164"/>
       <c r="E174" s="77"/>
-      <c r="F174" s="120"/>
+      <c r="F174" s="121"/>
       <c r="G174" s="24" t="s">
         <v>611</v>
       </c>
@@ -11700,11 +11736,11 @@
       <c r="C175" s="18" t="s">
         <v>629</v>
       </c>
-      <c r="D175" s="163" t="s">
+      <c r="D175" s="164" t="s">
         <v>1004</v>
       </c>
       <c r="E175" s="77"/>
-      <c r="F175" s="120" t="s">
+      <c r="F175" s="121" t="s">
         <v>734</v>
       </c>
       <c r="G175" s="24" t="s">
@@ -11721,14 +11757,14 @@
       <c r="C176" t="s">
         <v>629</v>
       </c>
-      <c r="D176" s="163"/>
+      <c r="D176" s="164"/>
       <c r="E176" s="77"/>
-      <c r="F176" s="120"/>
+      <c r="F176" s="121"/>
       <c r="G176" s="24" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="177" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A177" s="18" t="s">
         <v>138</v>
       </c>
@@ -11739,13 +11775,13 @@
         <v>630</v>
       </c>
       <c r="E177" s="77"/>
-      <c r="F177" s="120" t="s">
+      <c r="F177" s="121" t="s">
         <v>735</v>
       </c>
       <c r="G177" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H177" s="89" t="s">
+      <c r="H177" s="104" t="s">
         <v>2136</v>
       </c>
     </row>
@@ -11761,7 +11797,7 @@
       </c>
       <c r="D178" s="45"/>
       <c r="E178" s="77"/>
-      <c r="F178" s="120"/>
+      <c r="F178" s="121"/>
       <c r="G178" s="24" t="s">
         <v>611</v>
       </c>
@@ -11776,11 +11812,11 @@
       <c r="C179" s="18" t="s">
         <v>631</v>
       </c>
-      <c r="D179" s="163" t="s">
+      <c r="D179" s="164" t="s">
         <v>1005</v>
       </c>
       <c r="E179" s="77"/>
-      <c r="F179" s="120" t="s">
+      <c r="F179" s="121" t="s">
         <v>736</v>
       </c>
       <c r="G179" s="24" t="s">
@@ -11797,9 +11833,9 @@
       <c r="C180" t="s">
         <v>631</v>
       </c>
-      <c r="D180" s="163"/>
+      <c r="D180" s="164"/>
       <c r="E180" s="77"/>
-      <c r="F180" s="120"/>
+      <c r="F180" s="121"/>
       <c r="G180" s="24" t="s">
         <v>611</v>
       </c>
@@ -11814,10 +11850,10 @@
       <c r="C181" s="18" t="s">
         <v>632</v>
       </c>
-      <c r="E181" s="111" t="s">
+      <c r="E181" s="112" t="s">
         <v>695</v>
       </c>
-      <c r="F181" s="104" t="s">
+      <c r="F181" s="105" t="s">
         <v>737</v>
       </c>
       <c r="G181" s="78" t="s">
@@ -11835,8 +11871,8 @@
         <v>632</v>
       </c>
       <c r="D182" s="45"/>
-      <c r="E182" s="113"/>
-      <c r="F182" s="104"/>
+      <c r="E182" s="114"/>
+      <c r="F182" s="105"/>
       <c r="G182" s="78" t="s">
         <v>611</v>
       </c>
@@ -11851,13 +11887,13 @@
       <c r="C184" s="18" t="s">
         <v>635</v>
       </c>
-      <c r="D184" s="163" t="s">
+      <c r="D184" s="164" t="s">
         <v>1008</v>
       </c>
       <c r="E184" s="79" t="s">
         <v>694</v>
       </c>
-      <c r="F184" s="120" t="s">
+      <c r="F184" s="121" t="s">
         <v>890</v>
       </c>
       <c r="G184" s="24" t="s">
@@ -11874,9 +11910,9 @@
       <c r="C185" t="s">
         <v>635</v>
       </c>
-      <c r="D185" s="163"/>
+      <c r="D185" s="164"/>
       <c r="E185" s="77"/>
-      <c r="F185" s="120"/>
+      <c r="F185" s="121"/>
       <c r="G185" s="24" t="s">
         <v>611</v>
       </c>
@@ -11891,10 +11927,10 @@
       <c r="C186" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="E186" s="111" t="s">
+      <c r="E186" s="112" t="s">
         <v>695</v>
       </c>
-      <c r="F186" s="121" t="s">
+      <c r="F186" s="122" t="s">
         <v>2094</v>
       </c>
       <c r="G186" s="92" t="s">
@@ -11912,8 +11948,8 @@
         <v>636</v>
       </c>
       <c r="D187" s="45"/>
-      <c r="E187" s="112"/>
-      <c r="F187" s="122"/>
+      <c r="E187" s="113"/>
+      <c r="F187" s="123"/>
       <c r="G187" s="92" t="s">
         <v>2095</v>
       </c>
@@ -11928,8 +11964,8 @@
       <c r="C188" s="18" t="s">
         <v>637</v>
       </c>
-      <c r="E188" s="112"/>
-      <c r="F188" s="122"/>
+      <c r="E188" s="113"/>
+      <c r="F188" s="123"/>
       <c r="G188" s="92" t="s">
         <v>2095</v>
       </c>
@@ -11945,8 +11981,8 @@
         <v>637</v>
       </c>
       <c r="D189" s="45"/>
-      <c r="E189" s="113"/>
-      <c r="F189" s="123"/>
+      <c r="E189" s="114"/>
+      <c r="F189" s="124"/>
       <c r="G189" s="92" t="s">
         <v>2095</v>
       </c>
@@ -11961,11 +11997,11 @@
       <c r="C190" s="18" t="s">
         <v>638</v>
       </c>
-      <c r="D190" s="163" t="s">
+      <c r="D190" s="164" t="s">
         <v>1009</v>
       </c>
       <c r="E190" s="77"/>
-      <c r="F190" s="120" t="s">
+      <c r="F190" s="121" t="s">
         <v>738</v>
       </c>
       <c r="G190" s="24" t="s">
@@ -11982,9 +12018,9 @@
       <c r="C191" t="s">
         <v>638</v>
       </c>
-      <c r="D191" s="163"/>
+      <c r="D191" s="164"/>
       <c r="E191" s="77"/>
-      <c r="F191" s="120"/>
+      <c r="F191" s="121"/>
       <c r="G191" s="24" t="s">
         <v>611</v>
       </c>
@@ -11999,11 +12035,11 @@
       <c r="C192" s="18" t="s">
         <v>639</v>
       </c>
-      <c r="D192" s="163" t="s">
+      <c r="D192" s="164" t="s">
         <v>1010</v>
       </c>
       <c r="E192" s="77"/>
-      <c r="F192" s="120" t="s">
+      <c r="F192" s="121" t="s">
         <v>739</v>
       </c>
       <c r="G192" s="24" t="s">
@@ -12020,9 +12056,9 @@
       <c r="C193" t="s">
         <v>639</v>
       </c>
-      <c r="D193" s="163"/>
+      <c r="D193" s="164"/>
       <c r="E193" s="77"/>
-      <c r="F193" s="120"/>
+      <c r="F193" s="121"/>
       <c r="G193" s="24" t="s">
         <v>611</v>
       </c>
@@ -12037,13 +12073,13 @@
       <c r="C194" s="18" t="s">
         <v>640</v>
       </c>
-      <c r="D194" s="163" t="s">
+      <c r="D194" s="164" t="s">
         <v>606</v>
       </c>
-      <c r="E194" s="111" t="s">
+      <c r="E194" s="112" t="s">
         <v>695</v>
       </c>
-      <c r="F194" s="104" t="s">
+      <c r="F194" s="105" t="s">
         <v>740</v>
       </c>
       <c r="G194" s="78" t="s">
@@ -12060,9 +12096,9 @@
       <c r="C195" t="s">
         <v>640</v>
       </c>
-      <c r="D195" s="163"/>
-      <c r="E195" s="113"/>
-      <c r="F195" s="104"/>
+      <c r="D195" s="164"/>
+      <c r="E195" s="114"/>
+      <c r="F195" s="105"/>
       <c r="G195" s="78" t="s">
         <v>873</v>
       </c>
@@ -12077,11 +12113,11 @@
       <c r="C196" s="18" t="s">
         <v>877</v>
       </c>
-      <c r="D196" s="163" t="s">
+      <c r="D196" s="164" t="s">
         <v>1011</v>
       </c>
       <c r="E196" s="77"/>
-      <c r="F196" s="120" t="s">
+      <c r="F196" s="121" t="s">
         <v>741</v>
       </c>
       <c r="G196" s="24" t="s">
@@ -12098,9 +12134,9 @@
       <c r="C197" t="s">
         <v>877</v>
       </c>
-      <c r="D197" s="163"/>
+      <c r="D197" s="164"/>
       <c r="E197" s="77"/>
-      <c r="F197" s="120"/>
+      <c r="F197" s="121"/>
       <c r="G197" s="24" t="s">
         <v>611</v>
       </c>
@@ -12115,10 +12151,10 @@
       <c r="C198" s="18" t="s">
         <v>641</v>
       </c>
-      <c r="E198" s="111" t="s">
+      <c r="E198" s="112" t="s">
         <v>695</v>
       </c>
-      <c r="F198" s="104" t="s">
+      <c r="F198" s="105" t="s">
         <v>742</v>
       </c>
       <c r="G198" s="78" t="s">
@@ -12136,13 +12172,13 @@
         <v>641</v>
       </c>
       <c r="D199" s="45"/>
-      <c r="E199" s="113"/>
-      <c r="F199" s="104"/>
+      <c r="E199" s="114"/>
+      <c r="F199" s="105"/>
       <c r="G199" s="78" t="s">
         <v>873</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="200" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A200" s="18" t="s">
         <v>162</v>
       </c>
@@ -12153,13 +12189,13 @@
         <v>642</v>
       </c>
       <c r="E200" s="77"/>
-      <c r="F200" s="120" t="s">
+      <c r="F200" s="121" t="s">
         <v>743</v>
       </c>
       <c r="G200" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H200" s="89" t="s">
+      <c r="H200" s="104" t="s">
         <v>2138</v>
       </c>
     </row>
@@ -12175,12 +12211,12 @@
       </c>
       <c r="D201" s="45"/>
       <c r="E201" s="77"/>
-      <c r="F201" s="120"/>
+      <c r="F201" s="121"/>
       <c r="G201" s="24" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A202" s="18" t="s">
         <v>164</v>
       </c>
@@ -12191,13 +12227,13 @@
         <v>643</v>
       </c>
       <c r="E202" s="77"/>
-      <c r="F202" s="120" t="s">
+      <c r="F202" s="121" t="s">
         <v>744</v>
       </c>
       <c r="G202" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H202" s="89" t="s">
+      <c r="H202" s="104" t="s">
         <v>2137</v>
       </c>
     </row>
@@ -12213,7 +12249,7 @@
       </c>
       <c r="D203" s="45"/>
       <c r="E203" s="77"/>
-      <c r="F203" s="120"/>
+      <c r="F203" s="121"/>
       <c r="G203" s="24" t="s">
         <v>611</v>
       </c>
@@ -12229,7 +12265,7 @@
         <v>644</v>
       </c>
       <c r="E204" s="77"/>
-      <c r="F204" s="120" t="s">
+      <c r="F204" s="121" t="s">
         <v>745</v>
       </c>
       <c r="G204" s="24" t="s">
@@ -12248,7 +12284,7 @@
       </c>
       <c r="D205" s="45"/>
       <c r="E205" s="77"/>
-      <c r="F205" s="120"/>
+      <c r="F205" s="121"/>
       <c r="G205" s="24" t="s">
         <v>611</v>
       </c>
@@ -12263,11 +12299,11 @@
       <c r="C206" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="D206" s="163" t="s">
+      <c r="D206" s="164" t="s">
         <v>1012</v>
       </c>
       <c r="E206" s="77"/>
-      <c r="F206" s="120" t="s">
+      <c r="F206" s="121" t="s">
         <v>746</v>
       </c>
       <c r="G206" s="24" t="s">
@@ -12284,14 +12320,14 @@
       <c r="C207" t="s">
         <v>645</v>
       </c>
-      <c r="D207" s="163"/>
+      <c r="D207" s="164"/>
       <c r="E207" s="77"/>
-      <c r="F207" s="120"/>
+      <c r="F207" s="121"/>
       <c r="G207" s="24" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="208" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A208" s="18" t="s">
         <v>170</v>
       </c>
@@ -12302,17 +12338,17 @@
         <v>646</v>
       </c>
       <c r="E208" s="77"/>
-      <c r="F208" s="120" t="s">
+      <c r="F208" s="121" t="s">
         <v>891</v>
       </c>
       <c r="G208" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H208" s="90" t="s">
+      <c r="H208" s="104" t="s">
         <v>2139</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="209" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>449</v>
       </c>
@@ -12324,15 +12360,15 @@
       </c>
       <c r="D209" s="45"/>
       <c r="E209" s="77"/>
-      <c r="F209" s="120"/>
+      <c r="F209" s="121"/>
       <c r="G209" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H209" s="90" t="s">
+      <c r="H209" s="104" t="s">
         <v>2161</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="210" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A210" s="18" t="s">
         <v>235</v>
       </c>
@@ -12343,13 +12379,13 @@
         <v>647</v>
       </c>
       <c r="E210" s="77"/>
-      <c r="F210" s="120" t="s">
+      <c r="F210" s="121" t="s">
         <v>892</v>
       </c>
       <c r="G210" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H210" s="89" t="s">
+      <c r="H210" s="104" t="s">
         <v>2140</v>
       </c>
     </row>
@@ -12365,7 +12401,7 @@
       </c>
       <c r="D211" s="45"/>
       <c r="E211" s="77"/>
-      <c r="F211" s="120"/>
+      <c r="F211" s="121"/>
       <c r="G211" s="24" t="s">
         <v>611</v>
       </c>
@@ -12380,11 +12416,11 @@
       <c r="C212" s="18" t="s">
         <v>648</v>
       </c>
-      <c r="D212" s="163" t="s">
+      <c r="D212" s="164" t="s">
         <v>1013</v>
       </c>
       <c r="E212" s="77"/>
-      <c r="F212" s="120" t="s">
+      <c r="F212" s="121" t="s">
         <v>747</v>
       </c>
       <c r="G212" s="24" t="s">
@@ -12401,9 +12437,9 @@
       <c r="C213" t="s">
         <v>648</v>
       </c>
-      <c r="D213" s="163"/>
+      <c r="D213" s="164"/>
       <c r="E213" s="77"/>
-      <c r="F213" s="120"/>
+      <c r="F213" s="121"/>
       <c r="G213" s="24" t="s">
         <v>611</v>
       </c>
@@ -12427,13 +12463,13 @@
       <c r="C215" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="D215" s="163" t="s">
+      <c r="D215" s="164" t="s">
         <v>1015</v>
       </c>
       <c r="E215" s="77" t="s">
         <v>695</v>
       </c>
-      <c r="F215" s="132" t="s">
+      <c r="F215" s="133" t="s">
         <v>748</v>
       </c>
       <c r="G215" s="24" t="s">
@@ -12450,9 +12486,9 @@
       <c r="C216" t="s">
         <v>649</v>
       </c>
-      <c r="D216" s="163"/>
+      <c r="D216" s="164"/>
       <c r="E216" s="77"/>
-      <c r="F216" s="132"/>
+      <c r="F216" s="133"/>
       <c r="G216" s="24" t="s">
         <v>611</v>
       </c>
@@ -12467,9 +12503,9 @@
       <c r="C217" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="D217" s="163"/>
+      <c r="D217" s="164"/>
       <c r="E217" s="77"/>
-      <c r="F217" s="132"/>
+      <c r="F217" s="133"/>
       <c r="G217" s="24" t="s">
         <v>611</v>
       </c>
@@ -12484,9 +12520,9 @@
       <c r="C218" s="18" t="s">
         <v>649</v>
       </c>
-      <c r="D218" s="163"/>
+      <c r="D218" s="164"/>
       <c r="E218" s="77"/>
-      <c r="F218" s="132"/>
+      <c r="F218" s="133"/>
       <c r="G218" s="24" t="s">
         <v>611</v>
       </c>
@@ -12501,10 +12537,10 @@
       <c r="C219" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="E219" s="111" t="s">
+      <c r="E219" s="112" t="s">
         <v>695</v>
       </c>
-      <c r="F219" s="133" t="s">
+      <c r="F219" s="134" t="s">
         <v>749</v>
       </c>
       <c r="G219" s="92" t="s">
@@ -12522,8 +12558,8 @@
         <v>650</v>
       </c>
       <c r="D220" s="45"/>
-      <c r="E220" s="112"/>
-      <c r="F220" s="133"/>
+      <c r="E220" s="113"/>
+      <c r="F220" s="134"/>
       <c r="G220" s="92" t="s">
         <v>2095</v>
       </c>
@@ -12538,8 +12574,8 @@
       <c r="C221" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="E221" s="112"/>
-      <c r="F221" s="133"/>
+      <c r="E221" s="113"/>
+      <c r="F221" s="134"/>
       <c r="G221" s="92" t="s">
         <v>2095</v>
       </c>
@@ -12554,13 +12590,13 @@
       <c r="C222" s="18" t="s">
         <v>650</v>
       </c>
-      <c r="E222" s="113"/>
-      <c r="F222" s="133"/>
+      <c r="E222" s="114"/>
+      <c r="F222" s="134"/>
       <c r="G222" s="92" t="s">
         <v>2095</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="223" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A223" s="18" t="s">
         <v>243</v>
       </c>
@@ -12571,17 +12607,17 @@
         <v>651</v>
       </c>
       <c r="E223" s="77"/>
-      <c r="F223" s="132" t="s">
+      <c r="F223" s="133" t="s">
         <v>750</v>
       </c>
       <c r="G223" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H223" s="89" t="s">
+      <c r="H223" s="104" t="s">
         <v>2141</v>
       </c>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="224" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>465</v>
       </c>
@@ -12593,11 +12629,11 @@
       </c>
       <c r="D224" s="45"/>
       <c r="E224" s="77"/>
-      <c r="F224" s="132"/>
+      <c r="F224" s="133"/>
       <c r="G224" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H224" s="89" t="s">
+      <c r="H224" s="104" t="s">
         <v>2142</v>
       </c>
     </row>
@@ -12612,7 +12648,7 @@
         <v>651</v>
       </c>
       <c r="E225" s="77"/>
-      <c r="F225" s="132"/>
+      <c r="F225" s="133"/>
       <c r="G225" s="24" t="s">
         <v>611</v>
       </c>
@@ -12628,7 +12664,7 @@
         <v>651</v>
       </c>
       <c r="E226" s="77"/>
-      <c r="F226" s="132"/>
+      <c r="F226" s="133"/>
       <c r="G226" s="24" t="s">
         <v>611</v>
       </c>
@@ -12643,10 +12679,10 @@
       <c r="C227" s="18" t="s">
         <v>652</v>
       </c>
-      <c r="E227" s="111" t="s">
+      <c r="E227" s="112" t="s">
         <v>695</v>
       </c>
-      <c r="F227" s="104" t="s">
+      <c r="F227" s="105" t="s">
         <v>751</v>
       </c>
       <c r="G227" s="78" t="s">
@@ -12664,13 +12700,13 @@
         <v>652</v>
       </c>
       <c r="D228" s="45"/>
-      <c r="E228" s="113"/>
-      <c r="F228" s="104"/>
+      <c r="E228" s="114"/>
+      <c r="F228" s="105"/>
       <c r="G228" s="78" t="s">
         <v>2095</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="229" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A229" s="18" t="s">
         <v>247</v>
       </c>
@@ -12681,13 +12717,13 @@
         <v>653</v>
       </c>
       <c r="E229" s="77"/>
-      <c r="F229" s="120" t="s">
+      <c r="F229" s="121" t="s">
         <v>752</v>
       </c>
       <c r="G229" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H229" s="89" t="s">
+      <c r="H229" s="104" t="s">
         <v>2143</v>
       </c>
     </row>
@@ -12703,7 +12739,7 @@
       </c>
       <c r="D230" s="45"/>
       <c r="E230" s="77"/>
-      <c r="F230" s="120"/>
+      <c r="F230" s="121"/>
       <c r="G230" s="24" t="s">
         <v>611</v>
       </c>
@@ -12721,10 +12757,10 @@
       <c r="D231" s="44" t="s">
         <v>625</v>
       </c>
-      <c r="E231" s="111" t="s">
+      <c r="E231" s="112" t="s">
         <v>695</v>
       </c>
-      <c r="F231" s="104" t="s">
+      <c r="F231" s="105" t="s">
         <v>753</v>
       </c>
       <c r="G231" s="78" t="s">
@@ -12745,8 +12781,8 @@
         <v>654</v>
       </c>
       <c r="D232" s="45"/>
-      <c r="E232" s="113"/>
-      <c r="F232" s="104"/>
+      <c r="E232" s="114"/>
+      <c r="F232" s="105"/>
       <c r="G232" s="78" t="s">
         <v>873</v>
       </c>
@@ -12765,7 +12801,7 @@
         <v>625</v>
       </c>
       <c r="E233" s="93"/>
-      <c r="F233" s="104" t="s">
+      <c r="F233" s="105" t="s">
         <v>754</v>
       </c>
       <c r="G233" s="78" t="s">
@@ -12784,7 +12820,7 @@
       </c>
       <c r="D234" s="45"/>
       <c r="E234" s="93"/>
-      <c r="F234" s="104"/>
+      <c r="F234" s="105"/>
       <c r="G234" s="78" t="s">
         <v>873</v>
       </c>
@@ -12803,7 +12839,7 @@
         <v>625</v>
       </c>
       <c r="E235" s="93"/>
-      <c r="F235" s="104" t="s">
+      <c r="F235" s="105" t="s">
         <v>755</v>
       </c>
       <c r="G235" s="78" t="s">
@@ -12822,7 +12858,7 @@
       </c>
       <c r="D236" s="45"/>
       <c r="E236" s="93"/>
-      <c r="F236" s="104"/>
+      <c r="F236" s="105"/>
       <c r="G236" s="78" t="s">
         <v>873</v>
       </c>
@@ -12841,7 +12877,7 @@
         <v>625</v>
       </c>
       <c r="E237" s="93"/>
-      <c r="F237" s="104" t="s">
+      <c r="F237" s="105" t="s">
         <v>756</v>
       </c>
       <c r="G237" s="78" t="s">
@@ -12860,7 +12896,7 @@
       </c>
       <c r="D238" s="45"/>
       <c r="E238" s="93"/>
-      <c r="F238" s="104"/>
+      <c r="F238" s="105"/>
       <c r="G238" s="78" t="s">
         <v>873</v>
       </c>
@@ -12879,7 +12915,7 @@
         <v>625</v>
       </c>
       <c r="E239" s="93"/>
-      <c r="F239" s="104" t="s">
+      <c r="F239" s="105" t="s">
         <v>757</v>
       </c>
       <c r="G239" s="78" t="s">
@@ -12898,7 +12934,7 @@
       </c>
       <c r="D240" s="45"/>
       <c r="E240" s="93"/>
-      <c r="F240" s="104"/>
+      <c r="F240" s="105"/>
       <c r="G240" s="78" t="s">
         <v>873</v>
       </c>
@@ -12917,7 +12953,7 @@
         <v>625</v>
       </c>
       <c r="E241" s="93"/>
-      <c r="F241" s="104" t="s">
+      <c r="F241" s="105" t="s">
         <v>758</v>
       </c>
       <c r="G241" s="78" t="s">
@@ -12936,7 +12972,7 @@
       </c>
       <c r="D242" s="45"/>
       <c r="E242" s="93"/>
-      <c r="F242" s="104"/>
+      <c r="F242" s="105"/>
       <c r="G242" s="78" t="s">
         <v>873</v>
       </c>
@@ -12955,7 +12991,7 @@
         <v>625</v>
       </c>
       <c r="E243" s="93"/>
-      <c r="F243" s="104" t="s">
+      <c r="F243" s="105" t="s">
         <v>759</v>
       </c>
       <c r="G243" s="78" t="s">
@@ -12974,7 +13010,7 @@
       </c>
       <c r="D244" s="45"/>
       <c r="E244" s="93"/>
-      <c r="F244" s="104"/>
+      <c r="F244" s="105"/>
       <c r="G244" s="78" t="s">
         <v>873</v>
       </c>
@@ -12993,7 +13029,7 @@
         <v>625</v>
       </c>
       <c r="E245" s="93"/>
-      <c r="F245" s="104" t="s">
+      <c r="F245" s="105" t="s">
         <v>760</v>
       </c>
       <c r="G245" s="78" t="s">
@@ -13012,7 +13048,7 @@
       </c>
       <c r="D246" s="45"/>
       <c r="E246" s="93"/>
-      <c r="F246" s="104"/>
+      <c r="F246" s="105"/>
       <c r="G246" s="78" t="s">
         <v>873</v>
       </c>
@@ -13031,7 +13067,7 @@
         <v>625</v>
       </c>
       <c r="E247" s="93"/>
-      <c r="F247" s="104" t="s">
+      <c r="F247" s="105" t="s">
         <v>761</v>
       </c>
       <c r="G247" s="78" t="s">
@@ -13050,7 +13086,7 @@
       </c>
       <c r="D248" s="45"/>
       <c r="E248" s="93"/>
-      <c r="F248" s="104"/>
+      <c r="F248" s="105"/>
       <c r="G248" s="78" t="s">
         <v>873</v>
       </c>
@@ -13069,7 +13105,7 @@
         <v>625</v>
       </c>
       <c r="E249" s="93"/>
-      <c r="F249" s="104" t="s">
+      <c r="F249" s="105" t="s">
         <v>2072</v>
       </c>
       <c r="G249" s="78" t="s">
@@ -13088,7 +13124,7 @@
       </c>
       <c r="D250" s="45"/>
       <c r="E250" s="93"/>
-      <c r="F250" s="104"/>
+      <c r="F250" s="105"/>
       <c r="G250" s="78" t="s">
         <v>873</v>
       </c>
@@ -13107,7 +13143,7 @@
         <v>625</v>
       </c>
       <c r="E251" s="93"/>
-      <c r="F251" s="104" t="s">
+      <c r="F251" s="105" t="s">
         <v>762</v>
       </c>
       <c r="G251" s="78" t="s">
@@ -13126,7 +13162,7 @@
       </c>
       <c r="D252" s="45"/>
       <c r="E252" s="93"/>
-      <c r="F252" s="104"/>
+      <c r="F252" s="105"/>
       <c r="G252" s="78" t="s">
         <v>873</v>
       </c>
@@ -13142,7 +13178,7 @@
         <v>665</v>
       </c>
       <c r="E253" s="93"/>
-      <c r="F253" s="104" t="s">
+      <c r="F253" s="105" t="s">
         <v>763</v>
       </c>
       <c r="G253" s="78" t="s">
@@ -13161,7 +13197,7 @@
       </c>
       <c r="D254" s="45"/>
       <c r="E254" s="93"/>
-      <c r="F254" s="104"/>
+      <c r="F254" s="105"/>
       <c r="G254" s="78" t="s">
         <v>873</v>
       </c>
@@ -13186,7 +13222,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="258" spans="1:8" ht="24" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="258" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A258" s="18" t="s">
         <v>143</v>
       </c>
@@ -13208,7 +13244,7 @@
       <c r="G258" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H258" s="89" t="s">
+      <c r="H258" s="104" t="s">
         <v>2146</v>
       </c>
     </row>
@@ -13240,11 +13276,11 @@
       <c r="C260" s="18" t="s">
         <v>573</v>
       </c>
-      <c r="E260" s="107" t="s">
+      <c r="E260" s="108" t="s">
         <v>620</v>
       </c>
-      <c r="F260" s="108"/>
-      <c r="G260" s="155" t="s">
+      <c r="F260" s="109"/>
+      <c r="G260" s="156" t="s">
         <v>611</v>
       </c>
     </row>
@@ -13258,9 +13294,9 @@
       <c r="C261" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E261" s="107"/>
-      <c r="F261" s="108"/>
-      <c r="G261" s="156"/>
+      <c r="E261" s="108"/>
+      <c r="F261" s="109"/>
+      <c r="G261" s="157"/>
     </row>
     <row r="262" spans="1:8" x14ac:dyDescent="0.45">
       <c r="C262" s="23"/>
@@ -13349,7 +13385,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="267" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="267" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A267" s="18" t="s">
         <v>342</v>
       </c>
@@ -13368,7 +13404,7 @@
       <c r="G267" s="78" t="s">
         <v>611</v>
       </c>
-      <c r="H267" s="89" t="s">
+      <c r="H267" s="165" t="s">
         <v>2160</v>
       </c>
     </row>
@@ -13382,10 +13418,10 @@
       <c r="C268" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E268" s="106" t="s">
+      <c r="E268" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F268" s="106"/>
+      <c r="F268" s="107"/>
       <c r="G268" s="26" t="s">
         <v>611</v>
       </c>
@@ -13453,7 +13489,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="274" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="274" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>453</v>
       </c>
@@ -13471,7 +13507,7 @@
       <c r="G274" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H274" s="89" t="s">
+      <c r="H274" s="104" t="s">
         <v>2148</v>
       </c>
     </row>
@@ -13539,7 +13575,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="278" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="278" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>461</v>
       </c>
@@ -13557,7 +13593,7 @@
       <c r="G278" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H278" s="89" t="s">
+      <c r="H278" s="104" t="s">
         <v>2151</v>
       </c>
     </row>
@@ -13572,11 +13608,11 @@
         <v>573</v>
       </c>
       <c r="D279" s="45"/>
-      <c r="E279" s="106" t="s">
+      <c r="E279" s="107" t="s">
         <v>620</v>
       </c>
-      <c r="F279" s="106"/>
-      <c r="G279" s="105" t="s">
+      <c r="F279" s="107"/>
+      <c r="G279" s="106" t="s">
         <v>611</v>
       </c>
     </row>
@@ -13591,19 +13627,19 @@
         <v>601</v>
       </c>
       <c r="D280" s="45"/>
-      <c r="E280" s="106"/>
-      <c r="F280" s="106"/>
-      <c r="G280" s="105"/>
+      <c r="E280" s="107"/>
+      <c r="F280" s="107"/>
+      <c r="G280" s="106"/>
     </row>
     <row r="282" spans="1:8" x14ac:dyDescent="0.45">
       <c r="C282" s="23"/>
     </row>
     <row r="283" spans="1:8" x14ac:dyDescent="0.45">
       <c r="C283" s="23"/>
-      <c r="E283" s="124" t="s">
+      <c r="E283" s="125" t="s">
         <v>906</v>
       </c>
-      <c r="F283" s="124"/>
+      <c r="F283" s="125"/>
       <c r="G283" s="28" t="s">
         <v>613</v>
       </c>
@@ -13628,7 +13664,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="285" spans="1:8" ht="24" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="285" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A285" s="18" t="s">
         <v>284</v>
       </c>
@@ -13644,13 +13680,13 @@
       <c r="E285" s="93" t="s">
         <v>695</v>
       </c>
-      <c r="F285" s="104" t="s">
+      <c r="F285" s="105" t="s">
         <v>792</v>
       </c>
       <c r="G285" s="78" t="s">
         <v>611</v>
       </c>
-      <c r="H285" s="89" t="s">
+      <c r="H285" s="165" t="s">
         <v>2152</v>
       </c>
     </row>
@@ -13665,7 +13701,7 @@
         <v>669</v>
       </c>
       <c r="E286" s="93"/>
-      <c r="F286" s="104"/>
+      <c r="F286" s="105"/>
       <c r="G286" s="78" t="s">
         <v>611</v>
       </c>
@@ -13684,7 +13720,7 @@
         <v>621</v>
       </c>
       <c r="E287" s="93"/>
-      <c r="F287" s="104" t="s">
+      <c r="F287" s="105" t="s">
         <v>769</v>
       </c>
       <c r="G287" s="78" t="s">
@@ -13702,7 +13738,7 @@
         <v>670</v>
       </c>
       <c r="E288" s="93"/>
-      <c r="F288" s="104"/>
+      <c r="F288" s="105"/>
       <c r="G288" s="78" t="s">
         <v>611</v>
       </c>
@@ -13721,7 +13757,7 @@
         <v>621</v>
       </c>
       <c r="E289" s="93"/>
-      <c r="F289" s="104" t="s">
+      <c r="F289" s="105" t="s">
         <v>770</v>
       </c>
       <c r="G289" s="78" t="s">
@@ -13739,7 +13775,7 @@
         <v>671</v>
       </c>
       <c r="E290" s="93"/>
-      <c r="F290" s="104"/>
+      <c r="F290" s="105"/>
       <c r="G290" s="78" t="s">
         <v>611</v>
       </c>
@@ -13758,7 +13794,7 @@
         <v>622</v>
       </c>
       <c r="E291" s="93"/>
-      <c r="F291" s="104" t="s">
+      <c r="F291" s="105" t="s">
         <v>771</v>
       </c>
       <c r="G291" s="78" t="s">
@@ -13776,7 +13812,7 @@
         <v>672</v>
       </c>
       <c r="E292" s="93"/>
-      <c r="F292" s="104"/>
+      <c r="F292" s="105"/>
       <c r="G292" s="78" t="s">
         <v>614</v>
       </c>
@@ -13795,7 +13831,7 @@
         <v>622</v>
       </c>
       <c r="E293" s="93"/>
-      <c r="F293" s="104" t="s">
+      <c r="F293" s="105" t="s">
         <v>772</v>
       </c>
       <c r="G293" s="78" t="s">
@@ -13813,7 +13849,7 @@
         <v>673</v>
       </c>
       <c r="E294" s="93"/>
-      <c r="F294" s="104"/>
+      <c r="F294" s="105"/>
       <c r="G294" s="78" t="s">
         <v>614</v>
       </c>
@@ -13832,7 +13868,7 @@
         <v>621</v>
       </c>
       <c r="E295" s="93"/>
-      <c r="F295" s="104" t="s">
+      <c r="F295" s="105" t="s">
         <v>773</v>
       </c>
       <c r="G295" s="78" t="s">
@@ -13850,7 +13886,7 @@
         <v>674</v>
       </c>
       <c r="E296" s="93"/>
-      <c r="F296" s="104"/>
+      <c r="F296" s="105"/>
       <c r="G296" s="78" t="s">
         <v>611</v>
       </c>
@@ -13869,7 +13905,7 @@
         <v>621</v>
       </c>
       <c r="E297" s="93"/>
-      <c r="F297" s="104" t="s">
+      <c r="F297" s="105" t="s">
         <v>774</v>
       </c>
       <c r="G297" s="78" t="s">
@@ -13887,7 +13923,7 @@
         <v>675</v>
       </c>
       <c r="E298" s="93"/>
-      <c r="F298" s="104"/>
+      <c r="F298" s="105"/>
       <c r="G298" s="78" t="s">
         <v>611</v>
       </c>
@@ -13906,7 +13942,7 @@
         <v>621</v>
       </c>
       <c r="E299" s="93"/>
-      <c r="F299" s="104" t="s">
+      <c r="F299" s="105" t="s">
         <v>775</v>
       </c>
       <c r="G299" s="78" t="s">
@@ -13924,7 +13960,7 @@
         <v>676</v>
       </c>
       <c r="E300" s="93"/>
-      <c r="F300" s="104"/>
+      <c r="F300" s="105"/>
       <c r="G300" s="78" t="s">
         <v>611</v>
       </c>
@@ -13943,7 +13979,7 @@
         <v>623</v>
       </c>
       <c r="E301" s="93"/>
-      <c r="F301" s="104" t="s">
+      <c r="F301" s="105" t="s">
         <v>776</v>
       </c>
       <c r="G301" s="78" t="s">
@@ -13961,12 +13997,12 @@
         <v>677</v>
       </c>
       <c r="E302" s="93"/>
-      <c r="F302" s="104"/>
+      <c r="F302" s="105"/>
       <c r="G302" s="78" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="303" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="303" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A303" s="18" t="s">
         <v>304</v>
       </c>
@@ -13977,13 +14013,13 @@
         <v>678</v>
       </c>
       <c r="E303" s="77"/>
-      <c r="F303" s="120" t="s">
+      <c r="F303" s="121" t="s">
         <v>777</v>
       </c>
       <c r="G303" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H303" s="89" t="s">
+      <c r="H303" s="104" t="s">
         <v>2153</v>
       </c>
     </row>
@@ -13998,7 +14034,7 @@
         <v>678</v>
       </c>
       <c r="E304" s="77"/>
-      <c r="F304" s="120"/>
+      <c r="F304" s="121"/>
       <c r="G304" s="24" t="s">
         <v>611</v>
       </c>
@@ -14014,7 +14050,7 @@
         <v>679</v>
       </c>
       <c r="E305" s="93"/>
-      <c r="F305" s="104" t="s">
+      <c r="F305" s="105" t="s">
         <v>778</v>
       </c>
       <c r="G305" s="78" t="s">
@@ -14032,7 +14068,7 @@
         <v>679</v>
       </c>
       <c r="E306" s="93"/>
-      <c r="F306" s="104"/>
+      <c r="F306" s="105"/>
       <c r="G306" s="78" t="s">
         <v>611</v>
       </c>
@@ -14048,7 +14084,7 @@
         <v>680</v>
       </c>
       <c r="E307" s="93"/>
-      <c r="F307" s="104" t="s">
+      <c r="F307" s="105" t="s">
         <v>779</v>
       </c>
       <c r="G307" s="92" t="s">
@@ -14069,7 +14105,7 @@
         <v>680</v>
       </c>
       <c r="E308" s="93"/>
-      <c r="F308" s="104"/>
+      <c r="F308" s="105"/>
       <c r="G308" s="92" t="s">
         <v>618</v>
       </c>
@@ -14085,7 +14121,7 @@
         <v>682</v>
       </c>
       <c r="E309" s="93"/>
-      <c r="F309" s="104" t="s">
+      <c r="F309" s="105" t="s">
         <v>780</v>
       </c>
       <c r="G309" s="78" t="s">
@@ -14103,7 +14139,7 @@
         <v>682</v>
       </c>
       <c r="E310" s="93"/>
-      <c r="F310" s="104"/>
+      <c r="F310" s="105"/>
       <c r="G310" s="78" t="s">
         <v>611</v>
       </c>
@@ -14119,7 +14155,7 @@
         <v>683</v>
       </c>
       <c r="E311" s="93"/>
-      <c r="F311" s="104" t="s">
+      <c r="F311" s="105" t="s">
         <v>781</v>
       </c>
       <c r="G311" s="78" t="s">
@@ -14137,12 +14173,12 @@
         <v>683</v>
       </c>
       <c r="E312" s="93"/>
-      <c r="F312" s="104"/>
+      <c r="F312" s="105"/>
       <c r="G312" s="78" t="s">
         <v>2095</v>
       </c>
     </row>
-    <row r="313" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="313" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A313" s="18" t="s">
         <v>321</v>
       </c>
@@ -14153,13 +14189,13 @@
         <v>684</v>
       </c>
       <c r="E313" s="77"/>
-      <c r="F313" s="120" t="s">
+      <c r="F313" s="121" t="s">
         <v>782</v>
       </c>
       <c r="G313" s="24" t="s">
         <v>611</v>
       </c>
-      <c r="H313" s="89" t="s">
+      <c r="H313" s="104" t="s">
         <v>2156</v>
       </c>
     </row>
@@ -14174,7 +14210,7 @@
         <v>684</v>
       </c>
       <c r="E314" s="77"/>
-      <c r="F314" s="120"/>
+      <c r="F314" s="121"/>
       <c r="G314" s="24" t="s">
         <v>611</v>
       </c>
@@ -14190,7 +14226,7 @@
         <v>685</v>
       </c>
       <c r="E315" s="93"/>
-      <c r="F315" s="104" t="s">
+      <c r="F315" s="105" t="s">
         <v>783</v>
       </c>
       <c r="G315" s="78" t="s">
@@ -14208,7 +14244,7 @@
         <v>685</v>
       </c>
       <c r="E316" s="93"/>
-      <c r="F316" s="104"/>
+      <c r="F316" s="105"/>
       <c r="G316" s="78" t="s">
         <v>873</v>
       </c>
@@ -14224,7 +14260,7 @@
         <v>686</v>
       </c>
       <c r="E317" s="93"/>
-      <c r="F317" s="104" t="s">
+      <c r="F317" s="105" t="s">
         <v>784</v>
       </c>
       <c r="G317" s="78" t="s">
@@ -14242,7 +14278,7 @@
         <v>686</v>
       </c>
       <c r="E318" s="93"/>
-      <c r="F318" s="104"/>
+      <c r="F318" s="105"/>
       <c r="G318" s="78" t="s">
         <v>873</v>
       </c>
@@ -14258,7 +14294,7 @@
         <v>687</v>
       </c>
       <c r="E319" s="93"/>
-      <c r="F319" s="104" t="s">
+      <c r="F319" s="105" t="s">
         <v>785</v>
       </c>
       <c r="G319" s="78" t="s">
@@ -14276,7 +14312,7 @@
         <v>687</v>
       </c>
       <c r="E320" s="93"/>
-      <c r="F320" s="104"/>
+      <c r="F320" s="105"/>
       <c r="G320" s="78" t="s">
         <v>873</v>
       </c>
@@ -14292,7 +14328,7 @@
         <v>688</v>
       </c>
       <c r="E321" s="93"/>
-      <c r="F321" s="133" t="s">
+      <c r="F321" s="134" t="s">
         <v>786</v>
       </c>
       <c r="G321" s="78" t="s">
@@ -14310,7 +14346,7 @@
         <v>688</v>
       </c>
       <c r="E322" s="93"/>
-      <c r="F322" s="104"/>
+      <c r="F322" s="105"/>
       <c r="G322" s="78" t="s">
         <v>611</v>
       </c>
@@ -14410,11 +14446,11 @@
       <c r="C329" s="18" t="s">
         <v>573</v>
       </c>
-      <c r="E329" s="126" t="s">
+      <c r="E329" s="127" t="s">
         <v>620</v>
       </c>
-      <c r="F329" s="127"/>
-      <c r="G329" s="130" t="s">
+      <c r="F329" s="128"/>
+      <c r="G329" s="131" t="s">
         <v>611</v>
       </c>
     </row>
@@ -14428,9 +14464,9 @@
       <c r="C330" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E330" s="128"/>
-      <c r="F330" s="129"/>
-      <c r="G330" s="131"/>
+      <c r="E330" s="129"/>
+      <c r="F330" s="130"/>
+      <c r="G330" s="132"/>
     </row>
     <row r="333" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A333" s="38" t="s">
@@ -14527,11 +14563,11 @@
       <c r="C337" s="18" t="s">
         <v>573</v>
       </c>
-      <c r="E337" s="126" t="s">
+      <c r="E337" s="127" t="s">
         <v>620</v>
       </c>
-      <c r="F337" s="127"/>
-      <c r="G337" s="130" t="s">
+      <c r="F337" s="128"/>
+      <c r="G337" s="131" t="s">
         <v>611</v>
       </c>
     </row>
@@ -14545,9 +14581,9 @@
       <c r="C338" s="18" t="s">
         <v>601</v>
       </c>
-      <c r="E338" s="128"/>
-      <c r="F338" s="129"/>
-      <c r="G338" s="131"/>
+      <c r="E338" s="129"/>
+      <c r="F338" s="130"/>
+      <c r="G338" s="132"/>
     </row>
   </sheetData>
   <mergeCells count="193">

</xml_diff>

<commit_message>
update(metamodel): To Do's updated
</commit_message>
<xml_diff>
--- a/M150-Onto_Metamodel_Rework.xlsx
+++ b/M150-Onto_Metamodel_Rework.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jluis\Repositories\M150-Onto\m150-onto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FF8D4B-BE8D-4A21-9C3A-8A7C5BCE24E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3392E4C-A42D-4C02-9087-150921AFA5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="1" activeTab="1" xr2:uid="{FEE85CB8-E22B-44F8-B2C8-C132767C24A8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="1" activeTab="2" xr2:uid="{FEE85CB8-E22B-44F8-B2C8-C132767C24A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Template Scoring Matrix" sheetId="8" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Type Z Raw Data" sheetId="5" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'M150-Onto'!$A$184:$H$213</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'M150-Onto'!$E$1:$G$338</definedName>
     <definedName name="TypZ" localSheetId="3">'Type Z Raw Data'!$A$1:$Y$349</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -14586,6 +14586,7 @@
       <c r="G338" s="132"/>
     </row>
   </sheetData>
+  <autoFilter ref="E1:G338" xr:uid="{E6F8B2E1-92DB-4647-972B-7ABE25CA54AE}"/>
   <mergeCells count="193">
     <mergeCell ref="D212:D213"/>
     <mergeCell ref="D215:D218"/>

</xml_diff>